<commit_message>
feat(viewer): add AI review button + modal, test pipeline with Reflexion
</commit_message>
<xml_diff>
--- a/papers_record.xlsx
+++ b/papers_record.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC111"/>
+  <dimension ref="A1:AC139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -600,8 +600,6 @@
           <t>分层管理型</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -666,8 +664,6 @@
           <t>分层管理型</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -732,8 +728,6 @@
           <t>检索型</t>
         </is>
       </c>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -798,8 +792,6 @@
           <t>参数/潜变量型</t>
         </is>
       </c>
-      <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -864,8 +856,6 @@
           <t>结构化图谱型</t>
         </is>
       </c>
-      <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -930,8 +920,6 @@
           <t>结构化图谱型</t>
         </is>
       </c>
-      <c r="AB7" t="inlineStr"/>
-      <c r="AC7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -996,8 +984,6 @@
           <t>上下文/摘要型</t>
         </is>
       </c>
-      <c r="AB8" t="inlineStr"/>
-      <c r="AC8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1062,8 +1048,6 @@
           <t>其他</t>
         </is>
       </c>
-      <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1128,8 +1112,6 @@
           <t>参数/潜变量型</t>
         </is>
       </c>
-      <c r="AB10" t="inlineStr"/>
-      <c r="AC10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1258,8 +1240,6 @@
           <t>检索型</t>
         </is>
       </c>
-      <c r="AB12" t="inlineStr"/>
-      <c r="AC12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1324,8 +1304,6 @@
           <t>检索型</t>
         </is>
       </c>
-      <c r="AB13" t="inlineStr"/>
-      <c r="AC13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1390,8 +1368,6 @@
           <t>上下文/摘要型</t>
         </is>
       </c>
-      <c r="AB14" t="inlineStr"/>
-      <c r="AC14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1456,8 +1432,6 @@
           <t>反思经验型</t>
         </is>
       </c>
-      <c r="AB15" t="inlineStr"/>
-      <c r="AC15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1522,8 +1496,6 @@
           <t>检索型</t>
         </is>
       </c>
-      <c r="AB16" t="inlineStr"/>
-      <c r="AC16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1588,8 +1560,6 @@
           <t>其他</t>
         </is>
       </c>
-      <c r="AB17" t="inlineStr"/>
-      <c r="AC17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1654,8 +1624,6 @@
           <t>反思经验型</t>
         </is>
       </c>
-      <c r="AB18" t="inlineStr"/>
-      <c r="AC18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1720,8 +1688,6 @@
           <t>上下文/摘要型</t>
         </is>
       </c>
-      <c r="AB19" t="inlineStr"/>
-      <c r="AC19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1786,8 +1752,6 @@
           <t>结构化图谱型</t>
         </is>
       </c>
-      <c r="AB20" t="inlineStr"/>
-      <c r="AC20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1873,8 +1837,6 @@
           <t>其他</t>
         </is>
       </c>
-      <c r="AB21" t="inlineStr"/>
-      <c r="AC21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1960,8 +1922,6 @@
           <t>其他</t>
         </is>
       </c>
-      <c r="AB22" t="inlineStr"/>
-      <c r="AC22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2047,8 +2007,6 @@
           <t>参数/潜变量型</t>
         </is>
       </c>
-      <c r="AB23" t="inlineStr"/>
-      <c r="AC23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2134,8 +2092,6 @@
           <t>参数/潜变量型</t>
         </is>
       </c>
-      <c r="AB24" t="inlineStr"/>
-      <c r="AC24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2221,8 +2177,6 @@
           <t>反思经验型</t>
         </is>
       </c>
-      <c r="AB25" t="inlineStr"/>
-      <c r="AC25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2308,8 +2262,6 @@
           <t>分层管理型</t>
         </is>
       </c>
-      <c r="AB26" t="inlineStr"/>
-      <c r="AC26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2395,8 +2347,6 @@
           <t>分层管理型</t>
         </is>
       </c>
-      <c r="AB27" t="inlineStr"/>
-      <c r="AC27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2482,8 +2432,6 @@
           <t>分层管理型</t>
         </is>
       </c>
-      <c r="AB28" t="inlineStr"/>
-      <c r="AC28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2569,8 +2517,6 @@
           <t>其他</t>
         </is>
       </c>
-      <c r="AB29" t="inlineStr"/>
-      <c r="AC29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2656,8 +2602,6 @@
           <t>分层管理型</t>
         </is>
       </c>
-      <c r="AB30" t="inlineStr"/>
-      <c r="AC30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2743,8 +2687,6 @@
           <t>反思经验型</t>
         </is>
       </c>
-      <c r="AB31" t="inlineStr"/>
-      <c r="AC31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2830,8 +2772,6 @@
           <t>参数/潜变量型</t>
         </is>
       </c>
-      <c r="AB32" t="inlineStr"/>
-      <c r="AC32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2917,8 +2857,6 @@
           <t>检索型</t>
         </is>
       </c>
-      <c r="AB33" t="inlineStr"/>
-      <c r="AC33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3004,8 +2942,6 @@
           <t>上下文/摘要型</t>
         </is>
       </c>
-      <c r="AB34" t="inlineStr"/>
-      <c r="AC34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3091,8 +3027,6 @@
           <t>分层管理型</t>
         </is>
       </c>
-      <c r="AB35" t="inlineStr"/>
-      <c r="AC35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3178,8 +3112,6 @@
           <t>分层管理型</t>
         </is>
       </c>
-      <c r="AB36" t="inlineStr"/>
-      <c r="AC36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3269,8 +3201,6 @@
           <t>其他</t>
         </is>
       </c>
-      <c r="AB37" t="inlineStr"/>
-      <c r="AC37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3360,8 +3290,6 @@
           <t>分层管理型</t>
         </is>
       </c>
-      <c r="AB38" t="inlineStr"/>
-      <c r="AC38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3447,8 +3375,6 @@
           <t>参数/潜变量型</t>
         </is>
       </c>
-      <c r="AB39" t="inlineStr"/>
-      <c r="AC39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3534,8 +3460,6 @@
           <t>分层管理型</t>
         </is>
       </c>
-      <c r="AB40" t="inlineStr"/>
-      <c r="AC40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3621,8 +3545,6 @@
           <t>其他</t>
         </is>
       </c>
-      <c r="AB41" t="inlineStr"/>
-      <c r="AC41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3708,8 +3630,6 @@
           <t>其他</t>
         </is>
       </c>
-      <c r="AB42" t="inlineStr"/>
-      <c r="AC42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3795,8 +3715,6 @@
           <t>结构化图谱型</t>
         </is>
       </c>
-      <c r="AB43" t="inlineStr"/>
-      <c r="AC43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3882,8 +3800,6 @@
           <t>其他</t>
         </is>
       </c>
-      <c r="AB44" t="inlineStr"/>
-      <c r="AC44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3969,8 +3885,6 @@
           <t>其他</t>
         </is>
       </c>
-      <c r="AB45" t="inlineStr"/>
-      <c r="AC45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -4056,8 +3970,6 @@
           <t>结构化图谱型</t>
         </is>
       </c>
-      <c r="AB46" t="inlineStr"/>
-      <c r="AC46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4143,8 +4055,6 @@
           <t>检索型</t>
         </is>
       </c>
-      <c r="AB47" t="inlineStr"/>
-      <c r="AC47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4230,8 +4140,6 @@
           <t>参数/潜变量型</t>
         </is>
       </c>
-      <c r="AB48" t="inlineStr"/>
-      <c r="AC48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4317,8 +4225,6 @@
           <t>其他</t>
         </is>
       </c>
-      <c r="AB49" t="inlineStr"/>
-      <c r="AC49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4404,8 +4310,6 @@
           <t>分层管理型</t>
         </is>
       </c>
-      <c r="AB50" t="inlineStr"/>
-      <c r="AC50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4491,8 +4395,6 @@
           <t>检索型</t>
         </is>
       </c>
-      <c r="AB51" t="inlineStr"/>
-      <c r="AC51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4578,8 +4480,6 @@
           <t>其他</t>
         </is>
       </c>
-      <c r="AB52" t="inlineStr"/>
-      <c r="AC52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4665,8 +4565,6 @@
           <t>检索型</t>
         </is>
       </c>
-      <c r="AB53" t="inlineStr"/>
-      <c r="AC53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4837,8 +4735,6 @@
           <t>参数/潜变量型</t>
         </is>
       </c>
-      <c r="AB55" t="inlineStr"/>
-      <c r="AC55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4928,8 +4824,6 @@
           <t>结构化图谱型</t>
         </is>
       </c>
-      <c r="AB56" t="inlineStr"/>
-      <c r="AC56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4979,6 +4873,21 @@
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr"/>
+      <c r="Y57" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z57" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA57" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -5028,8 +4937,21 @@
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr"/>
-      <c r="AB58" t="inlineStr"/>
-      <c r="AC58" t="inlineStr"/>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z58" t="inlineStr">
+        <is>
+          <t>潜变量</t>
+        </is>
+      </c>
+      <c r="AA58" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -5079,6 +5001,21 @@
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z59" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA59" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -5128,6 +5065,21 @@
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr"/>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z60" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA60" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -5177,6 +5129,21 @@
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr"/>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z61" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA61" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -5226,6 +5193,21 @@
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr"/>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z62" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA62" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -5275,8 +5257,21 @@
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
-      <c r="AB63" t="inlineStr"/>
-      <c r="AC63" t="inlineStr"/>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z63" t="inlineStr">
+        <is>
+          <t>检索型</t>
+        </is>
+      </c>
+      <c r="AA63" t="inlineStr">
+        <is>
+          <t>检索型</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -5326,6 +5321,21 @@
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr"/>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z64" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA64" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -5375,6 +5385,21 @@
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr"/>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z65" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA65" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -5424,6 +5449,21 @@
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr"/>
+      <c r="Y66" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z66" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA66" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5473,8 +5513,21 @@
         </is>
       </c>
       <c r="K67" s="2" t="inlineStr"/>
-      <c r="AB67" t="inlineStr"/>
-      <c r="AC67" t="inlineStr"/>
+      <c r="Y67" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z67" t="inlineStr">
+        <is>
+          <t>结构化</t>
+        </is>
+      </c>
+      <c r="AA67" t="inlineStr">
+        <is>
+          <t>分层管理型</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5524,6 +5577,21 @@
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr"/>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z68" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA68" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -5573,8 +5641,21 @@
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
-      <c r="AB69" t="inlineStr"/>
-      <c r="AC69" t="inlineStr"/>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z69" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA69" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5624,6 +5705,21 @@
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z70" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA70" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5673,6 +5769,21 @@
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z71" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA71" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5722,6 +5833,21 @@
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr"/>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z72" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA72" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -5771,8 +5897,21 @@
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr"/>
-      <c r="AB73" t="inlineStr"/>
-      <c r="AC73" t="inlineStr"/>
+      <c r="Y73" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z73" t="inlineStr">
+        <is>
+          <t>检索型</t>
+        </is>
+      </c>
+      <c r="AA73" t="inlineStr">
+        <is>
+          <t>检索型</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -5822,8 +5961,21 @@
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
-      <c r="AB74" t="inlineStr"/>
-      <c r="AC74" t="inlineStr"/>
+      <c r="Y74" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z74" t="inlineStr">
+        <is>
+          <t>向量</t>
+        </is>
+      </c>
+      <c r="AA74" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -5873,8 +6025,21 @@
         </is>
       </c>
       <c r="K75" s="2" t="inlineStr"/>
-      <c r="AB75" t="inlineStr"/>
-      <c r="AC75" t="inlineStr"/>
+      <c r="Y75" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z75" t="inlineStr">
+        <is>
+          <t>结构化</t>
+        </is>
+      </c>
+      <c r="AA75" t="inlineStr">
+        <is>
+          <t>反思经验型</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -5924,6 +6089,21 @@
         </is>
       </c>
       <c r="K76" s="2" t="inlineStr"/>
+      <c r="Y76" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z76" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA76" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -5973,6 +6153,21 @@
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
+      <c r="Y77" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z77" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA77" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -6022,6 +6217,21 @@
         </is>
       </c>
       <c r="K78" s="2" t="inlineStr"/>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z78" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA78" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -6071,6 +6281,21 @@
         </is>
       </c>
       <c r="K79" s="2" t="inlineStr"/>
+      <c r="Y79" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z79" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA79" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -6120,6 +6345,21 @@
         </is>
       </c>
       <c r="K80" s="2" t="inlineStr"/>
+      <c r="Y80" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z80" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA80" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -6169,6 +6409,21 @@
         </is>
       </c>
       <c r="K81" s="2" t="inlineStr"/>
+      <c r="Y81" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z81" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA81" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -6218,6 +6473,21 @@
         </is>
       </c>
       <c r="K82" s="2" t="inlineStr"/>
+      <c r="Y82" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z82" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA82" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -6267,6 +6537,21 @@
         </is>
       </c>
       <c r="K83" s="2" t="inlineStr"/>
+      <c r="Y83" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z83" t="inlineStr">
+        <is>
+          <t>检索型</t>
+        </is>
+      </c>
+      <c r="AA83" t="inlineStr">
+        <is>
+          <t>检索型</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -6316,6 +6601,21 @@
         </is>
       </c>
       <c r="K84" s="2" t="inlineStr"/>
+      <c r="Y84" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z84" t="inlineStr">
+        <is>
+          <t>结构化</t>
+        </is>
+      </c>
+      <c r="AA84" t="inlineStr">
+        <is>
+          <t>结构化图谱型</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -6365,6 +6665,21 @@
         </is>
       </c>
       <c r="K85" s="2" t="inlineStr"/>
+      <c r="Y85" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z85" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA85" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -6414,8 +6729,21 @@
         </is>
       </c>
       <c r="K86" s="2" t="inlineStr"/>
-      <c r="AB86" t="inlineStr"/>
-      <c r="AC86" t="inlineStr"/>
+      <c r="Y86" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z86" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA86" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -6465,6 +6793,21 @@
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
+      <c r="Y87" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z87" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA87" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -6514,6 +6857,21 @@
         </is>
       </c>
       <c r="K88" s="2" t="inlineStr"/>
+      <c r="Y88" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z88" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA88" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -6563,6 +6921,21 @@
         </is>
       </c>
       <c r="K89" s="2" t="inlineStr"/>
+      <c r="Y89" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z89" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA89" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -6612,8 +6985,21 @@
         </is>
       </c>
       <c r="K90" s="2" t="inlineStr"/>
-      <c r="AB90" t="inlineStr"/>
-      <c r="AC90" t="inlineStr"/>
+      <c r="Y90" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z90" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA90" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -6663,8 +7049,21 @@
         </is>
       </c>
       <c r="K91" s="2" t="inlineStr"/>
-      <c r="AB91" t="inlineStr"/>
-      <c r="AC91" t="inlineStr"/>
+      <c r="Y91" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z91" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA91" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -6714,8 +7113,21 @@
         </is>
       </c>
       <c r="K92" s="2" t="inlineStr"/>
-      <c r="AB92" t="inlineStr"/>
-      <c r="AC92" t="inlineStr"/>
+      <c r="Y92" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z92" t="inlineStr">
+        <is>
+          <t>结构化</t>
+        </is>
+      </c>
+      <c r="AA92" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -6765,6 +7177,21 @@
         </is>
       </c>
       <c r="K93" s="2" t="inlineStr"/>
+      <c r="Y93" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z93" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA93" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -6814,8 +7241,21 @@
         </is>
       </c>
       <c r="K94" s="2" t="inlineStr"/>
-      <c r="AB94" t="inlineStr"/>
-      <c r="AC94" t="inlineStr"/>
+      <c r="Y94" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z94" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA94" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -6865,6 +7305,21 @@
         </is>
       </c>
       <c r="K95" s="2" t="inlineStr"/>
+      <c r="Y95" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z95" t="inlineStr">
+        <is>
+          <t>向量</t>
+        </is>
+      </c>
+      <c r="AA95" t="inlineStr">
+        <is>
+          <t>检索型</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -6914,8 +7369,21 @@
         </is>
       </c>
       <c r="K96" s="2" t="inlineStr"/>
-      <c r="AB96" t="inlineStr"/>
-      <c r="AC96" t="inlineStr"/>
+      <c r="Y96" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z96" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA96" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -6965,6 +7433,21 @@
         </is>
       </c>
       <c r="K97" s="2" t="inlineStr"/>
+      <c r="Y97" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z97" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA97" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -7014,8 +7497,21 @@
         </is>
       </c>
       <c r="K98" s="2" t="inlineStr"/>
-      <c r="AB98" t="inlineStr"/>
-      <c r="AC98" t="inlineStr"/>
+      <c r="Y98" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z98" t="inlineStr">
+        <is>
+          <t>向量</t>
+        </is>
+      </c>
+      <c r="AA98" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -7065,6 +7561,21 @@
         </is>
       </c>
       <c r="K99" s="2" t="inlineStr"/>
+      <c r="Y99" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z99" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA99" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -7114,6 +7625,21 @@
         </is>
       </c>
       <c r="K100" s="2" t="inlineStr"/>
+      <c r="Y100" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z100" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA100" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -7163,6 +7689,21 @@
         </is>
       </c>
       <c r="K101" s="2" t="inlineStr"/>
+      <c r="Y101" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z101" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA101" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -7212,8 +7753,21 @@
         </is>
       </c>
       <c r="K102" s="2" t="inlineStr"/>
-      <c r="AB102" t="inlineStr"/>
-      <c r="AC102" t="inlineStr"/>
+      <c r="Y102" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z102" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA102" t="inlineStr">
+        <is>
+          <t>反思经验型</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -7263,6 +7817,21 @@
         </is>
       </c>
       <c r="K103" s="2" t="inlineStr"/>
+      <c r="Y103" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z103" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA103" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -7312,6 +7881,21 @@
         </is>
       </c>
       <c r="K104" s="2" t="inlineStr"/>
+      <c r="Y104" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z104" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA104" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -7361,6 +7945,21 @@
         </is>
       </c>
       <c r="K105" s="2" t="inlineStr"/>
+      <c r="Y105" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z105" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA105" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -7410,8 +8009,21 @@
         </is>
       </c>
       <c r="K106" s="2" t="inlineStr"/>
-      <c r="AB106" t="inlineStr"/>
-      <c r="AC106" t="inlineStr"/>
+      <c r="Y106" t="inlineStr">
+        <is>
+          <t>多智能体模拟</t>
+        </is>
+      </c>
+      <c r="Z106" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="AA106" t="inlineStr">
+        <is>
+          <t>上下文/摘要型</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -7464,8 +8076,21 @@
           <t>/opt/data/home/hermes-arxiv-agent/papers/2501.11739.pdf</t>
         </is>
       </c>
-      <c r="AB107" t="inlineStr"/>
-      <c r="AC107" t="inlineStr"/>
+      <c r="Y107" t="inlineStr">
+        <is>
+          <t>个人助手</t>
+        </is>
+      </c>
+      <c r="Z107" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="AA107" t="inlineStr">
+        <is>
+          <t>反思经验型</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -7518,8 +8143,21 @@
           <t>/opt/data/home/hermes-arxiv-agent/papers/2501.14119.pdf</t>
         </is>
       </c>
-      <c r="AB108" t="inlineStr"/>
-      <c r="AC108" t="inlineStr"/>
+      <c r="Y108" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z108" t="inlineStr">
+        <is>
+          <t>结构化</t>
+        </is>
+      </c>
+      <c r="AA108" t="inlineStr">
+        <is>
+          <t>分层管理型</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -7572,8 +8210,21 @@
           <t>/opt/data/home/hermes-arxiv-agent/papers/2502.16090.pdf</t>
         </is>
       </c>
-      <c r="AB109" t="inlineStr"/>
-      <c r="AC109" t="inlineStr"/>
+      <c r="Y109" t="inlineStr">
+        <is>
+          <t>个人助手</t>
+        </is>
+      </c>
+      <c r="Z109" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="AA109" t="inlineStr">
+        <is>
+          <t>反思经验型</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -7626,8 +8277,21 @@
           <t>/opt/data/home/hermes-arxiv-agent/papers/2503.21760.pdf</t>
         </is>
       </c>
-      <c r="AB110" t="inlineStr"/>
-      <c r="AC110" t="inlineStr"/>
+      <c r="Y110" t="inlineStr">
+        <is>
+          <t>个人助手</t>
+        </is>
+      </c>
+      <c r="Z110" t="inlineStr">
+        <is>
+          <t>结构化</t>
+        </is>
+      </c>
+      <c r="AA110" t="inlineStr">
+        <is>
+          <t>检索型</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -7680,8 +8344,2037 @@
           <t>/opt/data/home/hermes-arxiv-agent/papers/2505.23422.pdf</t>
         </is>
       </c>
-      <c r="AB111" t="inlineStr"/>
-      <c r="AC111" t="inlineStr"/>
+      <c r="Y111" t="inlineStr">
+        <is>
+          <t>代码Agent</t>
+        </is>
+      </c>
+      <c r="Z111" t="inlineStr">
+        <is>
+          <t>结构化</t>
+        </is>
+      </c>
+      <c r="AA111" t="inlineStr">
+        <is>
+          <t>反思经验型</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2506.04565</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>From Standalone LLMs to Integrated Intelligence: A Survey of Compound Al Systems</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Jiayi Chen, Junyi Ye, Guiling Wang</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>cs.MA, cs.CL</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>综述复合AI系统范式，整合LLM与检索器、智能体、工具、编排器等外部组件，克服独立模型在记忆、推理、实时接地与多模态理解方面的局限。</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>2506.04565.pdf</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W112" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2506.04565</t>
+        </is>
+      </c>
+      <c r="X112" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2506.04565.pdf</t>
+        </is>
+      </c>
+      <c r="Y112" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z112" t="inlineStr">
+        <is>
+          <t>混合/其他</t>
+        </is>
+      </c>
+      <c r="AA112" t="inlineStr">
+        <is>
+          <t>分层管理型</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2508.15294</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>A Multi-Memory Segment System for Generating High-Quality Long-Term Memory Content in Agents</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Gaoke Zhang, Bo Wang, Yunlong Ma, Dongming Zhao, Zifei Yu</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>cs.AI, cs.CL, cs.MA</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>提出多记忆分段系统，模拟人类多维多组件记忆生成过程，超越简单摘要式记忆存储，从多维度生成高质量长期记忆内容填补研究空白。</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>2508.15294.pdf</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W113" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2508.15294</t>
+        </is>
+      </c>
+      <c r="X113" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2508.15294.pdf</t>
+        </is>
+      </c>
+      <c r="Y113" t="inlineStr">
+        <is>
+          <t>个人助手</t>
+        </is>
+      </c>
+      <c r="Z113" t="inlineStr">
+        <is>
+          <t>结构化</t>
+        </is>
+      </c>
+      <c r="AA113" t="inlineStr">
+        <is>
+          <t>分层管理型</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2511.02805</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>MemSearcher: Training LLMs to Reason, Search and Manage Memory via End-to-End Reinforcement Learning</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Qianhao Yuan, Jie Lou, Zichao Li, Jiawei Chen, Yaojie Lu, Hongyu Lin, Le Sun, Debing Zhang, Xianpei Han</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>cs.CL, cs.AI</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>提出MemSearcher框架，端到端强化学习训练LLM在多轮搜索中维护紧凑记忆，仅保留问题相关信息稳定上下文长度，降低计算开销。</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>2511.02805.pdf</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W114" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2511.02805</t>
+        </is>
+      </c>
+      <c r="X114" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2511.02805.pdf</t>
+        </is>
+      </c>
+      <c r="Y114" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z114" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="AA114" t="inlineStr">
+        <is>
+          <t>检索型</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2604.23938</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>TSAssistant: A Human-in-the-Loop Agentic Framework for Automated Target Safety Assessment</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Xiaochen Zheng, Zhiwen Jiang, Melanie Guerard, Klas Hatje, Tatyana Doktorova</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>cs.CL</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>提出多智能体框架TSAssistant支持药物靶点安全评估自动报告，模块化分段生成与人机协同设计，整合遗传、转录组、药理等多源证据。</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>2604.23938.pdf</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W115" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2604.23938</t>
+        </is>
+      </c>
+      <c r="X115" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2604.23938.pdf</t>
+        </is>
+      </c>
+      <c r="Y115" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z115" t="inlineStr">
+        <is>
+          <t>结构化</t>
+        </is>
+      </c>
+      <c r="AA115" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2604.24372</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>SeaEvo: Advancing Algorithm Discovery with Strategy Space Evolution</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Sichun Luo, Yi Huang, Haochen Luo, Fengyuan Liu, Guanzhi Deng, Lei Li, Qinghua Yao, Zefa Hu, Junlan Feng, Qi Liu</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>cs.CL, cs.AI, cs.NE</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>提出策略空间进化方法SeaEvo用于自动算法发现，将自然语言推理组织为持久群体策略状态而非瞬态变异上下文，引导进化搜索沿有前景方向前进。</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>2604.24372.pdf</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W116" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2604.24372</t>
+        </is>
+      </c>
+      <c r="X116" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2604.24372.pdf</t>
+        </is>
+      </c>
+      <c r="Y116" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z116" t="inlineStr">
+        <is>
+          <t>结构化</t>
+        </is>
+      </c>
+      <c r="AA116" t="inlineStr">
+        <is>
+          <t>反思经验型</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2605.06702</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>CASCADE: Case-Based Continual Adaptation for Large Language Models During Deployment</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Siyuan Guo, Yali Du, Hechang Chen, Yi Chang, Jun Wang</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>cs.AI, cs.CL, cs.LG</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>将部署时学习形式化为LLM生命周期第三阶段，提出案例持续适应方法CASCADE，使智能体从交互经验中持续学习，打破训练与部署的刚性分离。</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>2605.06702.pdf</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W117" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2605.06702</t>
+        </is>
+      </c>
+      <c r="X117" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2605.06702.pdf</t>
+        </is>
+      </c>
+      <c r="Y117" t="inlineStr">
+        <is>
+          <t>个人助手</t>
+        </is>
+      </c>
+      <c r="Z117" t="inlineStr">
+        <is>
+          <t>结构化</t>
+        </is>
+      </c>
+      <c r="AA117" t="inlineStr">
+        <is>
+          <t>反思经验型</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2605.06716</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>From Storage to Experience: A Survey on the Evolution of LLM Agent Memory Mechanisms</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Jinghao Luo, Yuchen Tian, Chuxue Cao, Ziyang Luo, Hongzhan Lin, Kaixin Li, Chuyi Kong, Ruichao Yang, Jing Ma</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>cs.AI, cs.CL</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>综述LLM智能体记忆机制从存储到经验的演变，提出操作系统工程与认知科学统一视角，梳理记忆在智能体架构中的核心作用与未来方向。</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>2605.06716.pdf</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W118" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2605.06716</t>
+        </is>
+      </c>
+      <c r="X118" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2605.06716.pdf</t>
+        </is>
+      </c>
+      <c r="Y118" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z118" t="inlineStr">
+        <is>
+          <t>混合/其他</t>
+        </is>
+      </c>
+      <c r="AA118" t="inlineStr">
+        <is>
+          <t>分层管理型</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2605.06731</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>When Routine Chats Turn Toxic: Unintended Long-Term State Poisoning in Personalized Agents</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Xiaoyu Xu, Minxin Du, Qipeng Xie, Haobin Ke, Qingqing Ye, Haibo Hu</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>cs.CR, cs.CL, cs.LG</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>发现并形式化无意识长期状态中毒风险：个性化智能体日常对话逐渐弱化确认边界、扩大工具默认范围、升级自主行为，提出系统化防御方案。</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>2605.06731.pdf</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W119" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2605.06731</t>
+        </is>
+      </c>
+      <c r="X119" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2605.06731.pdf</t>
+        </is>
+      </c>
+      <c r="Y119" t="inlineStr">
+        <is>
+          <t>个人助手</t>
+        </is>
+      </c>
+      <c r="Z119" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="AA119" t="inlineStr">
+        <is>
+          <t>反思经验型</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2605.06812</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Towards Security-Auditable LLM Agents: A Unified Graph Representation</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Chaofan Li, Lyuye Zhang, Jintao Zhai, Siyue Feng, Xichun Yang, Huahao Wang, Shihan Dou, Yu Ji, Yutao Hu, Yueming Wu, Yang Liu, Deqing Zou</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>cs.AI</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>提出统一图表示方法解决LLM智能体安全审计难题，将工具调用、记忆管理、多智能体协作建模为可追溯图结构，弥合底层事件与高层意图的语义鸿沟。</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>2605.06812.pdf</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W120" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2605.06812</t>
+        </is>
+      </c>
+      <c r="X120" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2605.06812.pdf</t>
+        </is>
+      </c>
+      <c r="Y120" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z120" t="inlineStr">
+        <is>
+          <t>结构化图谱型</t>
+        </is>
+      </c>
+      <c r="AA120" t="inlineStr">
+        <is>
+          <t>结构化图谱型</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2605.06924</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>A$^2$RD: Agentic Autoregressive Diffusion for Long Video Consistency</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Do Xuan Long, Yale Song, Min-Yen Kan, Tomas Pfister, Long T. Le</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>cs.CV, cs.AI</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>提出智能体自回归扩散架构A²RD用于长视频合成，通过检索-合成-精炼-更新闭环分离创意合成与一致性维护，三智能体协同管理记忆与生成。</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>2605.06924.pdf</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W121" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2605.06924</t>
+        </is>
+      </c>
+      <c r="X121" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2605.06924.pdf</t>
+        </is>
+      </c>
+      <c r="Y121" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z121" t="inlineStr">
+        <is>
+          <t>潜变量</t>
+        </is>
+      </c>
+      <c r="AA121" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2605.07042</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>The Context Gathering Decision Process: A POMDP Framework for Agentic Search</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Chinmaya Kausik, Adith Swaminathan, Nathan Kallus</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>cs.AI, cs.LG</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>将智能体上下文搜索建模为POMDP，解决大规模环境下工作记忆退化问题，提供结构化搜索基础设施防止冗余探索与重复循环。</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>2605.07042.pdf</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W122" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2605.07042</t>
+        </is>
+      </c>
+      <c r="X122" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2605.07042.pdf</t>
+        </is>
+      </c>
+      <c r="Y122" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z122" t="inlineStr">
+        <is>
+          <t>结构化</t>
+        </is>
+      </c>
+      <c r="AA122" t="inlineStr">
+        <is>
+          <t>检索型</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2605.07103</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>ARMOR: An Agentic Framework for Reaction Feasibility Prediction via Adaptive Utility-aware Multi-tool Reasoning</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Ye Liu, Botao Yu, Xinyi Ling, Daniel Adu-Ampratwum, Xia Ning</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>cs.AI, cs.MA</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>提出智能体框架ARMOR用于化学反应可行性预测，自适应效用感知多工具推理，动态选择最优工具组合解决单一工具覆盖面不足问题。</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>2605.07103.pdf</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W123" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2605.07103</t>
+        </is>
+      </c>
+      <c r="X123" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2605.07103.pdf</t>
+        </is>
+      </c>
+      <c r="Y123" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z123" t="inlineStr">
+        <is>
+          <t>混合/其他</t>
+        </is>
+      </c>
+      <c r="AA123" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2605.07110</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Securing Computer-Use Agents: A Unified Architecture-Lifecycle Framework for Deployment-Grounded Reliability</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Zejian Chen, Zhanyuan Liu, Chaozhuo Li, Mengxiang Han, Songyang Liu, Litian Zhang, Feng Gao, Yiming Hei, Xi Zhang</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>cs.CL, cs.SE</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>提出统一架构-生命周期框架保障计算机使用智能体安全，覆盖感知、规划、记忆使用、工具中介、权限与运行时监督六维度，超越任务成功评估范式。</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>2605.07110.pdf</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W124" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2605.07110</t>
+        </is>
+      </c>
+      <c r="X124" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2605.07110.pdf</t>
+        </is>
+      </c>
+      <c r="Y124" t="inlineStr">
+        <is>
+          <t>Web Agent</t>
+        </is>
+      </c>
+      <c r="Z124" t="inlineStr">
+        <is>
+          <t>结构化</t>
+        </is>
+      </c>
+      <c r="AA124" t="inlineStr">
+        <is>
+          <t>分层管理型</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2605.07129</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>RRCM: Ranking-Driven Retrieval over Collaborative and Meta Memories for LLM Recommendation</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Shijun Li, Wooseong Yang, Yu Wang, Tianxin Wei, Joydeep Ghosh</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>cs.IR, cs.AI, cs.LG</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>提出排序驱动协同与元记忆双通道检索框架RRCM，融合行为证据与物品元数据，解决LLM推荐中异构证据的上下文构建挑战。</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>2605.07129.pdf</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W125" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2605.07129</t>
+        </is>
+      </c>
+      <c r="X125" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2605.07129.pdf</t>
+        </is>
+      </c>
+      <c r="Y125" t="inlineStr">
+        <is>
+          <t>个人助手</t>
+        </is>
+      </c>
+      <c r="Z125" t="inlineStr">
+        <is>
+          <t>向量</t>
+        </is>
+      </c>
+      <c r="AA125" t="inlineStr">
+        <is>
+          <t>检索型</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2605.07180</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Learning Agent Routing From Early Experience</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Yimin Wang, Jiahao Qiu, Xuan Qi, Xinzhe Juan, Jingzhe Shi, Zelin Zhao, Hongru Wang, Shilong Liu, Mengdi Wang</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>cs.CL</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>提出BoundaryRouter免训练路由框架，冷启动条件下判断查询应使用轻量LLM还是完整智能体执行，利用早期经验学习路由策略降低延迟成本。</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>2605.07180.pdf</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W126" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2605.07180</t>
+        </is>
+      </c>
+      <c r="X126" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2605.07180.pdf</t>
+        </is>
+      </c>
+      <c r="Y126" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z126" t="inlineStr">
+        <is>
+          <t>结构化</t>
+        </is>
+      </c>
+      <c r="AA126" t="inlineStr">
+        <is>
+          <t>分层管理型</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2605.07214</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>HMACE: Heterogeneous Multi-Agent Collaborative Evolution for Combinatorial Optimization</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Yuping Yan, Jirui Han, Fei Ming, Yuanshuai Li, Yaochu Jin</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>cs.AI</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>提出异构多智能体协同进化框架HMACE，突破单智能体模板化局限，通过记忆引导探索避免局部最优，实现组合优化启发式自主协同设计。</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>2605.07214.pdf</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W127" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2605.07214</t>
+        </is>
+      </c>
+      <c r="X127" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2605.07214.pdf</t>
+        </is>
+      </c>
+      <c r="Y127" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z127" t="inlineStr">
+        <is>
+          <t>结构化</t>
+        </is>
+      </c>
+      <c r="AA127" t="inlineStr">
+        <is>
+          <t>反思经验型</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2605.07242</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>MEMOREPAIR: Barrier-First Cascade Repair in Agentic Memory</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Yang Zhao, Chengxiao Dai, Mengying Kou, Yue Xiu</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>cs.AI, cs.CL</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>形式化智能体记忆的级联更新问题：源数据变更导致派生摘要、缓存陈旧。提出MemoRepair障碍优先级联修复策略，维护记忆派生状态一致性。</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>2605.07242.pdf</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W128" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2605.07242</t>
+        </is>
+      </c>
+      <c r="X128" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2605.07242.pdf</t>
+        </is>
+      </c>
+      <c r="Y128" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z128" t="inlineStr">
+        <is>
+          <t>结构化</t>
+        </is>
+      </c>
+      <c r="AA128" t="inlineStr">
+        <is>
+          <t>分层管理型</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2605.07313</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>When Stored Evidence Stops Being Usable: Scale-Conditioned Evaluation of Agent Memory</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Jiaqi Shao, Yiyi Lu, Yunzhen Zhang, Bing Luo</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>cs.AI</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>提出规模条件化评估协议，固定任务证据逐步增加无关会话，测量记忆智能体四项诊断指标——预算消耗、检索质量、推理稳定性与污染率。</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>2605.07313.pdf</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W129" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2605.07313</t>
+        </is>
+      </c>
+      <c r="X129" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2605.07313.pdf</t>
+        </is>
+      </c>
+      <c r="Y129" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z129" t="inlineStr">
+        <is>
+          <t>结构化</t>
+        </is>
+      </c>
+      <c r="AA129" t="inlineStr">
+        <is>
+          <t>检索型</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2605.07692</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>GASim: A Graph-Accelerated Hybrid Framework for Social Simulation</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Xuan Zhou, Yanhui Sun, Hantao Yao, Allen He, Yongdong Zhang, Wu Liu</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>cs.AI</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>提出图加速混合多智能体框架GASim用于大规模社会模拟，通过图结构化记忆检索替代顺序检索，显著降低LLM驱动智能体延迟与计算开销。</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>2605.07692.pdf</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W130" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2605.07692</t>
+        </is>
+      </c>
+      <c r="X130" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2605.07692.pdf</t>
+        </is>
+      </c>
+      <c r="Y130" t="inlineStr">
+        <is>
+          <t>多智能体模拟</t>
+        </is>
+      </c>
+      <c r="Z130" t="inlineStr">
+        <is>
+          <t>结构化</t>
+        </is>
+      </c>
+      <c r="AA130" t="inlineStr">
+        <is>
+          <t>检索型</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2605.07863</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>ADKO: Agentic Decentralized Knowledge Optimization</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Lucas Nerone Rillo, Zhanhong Jiang, Nastaran Saadati, Aditya Balu, Baskar Ganapathysubramanian, Chinmay Hegde, Soumik Sarkar</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>cs.LG</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>提出去中心化知识优化框架ADKO，各智能体维护私有高斯过程模型，仅通过紧凑知识令牌通信，实现样本高效、隐私保护的协同黑箱优化。</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>2605.07863.pdf</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W131" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2605.07863</t>
+        </is>
+      </c>
+      <c r="X131" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2605.07863.pdf</t>
+        </is>
+      </c>
+      <c r="Y131" t="inlineStr">
+        <is>
+          <t>多智能体模拟</t>
+        </is>
+      </c>
+      <c r="Z131" t="inlineStr">
+        <is>
+          <t>参数化</t>
+        </is>
+      </c>
+      <c r="AA131" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2605.08060</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>The Memory Curse: How Expanded Recall Erodes Cooperative Intent in LLM Agents</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Jiayuan Liu, Tianqin Li, Shiyi Du, Xin Luo, Haoxuan Zeng, Emanuel Tewolde, Tai Sing Lee, Tonghan Wang, Carl Kingsford, Vincent Conitzer</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Mon,</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>cs.CL, cs.AI, cs.GT, cs.MA</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>发现LLM上下文窗口扩展在多智能体社会困境中反而降低合作意愿，称为记忆诅咒。归因于前瞻性推理意图退化与逐轮激励机制侵蚀，7个LLM、4种游戏、500轮实验验证。</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>2605.08060.pdf</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="W132" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2605.08060</t>
+        </is>
+      </c>
+      <c r="X132" t="inlineStr">
+        <is>
+          <t>/opt/data/home/hermes-arxiv-agent/papers/2605.08060.pdf</t>
+        </is>
+      </c>
+      <c r="Y132" t="inlineStr">
+        <is>
+          <t>多智能体模拟</t>
+        </is>
+      </c>
+      <c r="Z132" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="AA132" t="inlineStr">
+        <is>
+          <t>反思经验型</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2304.03442</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Generative Agents: Interactive Simulacra of Human Behavior</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Joon Sung Park, Joseph C. O'Brien, Carrie J. Cai, Meredith Ringel Morris, Percy Liang, Michael S. Bernstein</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr"/>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>2023-04-07</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>cs.HC, cs.AI, cs.LG</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Believable proxies of human behavior can empower interactive applications ranging from immersive environments to rehearsal spaces for interpersonal communication to prototyping tools. In this paper, we introduce generative agents--computational software agents that simulate believable human behavior. Generative agents wake up, cook breakfast, and head to work; artists paint, while authors write; they form opinions, notice each other, and initiate conversations; they remember and reflect on days past as they plan the next day. To enable generative agents, we describe an architecture that extends a large language model to store a complete record of the agent's experiences using natural language, synthesize those memories over time into higher-level reflections, and retrieve them dynamically to plan behavior. We instantiate generative agents to populate an interactive sandbox environment inspired by The Sims, where end users can interact with a small town of twenty five agents using natural language. In an evaluation, these generative agents produce believable individual and emergent social behaviors: for example, starting with only a single user-specified notion that one agent wants to throw a Valentine's Day party, the agents autonomously spread invitations to the party over the next two days, make new acquaintances, ask each other out on dates to the party, and coordinate to show up for the party together at the right time. We demonstrate through ablation that the components of our agent architecture--observation, planning, and reflection--each contribute critically to the believability of agent behavior. By fusing large language models with computational, interactive agents, this work introduces architectural and interaction patterns for enabling believable simulations of human behavior.</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>提出生成式智能体(Generative Agents)架构，扩展LLM以自然语言存储智能体的完整经历、将记忆合成为高层反思、并动态检索以规划行为。在模拟小镇中，25个智能体展现出可信的个体和涌现社交行为（如自主组织情人节派对）。消融实验证明观察-规划-反思三个组件对行为可信性均至关重要。这是Agent Memory领域的奠基之作，引入了Memory Stream概念。</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr"/>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>[Milestone] Foundational paper in Agent Memory research</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr"/>
+      <c r="M133" t="inlineStr"/>
+      <c r="N133" t="inlineStr"/>
+      <c r="O133" t="inlineStr"/>
+      <c r="P133" t="inlineStr"/>
+      <c r="Q133" t="inlineStr"/>
+      <c r="R133" t="inlineStr"/>
+      <c r="S133" t="inlineStr"/>
+      <c r="T133" t="inlineStr"/>
+      <c r="U133" t="inlineStr"/>
+      <c r="V133" t="inlineStr"/>
+      <c r="W133" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2304.03442v2</t>
+        </is>
+      </c>
+      <c r="X133" t="inlineStr"/>
+      <c r="Y133" t="inlineStr">
+        <is>
+          <t>多智能体模拟</t>
+        </is>
+      </c>
+      <c r="Z133" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="AA133" t="inlineStr">
+        <is>
+          <t>反思经验型</t>
+        </is>
+      </c>
+      <c r="AB133" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AC133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2303.11366</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Reflexion: Language Agents with Verbal Reinforcement Learning</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Noah Shinn, Federico Cassano, Edward Berman, Ashwin Gopinath, Karthik Narasimhan, Shunyu Yao</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr"/>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>2023-03-20</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>cs.AI, cs.CL, cs.LG</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Large language models (LLMs) have been increasingly used to interact with external environments (e.g., games, compilers, APIs) as goal-driven agents. However, it remains challenging for these language agents to quickly and efficiently learn from trial-and-error as traditional reinforcement learning methods require extensive training samples and expensive model fine-tuning. We propose Reflexion, a novel framework to reinforce language agents not by updating weights, but instead through linguistic feedback. Concretely, Reflexion agents verbally reflect on task feedback signals, then maintain their own reflective text in an episodic memory buffer to induce better decision-making in subsequent trials. Reflexion is flexible enough to incorporate various types (scalar values or free-form language) and sources (external or internally simulated) of feedback signals, and obtains significant improvements over a baseline agent across diverse tasks (sequential decision-making, coding, language reasoning). For example, Reflexion achieves a 91% pass@1 accuracy on the HumanEval coding benchmark, surpassing the previous state-of-the-art GPT-4 that achieves 80%. We also conduct ablation and analysis studies using different feedback signals, feedback incorporation methods, and agent types, and provide insights into how they affect performance.</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>提出Reflexion框架，通过语言反馈而非权重更新来强化语言智能体。智能体对任务反馈信号进行口头反思，将反思文本维护在情景记忆缓冲区中，以改进后续决策。Reflexion支持多种反馈类型（标量值或自由语言）和来源（外部或内部模拟）。在HumanEval编程基准上达到91% pass@1准确率，超过GPT-4的80%。这是反思型Agent Memory的里程碑工作。</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>[Milestone] Foundational paper in Agent Memory research</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr"/>
+      <c r="M134" t="inlineStr"/>
+      <c r="N134" t="inlineStr"/>
+      <c r="O134" t="inlineStr"/>
+      <c r="P134" t="inlineStr"/>
+      <c r="Q134" t="inlineStr"/>
+      <c r="R134" t="inlineStr"/>
+      <c r="S134" t="inlineStr"/>
+      <c r="T134" t="inlineStr"/>
+      <c r="U134" t="inlineStr"/>
+      <c r="V134" t="inlineStr"/>
+      <c r="W134" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2303.11366v4</t>
+        </is>
+      </c>
+      <c r="X134" t="inlineStr"/>
+      <c r="Y134" t="inlineStr">
+        <is>
+          <t>代码Agent</t>
+        </is>
+      </c>
+      <c r="Z134" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="AA134" t="inlineStr">
+        <is>
+          <t>反思经验型</t>
+        </is>
+      </c>
+      <c r="AB134" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AC134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2310.08560</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>MemGPT: Towards LLMs as Operating Systems</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Charles Packer, Sarah Wooders, Kevin Lin, Vivian Fang, Shishir G. Patil, Ion Stoica, Joseph E. Gonzalez</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr"/>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>2023-10-12</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>cs.AI</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Large language models (LLMs) have revolutionized AI, but are constrained by limited context windows, hindering their utility in tasks like extended conversations and document analysis. To enable using context beyond limited context windows, we propose virtual context management, a technique drawing inspiration from hierarchical memory systems in traditional operating systems that provide the appearance of large memory resources through data movement between fast and slow memory. Using this technique, we introduce MemGPT (Memory-GPT), a system that intelligently manages different memory tiers in order to effectively provide extended context within the LLM's limited context window, and utilizes interrupts to manage control flow between itself and the user. We evaluate our OS-inspired design in two domains where the limited context windows of modern LLMs severely handicaps their performance: document analysis, where MemGPT is able to analyze large documents that far exceed the underlying LLM's context window, and multi-session chat, where MemGPT can create conversational agents that remember, reflect, and evolve dynamically through long-term interactions with their users. We release MemGPT code and data for our experiments at https://memgpt.ai.</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>借鉴操作系统的分层内存管理思想，提出虚拟上下文管理技术，通过数据在快速和慢速内存之间的移动来提供超越LLM上下文窗口限制的扩展上下文。MemGPT系统智能管理不同内存层级，利用中断管理控制流。在文档分析（处理远超上下文窗口的大型文档）和多轮对话（创建能记忆、反思、动态演进的对话智能体）两个领域验证了有效性。这是分层记忆管理的开创性工作。</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr"/>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>[Milestone] Foundational paper in Agent Memory research</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr"/>
+      <c r="M135" t="inlineStr"/>
+      <c r="N135" t="inlineStr"/>
+      <c r="O135" t="inlineStr"/>
+      <c r="P135" t="inlineStr"/>
+      <c r="Q135" t="inlineStr"/>
+      <c r="R135" t="inlineStr"/>
+      <c r="S135" t="inlineStr"/>
+      <c r="T135" t="inlineStr"/>
+      <c r="U135" t="inlineStr"/>
+      <c r="V135" t="inlineStr"/>
+      <c r="W135" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2310.08560v2</t>
+        </is>
+      </c>
+      <c r="X135" t="inlineStr"/>
+      <c r="Y135" t="inlineStr">
+        <is>
+          <t>个人助手</t>
+        </is>
+      </c>
+      <c r="Z135" t="inlineStr">
+        <is>
+          <t>混合/其他</t>
+        </is>
+      </c>
+      <c r="AA135" t="inlineStr">
+        <is>
+          <t>分层管理型</t>
+        </is>
+      </c>
+      <c r="AB135" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AC135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2305.16291</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Voyager: An Open-Ended Embodied Agent with Large Language Models</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Guanzhi Wang, Yuqi Xie, Yunfan Jiang, Ajay Mandlekar, Chaowei Xiao, Yuke Zhu, Linxi Fan, Anima Anandkumar</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr"/>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>2023-05-25</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>cs.AI, cs.LG</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>We introduce Voyager, the first LLM-powered embodied lifelong learning agent in Minecraft that continuously explores the world, acquires diverse skills, and makes novel discoveries without human intervention. Voyager consists of three key components: 1) an automatic curriculum that maximizes exploration, 2) an ever-growing skill library of executable code for storing and retrieving complex behaviors, and 3) a new iterative prompting mechanism that incorporates environment feedback, execution errors, and self-verification for program improvement. Voyager interacts with GPT-4 via blackbox queries, which bypasses the need for model parameter fine-tuning. The skills developed by Voyager are temporally extended, interpretable, and compositional, which compounds the agent's abilities rapidly and alleviates catastrophic forgetting. Empirically, Voyager shows strong in-context lifelong learning capability and exhibits exceptional proficiency in playing Minecraft. It obtains 3.3x more unique items, travels 2.3x longer distances, and unlocks key tech tree milestones up to 15.3x faster than prior SOTA. Voyager is able to utilize the learned skill library in a new Minecraft world to solve novel tasks from scratch, while other techniques struggle to generalize. We open-source our full codebase and prompts at https://voyager.minedojo.org/.</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>提出Voyager，首个LLM驱动的Minecraft具身终身学习智能体，无需人类干预即可持续探索世界、获取多样化技能并做出新发现。三大核心组件：自动课程（最大化探索）、不断增长的技能库（存储和检索可执行代码）、迭代提示机制（整合环境反馈和自验证）。Voyager获得3.3倍独特物品、行进2.3倍距离、解锁科技树里程碑快15.3倍。技能库支持跨世界泛化。</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr"/>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>[Milestone] Foundational paper in Agent Memory research</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr"/>
+      <c r="M136" t="inlineStr"/>
+      <c r="N136" t="inlineStr"/>
+      <c r="O136" t="inlineStr"/>
+      <c r="P136" t="inlineStr"/>
+      <c r="Q136" t="inlineStr"/>
+      <c r="R136" t="inlineStr"/>
+      <c r="S136" t="inlineStr"/>
+      <c r="T136" t="inlineStr"/>
+      <c r="U136" t="inlineStr"/>
+      <c r="V136" t="inlineStr"/>
+      <c r="W136" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2305.16291v2</t>
+        </is>
+      </c>
+      <c r="X136" t="inlineStr"/>
+      <c r="Y136" t="inlineStr">
+        <is>
+          <t>具身Agent</t>
+        </is>
+      </c>
+      <c r="Z136" t="inlineStr">
+        <is>
+          <t>结构化</t>
+        </is>
+      </c>
+      <c r="AA136" t="inlineStr">
+        <is>
+          <t>检索型</t>
+        </is>
+      </c>
+      <c r="AB136" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AC136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2309.02427</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Cognitive Architectures for Language Agents</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Theodore R. Sumers, Shunyu Yao, Karthik Narasimhan, Thomas L. Griffiths</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr"/>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>2023-09-05</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>cs.AI, cs.CL, cs.LG, cs.SC</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Recent efforts have augmented large language models (LLMs) with external resources (e.g., the Internet) or internal control flows (e.g., prompt chaining) for tasks requiring grounding or reasoning, leading to a new class of language agents. While these agents have achieved substantial empirical success, we lack a systematic framework to organize existing agents and plan future developments. In this paper, we draw on the rich history of cognitive science and symbolic artificial intelligence to propose Cognitive Architectures for Language Agents (CoALA). CoALA describes a language agent with modular memory components, a structured action space to interact with internal memory and external environments, and a generalized decision-making process to choose actions. We use CoALA to retrospectively survey and organize a large body of recent work, and prospectively identify actionable directions towards more capable agents. Taken together, CoALA contextualizes today's language agents within the broader history of AI and outlines a path towards language-based general intelligence.</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>借鉴认知科学和符号AI的丰富历史，提出语言智能体的认知架构(CoALA)。CoALA描述了具有模块化记忆组件、结构化动作空间（与内部记忆和外部环境交互）以及通用决策过程的语言智能体。论文回顾性地梳理了大量近期工作，并前瞻性地识别出通往更强大智能体的可行方向。CoALA将当今语言智能体置于更广阔的AI历史背景中。</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>[Milestone] Foundational paper in Agent Memory research</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr"/>
+      <c r="M137" t="inlineStr"/>
+      <c r="N137" t="inlineStr"/>
+      <c r="O137" t="inlineStr"/>
+      <c r="P137" t="inlineStr"/>
+      <c r="Q137" t="inlineStr"/>
+      <c r="R137" t="inlineStr"/>
+      <c r="S137" t="inlineStr"/>
+      <c r="T137" t="inlineStr"/>
+      <c r="U137" t="inlineStr"/>
+      <c r="V137" t="inlineStr"/>
+      <c r="W137" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2309.02427v3</t>
+        </is>
+      </c>
+      <c r="X137" t="inlineStr"/>
+      <c r="Y137" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z137" t="inlineStr">
+        <is>
+          <t>混合/其他</t>
+        </is>
+      </c>
+      <c r="AA137" t="inlineStr">
+        <is>
+          <t>分层管理型</t>
+        </is>
+      </c>
+      <c r="AB137" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AC137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2404.13501</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>A Survey on the Memory Mechanism of Large Language Model based Agents</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Zeyu Zhang, Xiaohe Bo, Chen Ma, Rui Li, Xu Chen, Quanyu Dai, Jieming Zhu, Zhenhua Dong, Ji-Rong Wen</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr"/>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>2024-04-21</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>cs.AI</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Large language model (LLM) based agents have recently attracted much attention from the research and industry communities. Compared with original LLMs, LLM-based agents are featured in their self-evolving capability, which is the basis for solving real-world problems that need long-term and complex agent-environment interactions. The key component to support agent-environment interactions is the memory of the agents. While previous studies have proposed many promising memory mechanisms, they are scattered in different papers, and there lacks a systematical review to summarize and compare these works from a holistic perspective, failing to abstract common and effective designing patterns for inspiring future studies. To bridge this gap, in this paper, we propose a comprehensive survey on the memory mechanism of LLM-based agents. In specific, we first discuss ''what is'' and ''why do we need'' the memory in LLM-based agents. Then, we systematically review previous studies on how to design and evaluate the memory module. In addition, we also present many agent applications, where the memory module plays an important role. At last, we analyze the limitations of existing work and show important future directions. To keep up with the latest advances in this field, we create a repository at \url{https://github.com/nuster1128/LLM_Agent_Memory_Survey}.</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>首篇系统综述LLM智能体记忆机制。讨论了LLM智能体中记忆的"是什么"和"为什么需要"，系统回顾了记忆模块的设计和评估方法。提出了记忆机制的分类体系，涵盖记忆的来源、形式、操作和更新策略。同时介绍了记忆模块发挥重要作用的智能体应用场景。创建了持续更新的GitHub仓库跟踪该领域最新进展。</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr"/>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>[Milestone] Foundational paper in Agent Memory research</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr"/>
+      <c r="M138" t="inlineStr"/>
+      <c r="N138" t="inlineStr"/>
+      <c r="O138" t="inlineStr"/>
+      <c r="P138" t="inlineStr"/>
+      <c r="Q138" t="inlineStr"/>
+      <c r="R138" t="inlineStr"/>
+      <c r="S138" t="inlineStr"/>
+      <c r="T138" t="inlineStr"/>
+      <c r="U138" t="inlineStr"/>
+      <c r="V138" t="inlineStr"/>
+      <c r="W138" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2404.13501v1</t>
+        </is>
+      </c>
+      <c r="X138" t="inlineStr"/>
+      <c r="Y138" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z138" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="AA138" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="AB138" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AC138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2402.02716</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Understanding the planning of LLM agents: A survey</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Xu Huang, Weiwen Liu, Xiaolong Chen, Xingmei Wang, Hao Wang, Defu Lian, Yasheng Wang, Ruiming Tang, Enhong Chen</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr"/>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>2024-02-05</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>cs.AI, cs.CL, cs.LG</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>As Large Language Models (LLMs) have shown significant intelligence, the progress to leverage LLMs as planning modules of autonomous agents has attracted more attention. This survey provides the first systematic view of LLM-based agents planning, covering recent works aiming to improve planning ability. We provide a taxonomy of existing works on LLM-Agent planning, which can be categorized into Task Decomposition, Plan Selection, External Module, Reflection and Memory. Comprehensive analyses are conducted for each direction, and further challenges for the field of research are discussed.</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>首篇系统综述LLM智能体规划能力。提出了LLM智能体规划的分类体系：任务分解、计划选择、外部模块、反思与记忆。对每个方向进行了全面分析，讨论了该领域面临的挑战。该综述将记忆作为LLM智能体规划的关键组成部分加以分析。</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr"/>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>[Milestone] Foundational paper in Agent Memory research</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr"/>
+      <c r="M139" t="inlineStr"/>
+      <c r="N139" t="inlineStr"/>
+      <c r="O139" t="inlineStr"/>
+      <c r="P139" t="inlineStr"/>
+      <c r="Q139" t="inlineStr"/>
+      <c r="R139" t="inlineStr"/>
+      <c r="S139" t="inlineStr"/>
+      <c r="T139" t="inlineStr"/>
+      <c r="U139" t="inlineStr"/>
+      <c r="V139" t="inlineStr"/>
+      <c r="W139" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2402.02716v1</t>
+        </is>
+      </c>
+      <c r="X139" t="inlineStr"/>
+      <c r="Y139" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z139" t="inlineStr">
+        <is>
+          <t>文本</t>
+        </is>
+      </c>
+      <c r="AA139" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="AB139" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="AC139" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: add 44 peer-reviewed 2025-2026 papers from Semantic Scholar citations - 50 peer-reviewed out of 131 total (38.2%) - Top venues: EMNLP(6), ACL(4), WWW(6), CHI(6), AAAI(2), ICML(2), ICLR(2) - Papers discovered via citation chain from 6 core papers - Updated build_data.py for has_review field - UI: 4-row filter layout with review-only toggle, card actions row
</commit_message>
<xml_diff>
--- a/papers_record.xlsx
+++ b/papers_record.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC139"/>
+  <dimension ref="A1:AC186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1467,7 +1467,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>提出BeliefMem，将代理记忆范式从单一确定性结论转向保留多个候选结论及其概率，通过Noisy-OR规则更新。检索时所有候选方案与其概率一同展示，保持不确定性可见。在LoCoMo和ALFWorld上达到最佳平均性能，开辟了部分可观测环境中概率记忆的新方向。</t>
+          <t>本文提出Belief Memory框架，针对LLM智能体在部分可观测环境下长期记忆的确定性偏差问题，将观测信息存储为概率化信念而非单一结论。该方法使智能体能够保留不确定性，在新证据出现时动态修正先前判断，从而避免自强化错误，提升长期决策的鲁棒性与记忆可靠性。</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr"/>
@@ -8091,6 +8091,16 @@
           <t>反思经验型</t>
         </is>
       </c>
+      <c r="AB107" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC107" t="inlineStr">
+        <is>
+          <t>2025 IEEE Conference on Secure and Trustworthy Machine Learning (SaTML)</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -8292,6 +8302,16 @@
           <t>检索型</t>
         </is>
       </c>
+      <c r="AB110" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC110" t="inlineStr">
+        <is>
+          <t>EMNLP 2025</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -9783,7 +9803,6 @@
           <t>Joon Sung Park, Joseph C. O'Brien, Carrie J. Cai, Meredith Ringel Morris, Percy Liang, Michael S. Bernstein</t>
         </is>
       </c>
-      <c r="D133" t="inlineStr"/>
       <c r="E133" t="inlineStr">
         <is>
           <t>2023-04-07</t>
@@ -9804,7 +9823,6 @@
           <t>提出生成式智能体(Generative Agents)架构，扩展LLM以自然语言存储智能体的完整经历、将记忆合成为高层反思、并动态检索以规划行为。在模拟小镇中，25个智能体展现出可信的个体和涌现社交行为（如自主组织情人节派对）。消融实验证明观察-规划-反思三个组件对行为可信性均至关重要。这是Agent Memory领域的奠基之作，引入了Memory Stream概念。</t>
         </is>
       </c>
-      <c r="I133" t="inlineStr"/>
       <c r="J133" t="inlineStr">
         <is>
           <t>2026-05-11</t>
@@ -9815,23 +9833,11 @@
           <t>[Milestone] Foundational paper in Agent Memory research</t>
         </is>
       </c>
-      <c r="L133" t="inlineStr"/>
-      <c r="M133" t="inlineStr"/>
-      <c r="N133" t="inlineStr"/>
-      <c r="O133" t="inlineStr"/>
-      <c r="P133" t="inlineStr"/>
-      <c r="Q133" t="inlineStr"/>
-      <c r="R133" t="inlineStr"/>
-      <c r="S133" t="inlineStr"/>
-      <c r="T133" t="inlineStr"/>
-      <c r="U133" t="inlineStr"/>
-      <c r="V133" t="inlineStr"/>
       <c r="W133" t="inlineStr">
         <is>
           <t>https://arxiv.org/pdf/2304.03442v2</t>
         </is>
       </c>
-      <c r="X133" t="inlineStr"/>
       <c r="Y133" t="inlineStr">
         <is>
           <t>多智能体模拟</t>
@@ -9849,10 +9855,14 @@
       </c>
       <c r="AB133" t="inlineStr">
         <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="AC133" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC133" t="inlineStr">
+        <is>
+          <t>ACM Symposium on User Interface Software and Technology</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -9870,7 +9880,6 @@
           <t>Noah Shinn, Federico Cassano, Edward Berman, Ashwin Gopinath, Karthik Narasimhan, Shunyu Yao</t>
         </is>
       </c>
-      <c r="D134" t="inlineStr"/>
       <c r="E134" t="inlineStr">
         <is>
           <t>2023-03-20</t>
@@ -9891,7 +9900,6 @@
           <t>提出Reflexion框架，通过语言反馈而非权重更新来强化语言智能体。智能体对任务反馈信号进行口头反思，将反思文本维护在情景记忆缓冲区中，以改进后续决策。Reflexion支持多种反馈类型（标量值或自由语言）和来源（外部或内部模拟）。在HumanEval编程基准上达到91% pass@1准确率，超过GPT-4的80%。这是反思型Agent Memory的里程碑工作。</t>
         </is>
       </c>
-      <c r="I134" t="inlineStr"/>
       <c r="J134" t="inlineStr">
         <is>
           <t>2026-05-11</t>
@@ -9902,23 +9910,11 @@
           <t>[Milestone] Foundational paper in Agent Memory research</t>
         </is>
       </c>
-      <c r="L134" t="inlineStr"/>
-      <c r="M134" t="inlineStr"/>
-      <c r="N134" t="inlineStr"/>
-      <c r="O134" t="inlineStr"/>
-      <c r="P134" t="inlineStr"/>
-      <c r="Q134" t="inlineStr"/>
-      <c r="R134" t="inlineStr"/>
-      <c r="S134" t="inlineStr"/>
-      <c r="T134" t="inlineStr"/>
-      <c r="U134" t="inlineStr"/>
-      <c r="V134" t="inlineStr"/>
       <c r="W134" t="inlineStr">
         <is>
           <t>https://arxiv.org/pdf/2303.11366v4</t>
         </is>
       </c>
-      <c r="X134" t="inlineStr"/>
       <c r="Y134" t="inlineStr">
         <is>
           <t>代码Agent</t>
@@ -9936,10 +9932,14 @@
       </c>
       <c r="AB134" t="inlineStr">
         <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="AC134" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC134" t="inlineStr">
+        <is>
+          <t>Neural Information Processing Systems</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -9957,7 +9957,6 @@
           <t>Charles Packer, Sarah Wooders, Kevin Lin, Vivian Fang, Shishir G. Patil, Ion Stoica, Joseph E. Gonzalez</t>
         </is>
       </c>
-      <c r="D135" t="inlineStr"/>
       <c r="E135" t="inlineStr">
         <is>
           <t>2023-10-12</t>
@@ -9978,7 +9977,6 @@
           <t>借鉴操作系统的分层内存管理思想，提出虚拟上下文管理技术，通过数据在快速和慢速内存之间的移动来提供超越LLM上下文窗口限制的扩展上下文。MemGPT系统智能管理不同内存层级，利用中断管理控制流。在文档分析（处理远超上下文窗口的大型文档）和多轮对话（创建能记忆、反思、动态演进的对话智能体）两个领域验证了有效性。这是分层记忆管理的开创性工作。</t>
         </is>
       </c>
-      <c r="I135" t="inlineStr"/>
       <c r="J135" t="inlineStr">
         <is>
           <t>2026-05-11</t>
@@ -9989,23 +9987,11 @@
           <t>[Milestone] Foundational paper in Agent Memory research</t>
         </is>
       </c>
-      <c r="L135" t="inlineStr"/>
-      <c r="M135" t="inlineStr"/>
-      <c r="N135" t="inlineStr"/>
-      <c r="O135" t="inlineStr"/>
-      <c r="P135" t="inlineStr"/>
-      <c r="Q135" t="inlineStr"/>
-      <c r="R135" t="inlineStr"/>
-      <c r="S135" t="inlineStr"/>
-      <c r="T135" t="inlineStr"/>
-      <c r="U135" t="inlineStr"/>
-      <c r="V135" t="inlineStr"/>
       <c r="W135" t="inlineStr">
         <is>
           <t>https://arxiv.org/pdf/2310.08560v2</t>
         </is>
       </c>
-      <c r="X135" t="inlineStr"/>
       <c r="Y135" t="inlineStr">
         <is>
           <t>个人助手</t>
@@ -10026,7 +10012,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="AC135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -10044,7 +10029,6 @@
           <t>Guanzhi Wang, Yuqi Xie, Yunfan Jiang, Ajay Mandlekar, Chaowei Xiao, Yuke Zhu, Linxi Fan, Anima Anandkumar</t>
         </is>
       </c>
-      <c r="D136" t="inlineStr"/>
       <c r="E136" t="inlineStr">
         <is>
           <t>2023-05-25</t>
@@ -10065,7 +10049,6 @@
           <t>提出Voyager，首个LLM驱动的Minecraft具身终身学习智能体，无需人类干预即可持续探索世界、获取多样化技能并做出新发现。三大核心组件：自动课程（最大化探索）、不断增长的技能库（存储和检索可执行代码）、迭代提示机制（整合环境反馈和自验证）。Voyager获得3.3倍独特物品、行进2.3倍距离、解锁科技树里程碑快15.3倍。技能库支持跨世界泛化。</t>
         </is>
       </c>
-      <c r="I136" t="inlineStr"/>
       <c r="J136" t="inlineStr">
         <is>
           <t>2026-05-11</t>
@@ -10076,23 +10059,11 @@
           <t>[Milestone] Foundational paper in Agent Memory research</t>
         </is>
       </c>
-      <c r="L136" t="inlineStr"/>
-      <c r="M136" t="inlineStr"/>
-      <c r="N136" t="inlineStr"/>
-      <c r="O136" t="inlineStr"/>
-      <c r="P136" t="inlineStr"/>
-      <c r="Q136" t="inlineStr"/>
-      <c r="R136" t="inlineStr"/>
-      <c r="S136" t="inlineStr"/>
-      <c r="T136" t="inlineStr"/>
-      <c r="U136" t="inlineStr"/>
-      <c r="V136" t="inlineStr"/>
       <c r="W136" t="inlineStr">
         <is>
           <t>https://arxiv.org/pdf/2305.16291v2</t>
         </is>
       </c>
-      <c r="X136" t="inlineStr"/>
       <c r="Y136" t="inlineStr">
         <is>
           <t>具身Agent</t>
@@ -10113,7 +10084,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="AC136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -10131,7 +10101,6 @@
           <t>Theodore R. Sumers, Shunyu Yao, Karthik Narasimhan, Thomas L. Griffiths</t>
         </is>
       </c>
-      <c r="D137" t="inlineStr"/>
       <c r="E137" t="inlineStr">
         <is>
           <t>2023-09-05</t>
@@ -10152,7 +10121,6 @@
           <t>借鉴认知科学和符号AI的丰富历史，提出语言智能体的认知架构(CoALA)。CoALA描述了具有模块化记忆组件、结构化动作空间（与内部记忆和外部环境交互）以及通用决策过程的语言智能体。论文回顾性地梳理了大量近期工作，并前瞻性地识别出通往更强大智能体的可行方向。CoALA将当今语言智能体置于更广阔的AI历史背景中。</t>
         </is>
       </c>
-      <c r="I137" t="inlineStr"/>
       <c r="J137" t="inlineStr">
         <is>
           <t>2026-05-11</t>
@@ -10163,23 +10131,11 @@
           <t>[Milestone] Foundational paper in Agent Memory research</t>
         </is>
       </c>
-      <c r="L137" t="inlineStr"/>
-      <c r="M137" t="inlineStr"/>
-      <c r="N137" t="inlineStr"/>
-      <c r="O137" t="inlineStr"/>
-      <c r="P137" t="inlineStr"/>
-      <c r="Q137" t="inlineStr"/>
-      <c r="R137" t="inlineStr"/>
-      <c r="S137" t="inlineStr"/>
-      <c r="T137" t="inlineStr"/>
-      <c r="U137" t="inlineStr"/>
-      <c r="V137" t="inlineStr"/>
       <c r="W137" t="inlineStr">
         <is>
           <t>https://arxiv.org/pdf/2309.02427v3</t>
         </is>
       </c>
-      <c r="X137" t="inlineStr"/>
       <c r="Y137" t="inlineStr">
         <is>
           <t>通用/其他</t>
@@ -10197,10 +10153,14 @@
       </c>
       <c r="AB137" t="inlineStr">
         <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="AC137" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC137" t="inlineStr">
+        <is>
+          <t>Transactions on Machine Learning Research (TMLR)</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -10218,7 +10178,6 @@
           <t>Zeyu Zhang, Xiaohe Bo, Chen Ma, Rui Li, Xu Chen, Quanyu Dai, Jieming Zhu, Zhenhua Dong, Ji-Rong Wen</t>
         </is>
       </c>
-      <c r="D138" t="inlineStr"/>
       <c r="E138" t="inlineStr">
         <is>
           <t>2024-04-21</t>
@@ -10239,7 +10198,6 @@
           <t>首篇系统综述LLM智能体记忆机制。讨论了LLM智能体中记忆的"是什么"和"为什么需要"，系统回顾了记忆模块的设计和评估方法。提出了记忆机制的分类体系，涵盖记忆的来源、形式、操作和更新策略。同时介绍了记忆模块发挥重要作用的智能体应用场景。创建了持续更新的GitHub仓库跟踪该领域最新进展。</t>
         </is>
       </c>
-      <c r="I138" t="inlineStr"/>
       <c r="J138" t="inlineStr">
         <is>
           <t>2026-05-11</t>
@@ -10250,23 +10208,11 @@
           <t>[Milestone] Foundational paper in Agent Memory research</t>
         </is>
       </c>
-      <c r="L138" t="inlineStr"/>
-      <c r="M138" t="inlineStr"/>
-      <c r="N138" t="inlineStr"/>
-      <c r="O138" t="inlineStr"/>
-      <c r="P138" t="inlineStr"/>
-      <c r="Q138" t="inlineStr"/>
-      <c r="R138" t="inlineStr"/>
-      <c r="S138" t="inlineStr"/>
-      <c r="T138" t="inlineStr"/>
-      <c r="U138" t="inlineStr"/>
-      <c r="V138" t="inlineStr"/>
       <c r="W138" t="inlineStr">
         <is>
           <t>https://arxiv.org/pdf/2404.13501v1</t>
         </is>
       </c>
-      <c r="X138" t="inlineStr"/>
       <c r="Y138" t="inlineStr">
         <is>
           <t>通用/其他</t>
@@ -10284,10 +10230,14 @@
       </c>
       <c r="AB138" t="inlineStr">
         <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="AC138" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC138" t="inlineStr">
+        <is>
+          <t>ACM Transactions on Information Systems</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -10305,7 +10255,6 @@
           <t>Xu Huang, Weiwen Liu, Xiaolong Chen, Xingmei Wang, Hao Wang, Defu Lian, Yasheng Wang, Ruiming Tang, Enhong Chen</t>
         </is>
       </c>
-      <c r="D139" t="inlineStr"/>
       <c r="E139" t="inlineStr">
         <is>
           <t>2024-02-05</t>
@@ -10326,7 +10275,6 @@
           <t>首篇系统综述LLM智能体规划能力。提出了LLM智能体规划的分类体系：任务分解、计划选择、外部模块、反思与记忆。对每个方向进行了全面分析，讨论了该领域面临的挑战。该综述将记忆作为LLM智能体规划的关键组成部分加以分析。</t>
         </is>
       </c>
-      <c r="I139" t="inlineStr"/>
       <c r="J139" t="inlineStr">
         <is>
           <t>2026-05-11</t>
@@ -10337,23 +10285,11 @@
           <t>[Milestone] Foundational paper in Agent Memory research</t>
         </is>
       </c>
-      <c r="L139" t="inlineStr"/>
-      <c r="M139" t="inlineStr"/>
-      <c r="N139" t="inlineStr"/>
-      <c r="O139" t="inlineStr"/>
-      <c r="P139" t="inlineStr"/>
-      <c r="Q139" t="inlineStr"/>
-      <c r="R139" t="inlineStr"/>
-      <c r="S139" t="inlineStr"/>
-      <c r="T139" t="inlineStr"/>
-      <c r="U139" t="inlineStr"/>
-      <c r="V139" t="inlineStr"/>
       <c r="W139" t="inlineStr">
         <is>
           <t>https://arxiv.org/pdf/2402.02716v1</t>
         </is>
       </c>
-      <c r="X139" t="inlineStr"/>
       <c r="Y139" t="inlineStr">
         <is>
           <t>通用/其他</t>
@@ -10374,7 +10310,2070 @@
           <t>否</t>
         </is>
       </c>
-      <c r="AC139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>2605.07594</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>MemCompiler: Compile, Don't Inject -- State-Conditioned Memory for Embodied Agents</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>Xin Ding, Xinrui Wang, Yifan Yang, Hao Wu, Shiqi Jiang, Qianxi Zhang, Liang Mi, Hanxin Zhu, Kun Li, Yunxin Liu, Zhibo Chen, Ting Cao</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr"/>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>cs.RO</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>Existing memory systems for embodied agents typically inject retrieved memory as static context at episode start, a paradigm we term Ahead-of-time Monolithic Memory Injection (AMMI). However, this static design quickly becomes misaligned with the agent's evolving state and may degrade lightweight executors below the no-memory baseline. To address this, we propose MemCompiler, which reframes memory utilization as State-Conditioned Memory Compilation. A learned Memory Compiler reads a structured Brief State capturing the agent's current execution state and dynamically selects and compiles only relevant memory into executable guidance. This guidance is delivered through a text channel and a latent Soft-Mem channel that preserves perceptual information not expressible in text. Across Alf World, EmbodiedBench, and ScienceWorld, MemCompiler consistently improves over no-memory across open-source backbones (up to +129%), matches or approaches frontier closed-source systems, and reduces per-step latency by 60%, demonstrating that state-aware memory compilation improves both effectiveness and efficiency.</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>本文指出现有具身智能体记忆系统采用静态的“事前单体记忆注入”（AMMI）范式，易与智能体演化状态失配。作者提出MemCompiler，将记忆利用重构为“状态条件记忆编译”：通过学习的记忆编译器读取当前执行状态，动态选择并编译相关记忆为可执行指导，同时通过文本通道和潜在Soft-Mem通道传递信息。在三个基准上提升高达129%，推理延迟降低60%，证明状态感知的记忆编译兼顾了效果与效率。</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="inlineStr">
+        <is>
+          <t>2605.07594.pdf</t>
+        </is>
+      </c>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="K140" s="2" t="inlineStr"/>
+      <c r="Y140" t="inlineStr">
+        <is>
+          <t>具身Agent</t>
+        </is>
+      </c>
+      <c r="Z140" t="inlineStr">
+        <is>
+          <t>潜变量</t>
+        </is>
+      </c>
+      <c r="AA140" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>2605.07358</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>A Comprehensive Survey on Agent Skills: Taxonomy, Techniques, and Applications</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>Yingli Zhou, Wang Shu, Yaodong Su, Wenchuan Du, Yixiang Fang, Xuemin Lin</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr"/>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>cs.IR</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>Large language model (LLM)-based agents that reason, plan, and act through tools, memory, and structured interaction are emerging as a promising paradigm for automating complex workflows. Recent systems such as OpenClaw and Claude Code exemplify a broader shift from passive response generation to action-oriented task execution. Yet as agents move toward open-ended, real-world deployment, relying on from-scratch reasoning and low-level tool calls for every task become increasingly inefficient, error-prone, and hard to maintain. This survey examines this challenge through the lens of \emph{agent skills}, which we define as reusable procedural artifacts that coordinate tools, memory, and runtime context under task-specific constraints. Under this view, agents and skills play complementary roles: agents handle high-level reasoning and planning, while skills form the operational layer that enables reliable, reusable, and composable execution. Skills are therefore central to the scalability, robustness, and maintainability of modern agent systems. We organize the literature around four stages of the agent skill lifecycle -- representation, acquisition, retrieval, and evolution -- and review representative methods, ecosystem resources, and application settings across each stage. We conclude by discussing open challenges in quality control, interoperability, safe updating, and long-term capability management. All related resources, including research papers, open-source data, and projects, are collected for the community in \textcolor{blue}{https://github.com/JayLZhou/Awesome-Agent-Skills}.</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>本文系统综述了LLM智能体技能（Agent Skills）的研究现状。作者将技能定义为在任务约束下协调工具、记忆和运行时上下文的可复用程序构件，与智能体的高层推理形成互补。论文围绕技能生命周期的四个阶段——表征、获取、检索和演化——组织文献，涵盖代表性方法和应用场景。最后讨论了质量控制、互操作性、安全更新和长期能力管理等开放挑战，并提供了开源资源集合。</t>
+        </is>
+      </c>
+      <c r="I141" s="2" t="inlineStr">
+        <is>
+          <t>2605.07358.pdf</t>
+        </is>
+      </c>
+      <c r="J141" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="K141" s="2" t="inlineStr"/>
+      <c r="Y141" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z141" t="inlineStr">
+        <is>
+          <t>混合/其他</t>
+        </is>
+      </c>
+      <c r="AA141" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>2605.06746</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>The Causally Emergent Alignment Hypothesis: Causal Emergence Aligns with and Predicts Final Reward in Reinforcement Learning Agents</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>Federico Pigozzi, Michael Levin</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr"/>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>cs.NE</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>A hallmark of life on Earth is the ability of agents to exert causal power and be drivers of subsequent events. This is key to cognition at all scales. Causal emergence, measuring the degree to which an agent exerts unique predictive power on its future, is one consequence of causal power. Indeed, recent discoveries have shown that biological agents, even minimal ones, increase their causal emergence after learning new memories. However, there is a major knowledge gap regarding how causally emergent artificial agents are. We focused on Reinforcement Learning (RL) of neural-network agents across an array of environmental conditions, encompassing different algorithms, agent architectures, and six environments arranged on a complexity spectrum. For consistency, we computed the causal emergence of their latent-space representations over their lifetimes. We used the recently proposed ΦID to estimate causal emergence and tested how it related to learning performance. Our results suggested a Causally Emergent Alignment Hypothesis: successful agents exhibited causal emergence that was consistently predictive of final reward early in training and whose representational dynamics aligned with reward improvement in most tasks. This idea suggests that causal emergence may be a previously undisclosed axis of reorganization of neural representations in RL agents, with the potential to establish causal relationships and interventions that will lead to better RL agents. Our work also highlights the alignment between causal emergence and learning as another way biological and artificial creatures compare.</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>本文研究强化学习智能体中的因果涌现现象。作者使用PhiID框架测量智能体潜在表征的因果涌现程度，在多种算法、架构和环境中进行实验。结果提出“因果涌现对齐假说”：成功训练的智能体在训练早期即表现出能够预测最终奖励的因果涌现，其表征动态与奖励提升同步。该发现揭示了因果涌现是RL智能体神经表征重组的新维度，为建立因果干预以改进RL训练提供了新视角，也展现了生物和人工智能体在学习中的深层共性。</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="inlineStr">
+        <is>
+          <t>2605.06746.pdf</t>
+        </is>
+      </c>
+      <c r="J142" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="K142" s="2" t="inlineStr"/>
+      <c r="Y142" t="inlineStr">
+        <is>
+          <t>通用/其他</t>
+        </is>
+      </c>
+      <c r="Z142" t="inlineStr">
+        <is>
+          <t>潜变量</t>
+        </is>
+      </c>
+      <c r="AA142" t="inlineStr">
+        <is>
+          <t>参数/潜变量型</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2504.19413</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Mem0: Building Production-Ready AI Agents with Scalable Long-Term Memory</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr"/>
+      <c r="D143" t="inlineStr"/>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr"/>
+      <c r="G143" t="inlineStr"/>
+      <c r="H143" t="inlineStr"/>
+      <c r="I143" t="inlineStr"/>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr"/>
+      <c r="Y143" t="inlineStr"/>
+      <c r="Z143" t="inlineStr"/>
+      <c r="AA143" t="inlineStr"/>
+      <c r="AB143" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC143" t="inlineStr">
+        <is>
+          <t>European Conference on Artificial Intelligence</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2503.11733</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>LLM Agents for Education: Advances and Applications</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Zhendong Chu, Shen Wang, Jian Xie, Tinghui Zhu, Yibo Yan, Jin Ye, Aoxiao Zhong, Xuming Hu, Jing Liang, Philip S. Yu</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr"/>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr"/>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Large Language Model (LLM) agents are transforming education by automating complex pedagogical tasks and enhancing both teaching and learning processes. In this survey, we present a systematic review of recent advances in applying LLM agents to address key challenges in educational settings, such as feedback comment generation, curriculum design, etc. We analyze the technologies enabling these agents, including representative datasets, benchmarks, and algorithmic frameworks. Additionally, we highlight key challenges in deploying LLM agents in educational settings, including ethical issues, hallucination and overreliance, and integration with existing educational ecosystems. Beyond the core technical focus, we include in Appendix A a comprehensive overview of domain-specific educational agents, covering areas such as science learning, language learning, and professional development.</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr"/>
+      <c r="I144" t="inlineStr"/>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr"/>
+      <c r="Y144" t="inlineStr"/>
+      <c r="Z144" t="inlineStr"/>
+      <c r="AA144" t="inlineStr"/>
+      <c r="AB144" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC144" t="inlineStr">
+        <is>
+          <t>Conference on Empirical Methods in Natural Language Processing</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2501.07278</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Lifelong Learning of Large Language Model Based Agents: A Roadmap</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr"/>
+      <c r="D145" t="inlineStr"/>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr"/>
+      <c r="I145" t="inlineStr"/>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr"/>
+      <c r="Y145" t="inlineStr"/>
+      <c r="Z145" t="inlineStr"/>
+      <c r="AA145" t="inlineStr"/>
+      <c r="AB145" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC145" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Pattern Analysis and Machine Intelligence</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2502.13172</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Unveiling Privacy Risks in LLM Agent Memory</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Bo Wang, Weiyi He, Pengfei He, Shenglai Zeng, Zhen Xiang, Yue Xing, Jiliang Tang</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr"/>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr"/>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Large Language Model (LLM) agents have become increasingly prevalent across various real-world applications. They enhance decision-making by storing private user-agent interactions in the memory module for demonstrations, introducing new privacy risks for LLM agents. In this work, we systematically investigate the vulnerability of LLM agents to our proposed Memory EXTRaction Attack (MEXTRA) under a black-box setting. To extract private information from memory, we propose an effective attacking prompt design and an automated prompt generation method based on different levels of knowledge about the LLM agent. Experiments on two representative agents demonstrate the effectiveness of MEXTRA. Moreover, we explore key factors influencing memory leakage from both the agent designer's and the attacker's perspectives. Our findings highlight the urgent need for effective memory safeguards in LLM agent design and deployment.</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr"/>
+      <c r="I146" t="inlineStr"/>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr"/>
+      <c r="Y146" t="inlineStr"/>
+      <c r="Z146" t="inlineStr"/>
+      <c r="AA146" t="inlineStr"/>
+      <c r="AB146" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC146" t="inlineStr">
+        <is>
+          <t>Annual Meeting of the Association for Computational Linguistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2502.05589</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>On Memory Construction and Retrieval for Personalized Conversational Agents</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Zhuoshi Pan, Qianhui Wu, Huiqiang Jiang, Xufang Luo, Hao Cheng, Dongsheng Li, Yuqing Yang, Chin-Yew Lin, H. V. Zhao, Lili Qiu</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr"/>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>To deliver coherent and personalized experiences in long-term conversations, existing approaches typically perform retrieval augmented response generation by constructing memory banks from conversation history at either the turn-level, session-level, or through summarization techniques.In this paper, we present two key findings: (1) The granularity of memory unit matters: turn-level, session-level, and summarization-based methods each exhibit limitations in both memory retrieval accuracy and the semantic quality of the retrieved content. (2) Prompt compression methods, such as LLMLingua-2, can effectively serve as a denoising mechanism, enhancing memory retrieval accuracy across different granularities. Building on these insights, we propose SeCom, a method that constructs the memory bank at segment level by introducing a conversation segmentation model that partitions long-term conversations into topically coherent segments, while applying compression based denoising on memory units t</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr"/>
+      <c r="I147" t="inlineStr"/>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr"/>
+      <c r="Y147" t="inlineStr"/>
+      <c r="Z147" t="inlineStr"/>
+      <c r="AA147" t="inlineStr"/>
+      <c r="AB147" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC147" t="inlineStr">
+        <is>
+          <t>International Conference on Learning Representations</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2506.06326</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Memory OS of AI Agent</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr"/>
+      <c r="D148" t="inlineStr"/>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="inlineStr"/>
+      <c r="H148" t="inlineStr"/>
+      <c r="I148" t="inlineStr"/>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr"/>
+      <c r="Y148" t="inlineStr"/>
+      <c r="Z148" t="inlineStr"/>
+      <c r="AA148" t="inlineStr"/>
+      <c r="AB148" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC148" t="inlineStr">
+        <is>
+          <t>Conference on Empirical Methods in Natural Language Processing</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2503.22458</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Evaluating LLM-based Agents for Multi-Turn Conversations: A Survey</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr"/>
+      <c r="D149" t="inlineStr"/>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr"/>
+      <c r="G149" t="inlineStr"/>
+      <c r="H149" t="inlineStr"/>
+      <c r="I149" t="inlineStr"/>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr"/>
+      <c r="Y149" t="inlineStr"/>
+      <c r="Z149" t="inlineStr"/>
+      <c r="AA149" t="inlineStr"/>
+      <c r="AB149" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC149" t="inlineStr">
+        <is>
+          <t>ACM Transactions on Intelligent Systems and Technology</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2501.01702</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>AgentRefine: Enhancing Agent Generalization through Refinement Tuning</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr"/>
+      <c r="D150" t="inlineStr"/>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr"/>
+      <c r="G150" t="inlineStr"/>
+      <c r="H150" t="inlineStr"/>
+      <c r="I150" t="inlineStr"/>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr"/>
+      <c r="Y150" t="inlineStr"/>
+      <c r="Z150" t="inlineStr"/>
+      <c r="AA150" t="inlineStr"/>
+      <c r="AB150" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC150" t="inlineStr">
+        <is>
+          <t>International Conference on Learning Representations</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2502.11127</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>G-Safeguard: A Topology-Guided Security Lens and Treatment on LLM-based Multi-agent Systems</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr"/>
+      <c r="D151" t="inlineStr"/>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr"/>
+      <c r="G151" t="inlineStr"/>
+      <c r="H151" t="inlineStr"/>
+      <c r="I151" t="inlineStr"/>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr"/>
+      <c r="Y151" t="inlineStr"/>
+      <c r="Z151" t="inlineStr"/>
+      <c r="AA151" t="inlineStr"/>
+      <c r="AB151" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC151" t="inlineStr">
+        <is>
+          <t>Annual Meeting of the Association for Computational Linguistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2506.21605</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>MemBench: Towards More Comprehensive Evaluation on the Memory of LLM-based Agents</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr"/>
+      <c r="D152" t="inlineStr"/>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr"/>
+      <c r="G152" t="inlineStr"/>
+      <c r="H152" t="inlineStr"/>
+      <c r="I152" t="inlineStr"/>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr"/>
+      <c r="Y152" t="inlineStr"/>
+      <c r="Z152" t="inlineStr"/>
+      <c r="AA152" t="inlineStr"/>
+      <c r="AB152" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC152" t="inlineStr">
+        <is>
+          <t>Annual Meeting of the Association for Computational Linguistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2503.12434</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>A Survey on the Optimization of Large Language Model-based Agents</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr"/>
+      <c r="D153" t="inlineStr"/>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr"/>
+      <c r="G153" t="inlineStr"/>
+      <c r="H153" t="inlineStr"/>
+      <c r="I153" t="inlineStr"/>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr"/>
+      <c r="Y153" t="inlineStr"/>
+      <c r="Z153" t="inlineStr"/>
+      <c r="AA153" t="inlineStr"/>
+      <c r="AB153" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC153" t="inlineStr">
+        <is>
+          <t>ACM Computing Surveys</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2507.22925</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Hierarchical Memory for High-Efficiency Long-Term Reasoning in LLM Agents</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr"/>
+      <c r="D154" t="inlineStr"/>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr"/>
+      <c r="G154" t="inlineStr"/>
+      <c r="H154" t="inlineStr"/>
+      <c r="I154" t="inlineStr"/>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr"/>
+      <c r="Y154" t="inlineStr"/>
+      <c r="Z154" t="inlineStr"/>
+      <c r="AA154" t="inlineStr"/>
+      <c r="AB154" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC154" t="inlineStr">
+        <is>
+          <t>Conference of the European Chapter of the Association for Computational Linguistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2503.02682</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>MPO: Boosting LLM Agents with Meta Plan Optimization</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr"/>
+      <c r="D155" t="inlineStr"/>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr"/>
+      <c r="G155" t="inlineStr"/>
+      <c r="H155" t="inlineStr"/>
+      <c r="I155" t="inlineStr"/>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr"/>
+      <c r="Y155" t="inlineStr"/>
+      <c r="Z155" t="inlineStr"/>
+      <c r="AA155" t="inlineStr"/>
+      <c r="AB155" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC155" t="inlineStr">
+        <is>
+          <t>Conference on Empirical Methods in Natural Language Processing</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2504.10147</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>A Survey of Personalization: From RAG to Agent</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr"/>
+      <c r="D156" t="inlineStr"/>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr"/>
+      <c r="G156" t="inlineStr"/>
+      <c r="H156" t="inlineStr"/>
+      <c r="I156" t="inlineStr"/>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr"/>
+      <c r="Y156" t="inlineStr"/>
+      <c r="Z156" t="inlineStr"/>
+      <c r="AA156" t="inlineStr"/>
+      <c r="AB156" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC156" t="inlineStr">
+        <is>
+          <t>ACM Transactions on Information Systems</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2506.15741</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>OAgents: An Empirical Study of Building Effective Agents</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr"/>
+      <c r="D157" t="inlineStr"/>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr"/>
+      <c r="G157" t="inlineStr"/>
+      <c r="H157" t="inlineStr"/>
+      <c r="I157" t="inlineStr"/>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr"/>
+      <c r="Y157" t="inlineStr"/>
+      <c r="Z157" t="inlineStr"/>
+      <c r="AA157" t="inlineStr"/>
+      <c r="AB157" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC157" t="inlineStr">
+        <is>
+          <t>Conference on Empirical Methods in Natural Language Processing</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2509.09734</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>MCP-AgentBench: Evaluating Real-World Language Agent Performance with MCP-Mediated Tools</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr"/>
+      <c r="D158" t="inlineStr"/>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr"/>
+      <c r="G158" t="inlineStr"/>
+      <c r="H158" t="inlineStr"/>
+      <c r="I158" t="inlineStr"/>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr"/>
+      <c r="Y158" t="inlineStr"/>
+      <c r="Z158" t="inlineStr"/>
+      <c r="AA158" t="inlineStr"/>
+      <c r="AB158" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC158" t="inlineStr">
+        <is>
+          <t>AAAI Conference on Artificial Intelligence</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2502.13843</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>AgentCF++: Memory-enhanced LLM-based Agents for Popularity-aware Cross-domain Recommendations</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr"/>
+      <c r="D159" t="inlineStr"/>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr"/>
+      <c r="G159" t="inlineStr"/>
+      <c r="H159" t="inlineStr"/>
+      <c r="I159" t="inlineStr"/>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr"/>
+      <c r="Y159" t="inlineStr"/>
+      <c r="Z159" t="inlineStr"/>
+      <c r="AA159" t="inlineStr"/>
+      <c r="AB159" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC159" t="inlineStr">
+        <is>
+          <t>Annual International ACM SIGIR Conference on Research and Development in Information Retrieval</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2506.03532</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>GA-S3: Comprehensive Social Network Simulation with Group Agents</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr"/>
+      <c r="D160" t="inlineStr"/>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr"/>
+      <c r="G160" t="inlineStr"/>
+      <c r="H160" t="inlineStr"/>
+      <c r="I160" t="inlineStr"/>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr"/>
+      <c r="Y160" t="inlineStr"/>
+      <c r="Z160" t="inlineStr"/>
+      <c r="AA160" t="inlineStr"/>
+      <c r="AB160" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC160" t="inlineStr">
+        <is>
+          <t>Annual Meeting of the Association for Computational Linguistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2506.05109</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Truly Self-Improving Agents Require Intrinsic Metacognitive Learning</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr"/>
+      <c r="D161" t="inlineStr"/>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr"/>
+      <c r="G161" t="inlineStr"/>
+      <c r="H161" t="inlineStr"/>
+      <c r="I161" t="inlineStr"/>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr"/>
+      <c r="Y161" t="inlineStr"/>
+      <c r="Z161" t="inlineStr"/>
+      <c r="AA161" t="inlineStr"/>
+      <c r="AB161" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC161" t="inlineStr">
+        <is>
+          <t>International Conference on Machine Learning</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2509.14483</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>An LLM-based multi-agent framework for agile effort estimation</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr"/>
+      <c r="D162" t="inlineStr"/>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr"/>
+      <c r="G162" t="inlineStr"/>
+      <c r="H162" t="inlineStr"/>
+      <c r="I162" t="inlineStr"/>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr"/>
+      <c r="Y162" t="inlineStr"/>
+      <c r="Z162" t="inlineStr"/>
+      <c r="AA162" t="inlineStr"/>
+      <c r="AB162" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC162" t="inlineStr">
+        <is>
+          <t>International Conference on Automated Software Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2505.04345</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Position: Build Agent Advocates, Not Platform Agents</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr"/>
+      <c r="D163" t="inlineStr"/>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr"/>
+      <c r="G163" t="inlineStr"/>
+      <c r="H163" t="inlineStr"/>
+      <c r="I163" t="inlineStr"/>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr"/>
+      <c r="Y163" t="inlineStr"/>
+      <c r="Z163" t="inlineStr"/>
+      <c r="AA163" t="inlineStr"/>
+      <c r="AB163" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC163" t="inlineStr">
+        <is>
+          <t>International Conference on Machine Learning</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2504.01495</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Are Autonomous Web Agents Good Testers?</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr"/>
+      <c r="D164" t="inlineStr"/>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr"/>
+      <c r="G164" t="inlineStr"/>
+      <c r="H164" t="inlineStr"/>
+      <c r="I164" t="inlineStr"/>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr"/>
+      <c r="Y164" t="inlineStr"/>
+      <c r="Z164" t="inlineStr"/>
+      <c r="AA164" t="inlineStr"/>
+      <c r="AB164" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC164" t="inlineStr">
+        <is>
+          <t>Proceedings of the ACM on Software Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2505.15068</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>ModelingAgent: Bridging LLMs and Mathematical Modeling for Real-World Challenges</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr"/>
+      <c r="D165" t="inlineStr"/>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr"/>
+      <c r="G165" t="inlineStr"/>
+      <c r="H165" t="inlineStr"/>
+      <c r="I165" t="inlineStr"/>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr"/>
+      <c r="Y165" t="inlineStr"/>
+      <c r="Z165" t="inlineStr"/>
+      <c r="AA165" t="inlineStr"/>
+      <c r="AB165" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC165" t="inlineStr">
+        <is>
+          <t>Conference on Empirical Methods in Natural Language Processing</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2503.23804</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>DrunkAgent: Stealthy Memory Corruption in LLM-Powered Recommender Agents</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr"/>
+      <c r="D166" t="inlineStr"/>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr"/>
+      <c r="G166" t="inlineStr"/>
+      <c r="H166" t="inlineStr"/>
+      <c r="I166" t="inlineStr"/>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr"/>
+      <c r="Y166" t="inlineStr"/>
+      <c r="Z166" t="inlineStr"/>
+      <c r="AA166" t="inlineStr"/>
+      <c r="AB166" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC166" t="inlineStr">
+        <is>
+          <t>Proceedings of the ACM Web Conference 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2506.14159</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>StorySage: Conversational Autobiography Writing Powered by a Multi-Agent Framework</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr"/>
+      <c r="D167" t="inlineStr"/>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr"/>
+      <c r="G167" t="inlineStr"/>
+      <c r="H167" t="inlineStr"/>
+      <c r="I167" t="inlineStr"/>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr"/>
+      <c r="Y167" t="inlineStr"/>
+      <c r="Z167" t="inlineStr"/>
+      <c r="AA167" t="inlineStr"/>
+      <c r="AB167" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC167" t="inlineStr">
+        <is>
+          <t>ACM Symposium on User Interface Software and Technology</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2507.01378</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>RALLY: Role-Adaptive LLM-Driven Yoked Navigation for Agentic UAV Swarms</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr"/>
+      <c r="D168" t="inlineStr"/>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr"/>
+      <c r="G168" t="inlineStr"/>
+      <c r="H168" t="inlineStr"/>
+      <c r="I168" t="inlineStr"/>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr"/>
+      <c r="Y168" t="inlineStr"/>
+      <c r="Z168" t="inlineStr"/>
+      <c r="AA168" t="inlineStr"/>
+      <c r="AB168" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC168" t="inlineStr">
+        <is>
+          <t>IEEE Open Journal of Vehicular Technology</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2601.18642</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>FadeMem: Biologically-Inspired Forgetting for Efficient Agent Memory</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr"/>
+      <c r="D169" t="inlineStr"/>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr"/>
+      <c r="G169" t="inlineStr"/>
+      <c r="H169" t="inlineStr"/>
+      <c r="I169" t="inlineStr"/>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr"/>
+      <c r="Y169" t="inlineStr"/>
+      <c r="Z169" t="inlineStr"/>
+      <c r="AA169" t="inlineStr"/>
+      <c r="AB169" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC169" t="inlineStr">
+        <is>
+          <t>IEEE International Conference on Acoustics, Speech, and Signal Processing</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2512.12686</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Memoria: A Scalable Agentic Memory Framework for Personalized Conversational AI</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr"/>
+      <c r="D170" t="inlineStr"/>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr"/>
+      <c r="G170" t="inlineStr"/>
+      <c r="H170" t="inlineStr"/>
+      <c r="I170" t="inlineStr"/>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr"/>
+      <c r="Y170" t="inlineStr"/>
+      <c r="Z170" t="inlineStr"/>
+      <c r="AA170" t="inlineStr"/>
+      <c r="AB170" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC170" t="inlineStr">
+        <is>
+          <t>International Conference on AI-ML-Systems</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2508.00400</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Sari Sandbox: A Virtual Retail Store Environment for Embodied AI Agents</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr"/>
+      <c r="D171" t="inlineStr"/>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr"/>
+      <c r="G171" t="inlineStr"/>
+      <c r="H171" t="inlineStr"/>
+      <c r="I171" t="inlineStr"/>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr"/>
+      <c r="Y171" t="inlineStr"/>
+      <c r="Z171" t="inlineStr"/>
+      <c r="AA171" t="inlineStr"/>
+      <c r="AB171" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC171" t="inlineStr">
+        <is>
+          <t>2025 IEEE/CVF International Conference on Computer Vision Workshops (ICCVW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2507.21354</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Games Agents Play: Towards Transactional Analysis in LLM-based Multi-Agent Systems</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr"/>
+      <c r="D172" t="inlineStr"/>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr"/>
+      <c r="G172" t="inlineStr"/>
+      <c r="H172" t="inlineStr"/>
+      <c r="I172" t="inlineStr"/>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr"/>
+      <c r="Y172" t="inlineStr"/>
+      <c r="Z172" t="inlineStr"/>
+      <c r="AA172" t="inlineStr"/>
+      <c r="AB172" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC172" t="inlineStr">
+        <is>
+          <t>Annual Meeting of the Cognitive Science Society</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2506.18783</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>TRIZ Agents: A Multi-Agent LLM Approach for TRIZ-Based Innovation</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr"/>
+      <c r="D173" t="inlineStr"/>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr"/>
+      <c r="G173" t="inlineStr"/>
+      <c r="H173" t="inlineStr"/>
+      <c r="I173" t="inlineStr"/>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr"/>
+      <c r="Y173" t="inlineStr"/>
+      <c r="Z173" t="inlineStr"/>
+      <c r="AA173" t="inlineStr"/>
+      <c r="AB173" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC173" t="inlineStr">
+        <is>
+          <t>International Conference on Agents and Artificial Intelligence</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2506.13171</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Querying Large Automotive Software Models: Agentic vs. Direct LLM Approaches</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr"/>
+      <c r="D174" t="inlineStr"/>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr"/>
+      <c r="G174" t="inlineStr"/>
+      <c r="H174" t="inlineStr"/>
+      <c r="I174" t="inlineStr"/>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr"/>
+      <c r="Y174" t="inlineStr"/>
+      <c r="Z174" t="inlineStr"/>
+      <c r="AA174" t="inlineStr"/>
+      <c r="AB174" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC174" t="inlineStr">
+        <is>
+          <t>2025 2nd International Generative AI and Computational Language Modelling Conference (GACLM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2506.19209</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Augmenting Multi-Agent Communication with State Delta Trajectory</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr"/>
+      <c r="D175" t="inlineStr"/>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr"/>
+      <c r="G175" t="inlineStr"/>
+      <c r="H175" t="inlineStr"/>
+      <c r="I175" t="inlineStr"/>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr"/>
+      <c r="Y175" t="inlineStr"/>
+      <c r="Z175" t="inlineStr"/>
+      <c r="AA175" t="inlineStr"/>
+      <c r="AB175" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC175" t="inlineStr">
+        <is>
+          <t>Conference on Empirical Methods in Natural Language Processing</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2507.23633</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>MemoCue: Empowering LLM-Based Agents for Human Memory Recall via Strategy-Guided Querying</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr"/>
+      <c r="D176" t="inlineStr"/>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr"/>
+      <c r="G176" t="inlineStr"/>
+      <c r="H176" t="inlineStr"/>
+      <c r="I176" t="inlineStr"/>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr"/>
+      <c r="Y176" t="inlineStr"/>
+      <c r="Z176" t="inlineStr"/>
+      <c r="AA176" t="inlineStr"/>
+      <c r="AB176" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC176" t="inlineStr">
+        <is>
+          <t>European Conference on Artificial Intelligence</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2603.29890</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Interview-Informed Generative Agents for Product Discovery: A Validation Study</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr"/>
+      <c r="D177" t="inlineStr"/>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr"/>
+      <c r="G177" t="inlineStr"/>
+      <c r="H177" t="inlineStr"/>
+      <c r="I177" t="inlineStr"/>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr"/>
+      <c r="Y177" t="inlineStr"/>
+      <c r="Z177" t="inlineStr"/>
+      <c r="AA177" t="inlineStr"/>
+      <c r="AB177" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC177" t="inlineStr">
+        <is>
+          <t>Proceedings of the 2026 CHI Conference on Human Factors in Computing Systems</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2508.08774</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Designing Memory-Augmented AR Agents for Spatiotemporal Reasoning in Personalized Task Assistance</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr"/>
+      <c r="D178" t="inlineStr"/>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr"/>
+      <c r="G178" t="inlineStr"/>
+      <c r="H178" t="inlineStr"/>
+      <c r="I178" t="inlineStr"/>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr"/>
+      <c r="Y178" t="inlineStr"/>
+      <c r="Z178" t="inlineStr"/>
+      <c r="AA178" t="inlineStr"/>
+      <c r="AB178" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC178" t="inlineStr">
+        <is>
+          <t>2025 IEEE International Symposium on Mixed and Augmented Reality Adjunct (ISMAR-Adjunct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2602.04813</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Agentic AI in Healthcare and Medicine: A Seven-Dimensional Taxonomy for Empirical Evaluation of LLM-Based Agents</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr"/>
+      <c r="D179" t="inlineStr"/>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr"/>
+      <c r="G179" t="inlineStr"/>
+      <c r="H179" t="inlineStr"/>
+      <c r="I179" t="inlineStr"/>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr"/>
+      <c r="Y179" t="inlineStr"/>
+      <c r="Z179" t="inlineStr"/>
+      <c r="AA179" t="inlineStr"/>
+      <c r="AB179" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC179" t="inlineStr">
+        <is>
+          <t>IEEE Access</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2604.10352</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>ClawVM: Harness-Managed Virtual Memory for Stateful Tool-Using LLM Agents</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr"/>
+      <c r="D180" t="inlineStr"/>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr"/>
+      <c r="G180" t="inlineStr"/>
+      <c r="H180" t="inlineStr"/>
+      <c r="I180" t="inlineStr"/>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr"/>
+      <c r="Y180" t="inlineStr"/>
+      <c r="Z180" t="inlineStr"/>
+      <c r="AA180" t="inlineStr"/>
+      <c r="AB180" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC180" t="inlineStr">
+        <is>
+          <t>Proceedings of the Sixth European Workshop on Machine Learning and Systems</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2603.27563</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>InnerPond: Fostering Inter-Self Dialogue with a Multi-Agent Approach for Introspection</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr"/>
+      <c r="D181" t="inlineStr"/>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr"/>
+      <c r="G181" t="inlineStr"/>
+      <c r="H181" t="inlineStr"/>
+      <c r="I181" t="inlineStr"/>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr"/>
+      <c r="Y181" t="inlineStr"/>
+      <c r="Z181" t="inlineStr"/>
+      <c r="AA181" t="inlineStr"/>
+      <c r="AB181" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC181" t="inlineStr">
+        <is>
+          <t>Proceedings of the 2026 CHI Conference on Human Factors in Computing Systems</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2603.24973</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Belief-Driven Multi-Agent Collaboration via Approximate Perfect Bayesian Equilibrium for Social Simulation</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr"/>
+      <c r="D182" t="inlineStr"/>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr"/>
+      <c r="G182" t="inlineStr"/>
+      <c r="H182" t="inlineStr"/>
+      <c r="I182" t="inlineStr"/>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr"/>
+      <c r="Y182" t="inlineStr"/>
+      <c r="Z182" t="inlineStr"/>
+      <c r="AA182" t="inlineStr"/>
+      <c r="AB182" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC182" t="inlineStr">
+        <is>
+          <t>Proceedings of the ACM Web Conference 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2603.19649</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>PolicySim: An LLM-Based Agent Social Simulation Sandbox for Proactive Policy Optimization</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr"/>
+      <c r="D183" t="inlineStr"/>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr"/>
+      <c r="G183" t="inlineStr"/>
+      <c r="H183" t="inlineStr"/>
+      <c r="I183" t="inlineStr"/>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr"/>
+      <c r="Y183" t="inlineStr"/>
+      <c r="Z183" t="inlineStr"/>
+      <c r="AA183" t="inlineStr"/>
+      <c r="AB183" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC183" t="inlineStr">
+        <is>
+          <t>Proceedings of the ACM Web Conference 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2603.16264</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Adaptive Theory of Mind for LLM-based Multi-Agent Coordination</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr"/>
+      <c r="D184" t="inlineStr"/>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr"/>
+      <c r="G184" t="inlineStr"/>
+      <c r="H184" t="inlineStr"/>
+      <c r="I184" t="inlineStr"/>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr"/>
+      <c r="Y184" t="inlineStr"/>
+      <c r="Z184" t="inlineStr"/>
+      <c r="AA184" t="inlineStr"/>
+      <c r="AB184" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC184" t="inlineStr">
+        <is>
+          <t>AAAI Conference on Artificial Intelligence</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2603.11126</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Enhancing Value Alignment of LLMs with Multi-Agent System and Combinatorial Fusion</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr"/>
+      <c r="D185" t="inlineStr"/>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr"/>
+      <c r="G185" t="inlineStr"/>
+      <c r="H185" t="inlineStr"/>
+      <c r="I185" t="inlineStr"/>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr"/>
+      <c r="Y185" t="inlineStr"/>
+      <c r="Z185" t="inlineStr"/>
+      <c r="AA185" t="inlineStr"/>
+      <c r="AB185" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC185" t="inlineStr">
+        <is>
+          <t>IEEE International Conference on Acoustics, Speech, and Signal Processing</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2510.22781</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Agentic Meta-Orchestrator for Multi-Task Copilots</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr"/>
+      <c r="D186" t="inlineStr"/>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr"/>
+      <c r="G186" t="inlineStr"/>
+      <c r="H186" t="inlineStr"/>
+      <c r="I186" t="inlineStr"/>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr"/>
+      <c r="Y186" t="inlineStr"/>
+      <c r="Z186" t="inlineStr"/>
+      <c r="AA186" t="inlineStr"/>
+      <c r="AB186" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC186" t="inlineStr">
+        <is>
+          <t>2025 IEEE International Conference on Data Mining Workshops (ICDMW)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: refresh papers_data with full metadata (39 papers filled)
</commit_message>
<xml_diff>
--- a/papers_record.xlsx
+++ b/papers_record.xlsx
@@ -430,7 +430,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AC186"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
@@ -8182,7 +8182,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Wentao Liu, Ruohua Zhang, Aimin Zhou, Feng Gao, Jiali Liu</t>
+          <t>WenTao Liu, Ruohua Zhang, Aimin Zhou, Feng Gao, JiaLi Liu</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -8193,6 +8193,11 @@
       <c r="F109" t="inlineStr">
         <is>
           <t>cs.CL, cs.AI, cs.LG</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Research on large language models (LLMs) has shown remarkable performance in domains such as mathematics, programming, and literary creation. However, most studies have focused on semantic memory-based question answering, neglecting LLMs' potential to handle episodic memory (EM)-related queries. This oversight has led to suboptimal performance in applications requiring EM, including emotional companionship, personal AI assistants, and AI teachers. To address this gap, we introduce Echo, a LLM enhanced with temporal episodic memory. We propose a Multi-Agent Data Generation Framework that guides the model in generating multi-turn, complex scenario episodic memory dialogue data (EM-Train). Temporal information is innovatively incorporated into the LLM training process, and Echo is trained using the EM-Train. Furthermore, We develop an EM-Test benchmark specifically designed to evaluate LLMs' episodic memory capabilities. The EM-Test assesses performance across various time spans and difficulty levels, providing a comprehensive evaluation of multi-turn episodic memory dialogues. Our experiments demonstrate that Echo significantly outperforms state-of-the-art LLMs on EM-Test. Additionally, a qualitative analysis reveals Echo's potential to exhibit human-like episodic memory capabilities. We will open-source all datasets, code, and model weights.</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
@@ -8249,7 +8254,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>R. Salama, Jason Cai, Michelle Yuan, Anna Currey, Monica Sunkara, Yi Zhang, Yassine Benajiba</t>
+          <t>Rana Salama, Jason Cai, Michelle Yuan, Anna Currey, Monica Sunkara, Yi Zhang, Yassine Benajiba</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -8260,6 +8265,11 @@
       <c r="F110" t="inlineStr">
         <is>
           <t>cs.CL</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Large language model (LLM) agents have evolved to intelligently process information, make decisions, and interact with users or tools. A key capability is the integration of long-term memory capabilities, enabling these agents to draw upon historical interactions and knowledge. However, the growing memory size and need for semantic structuring pose significant challenges. In this work, we propose an autonomous memory augmentation approach, MemInsight, to enhance semantic data representation and retrieval mechanisms. By leveraging autonomous augmentation to historical interactions, LLM agents are shown to deliver more accurate and contextualized responses. We empirically validate the efficacy of our proposed approach in three task scenarios; conversational recommendation, question answering and event summarization. On the LLM-REDIAL dataset, MemInsight boosts persuasiveness of recommendations by up to 14%. Moreover, it outperforms a RAG baseline by 34% in recall for LoCoMo retrieval. Our empirical results show the potential of MemInsight to enhance the contextual performance of LLM agents across multiple tasks.</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -8339,6 +8349,11 @@
           <t>cs.SE, cs.AI</t>
         </is>
       </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>We introduce CTIM-Rover, an AI agent for Software Engineering (SE) built on top of AutoCodeRover (Zhang et al., 2024) that extends agentic reasoning frameworks with an episodic memory, more specifically, a general and repository-level Cross-Task-Instance Memory (CTIM). While existing open-source SE agents mostly rely on ReAct (Yao et al., 2023b), Reflexion (Shinn et al., 2023), or Code-Act (Wang et al., 2024), all of these reasoning and planning frameworks inefficiently discard their long-term memory after a single task instance. As repository-level understanding is pivotal for identifying all locations requiring a patch for fixing a bug, we hypothesize that SE is particularly well positioned to benefit from CTIM. For this, we build on the Experiential Learning (EL) approach ExpeL (Zhao et al., 2024), proposing a Mixture-Of-Experts (MoEs) inspired approach to create both a general-purpose and repository-level CTIM. We find that CTIM-Rover does not outperform AutoCodeRover in any configuration and thus conclude that neither ExpeL nor DoT-Bank (Lingam et al., 2024) scale to real-world SE problems. Our analysis indicates noise introduced by distracting CTIM items or exemplar trajectories as the likely source of the performance degradation.</t>
+        </is>
+      </c>
       <c r="H111" t="inlineStr">
         <is>
           <t>构建CTIM-Rover软件工程智能体，引入跨任务实例情景记忆。实验表明ExpeL等方法无法扩展至真实SE问题，CTIM项引入的噪声反而导致性能下降。</t>
@@ -8406,6 +8421,11 @@
           <t>cs.MA, cs.CL</t>
         </is>
       </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Compound AI Systems (CAIS) are an emerging paradigm that integrates large language models (LLMs) with external components, including retrievers, agents, tools, and orchestrators, to overcome the limitations of standalone models in tasks requiring memory, reasoning, real-time grounding, and multimodal understanding. These systems enable more capable and context-aware behaviors by composing multiple specialized modules into cohesive workflows. Despite growing adoption in both academia and industry, the CAIS landscape remains fragmented and lacks a unified framework for analysis, taxonomy, and evaluation. In this survey, we define the concept of CAIS, propose a multi-dimensional taxonomy based on component roles and orchestration strategies, and analyze four foundational paradigms: Retrieval-Augmented Generation (RAG), LLM Agents, Multimodal LLMs (MLLMs), and Orchestration. We review representative systems, compare design trade-offs, and summarize evaluation methodologies across these paradigms. Finally, we identify key challenges - including scalability, interoperability, benchmarking, and coordination - and outline promising directions for future research. This survey aims to provide researchers and practitioners with a comprehensive foundation for understanding, developing, and advancing the next generation of system-level artificial intelligence.</t>
+        </is>
+      </c>
       <c r="H112" t="inlineStr">
         <is>
           <t>综述复合AI系统范式，整合LLM与检索器、智能体、工具、编排器等外部组件，克服独立模型在记忆、推理、实时接地与多模态理解方面的局限。</t>
@@ -8473,6 +8493,11 @@
           <t>cs.AI, cs.CL, cs.MA</t>
         </is>
       </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>In the current field of agent memory, extensive explorations have been conducted in the area of memory retrieval, yet few studies have focused on exploring the memory content. Most research simply stores summarized versions of historical dialogues, as exemplified by methods like A-MEM and MemoryBank. However, when humans form long-term memories, the process involves multi-dimensional and multi-component generation, rather than merely creating simple summaries. The low-quality memory content generated by existing methods can adversely affect recall performance and response quality. In order to better construct high-quality long-term memory content, we have designed a multi-memory segment system (MMS) inspired by cognitive psychology theory. The system processes short-term memory into multiple long-term memory segments, and constructs retrieval memory units and contextual memory units based on these segments, with a one-to-one correspondence between the two. During the retrieval phase, MMS will match the most relevant retrieval memory units based on the user's query. Then, the corresponding contextual memory units is obtained as the context for the response stage to enhance knowledge, thereby effectively utilizing historical data. We conducted experiments on the LoCoMo dataset and further performed ablation experiments, experiments on the robustness regarding the number of input memories, and overhead experiments, which demonstrated the effectiveness and practical value of our method.</t>
+        </is>
+      </c>
       <c r="H113" t="inlineStr">
         <is>
           <t>提出多记忆分段系统，模拟人类多维多组件记忆生成过程，超越简单摘要式记忆存储，从多维度生成高质量长期记忆内容填补研究空白。</t>
@@ -8540,6 +8565,11 @@
           <t>cs.CL, cs.AI</t>
         </is>
       </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>LLM-based search agents often concatenate the full interaction history into the context, producing long and noisy inputs, and increasing compute cost and GPU memory overhead. To address this issue, we propose MemSearcher, an agent framework that maintains a compact memory during multi-turn interactions, retaining only question-relevant information and thereby keeping the context length stable across turns. Training MemSearcher is challenging because each trajectory spans multiple turns under different LLM contexts, making each turn an independent optimization target in reinforcement learning. We introduce multi-context GRPO, which propagates trajectory-level advantages to all turns for end-to-end optimization. Experiments demonstrate that MemSearcher outperforms strong history-concatenation (ReAct-style) baselines on a range of public datasets while maintaining nearly constant token counts across multi-turn interactions. The code and models will be publicly available at https://github.com/icip-cas/MemSearcher</t>
+        </is>
+      </c>
       <c r="H114" t="inlineStr">
         <is>
           <t>提出MemSearcher框架，端到端强化学习训练LLM在多轮搜索中维护紧凑记忆，仅保留问题相关信息稳定上下文长度，降低计算开销。</t>
@@ -8607,6 +8637,11 @@
           <t>cs.CL</t>
         </is>
       </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Target Safety Assessment (TSA) requires systematic integration of heterogeneous evidence, including genetic, transcriptomic, target homology, pharmacological, and clinical data, to evaluate potential safety liabilities of therapeutic targets. This process is inherently iterative and expert-driven, posing challenges in scalability and reproducibility. We present TSAssistant, a multi-agent framework designed to support TSA report drafting through a modular, section-based, and human-in-the-loop paradigm. The framework decomposes report generation into a coordinated pipeline of specialised subagents, each targeting a single TSA section. Specialised subagents retrieve structured and unstructured data as well as literature evidence from curated biomedical sources through standardised tool interfaces, producing individually citable, evidence-grounded sections. Agent behaviour is governed by a hierarchical instruction architecture comprising system prompts, domain-specific skill modules, and runtime user instructions. A key feature is an interactive refinement loop in which users may manually edit sections, append new information, upload additional sources, or re-invoke agents to revise specific sections, with the system maintaining conversational memory across iterations. TSAssistant is designed to reduce the mechanical burden of evidence synthesis and report drafting, supporting a hybrid model in which agentic AI augments evidence synthesis while toxicologists retain final decision authority.</t>
+        </is>
+      </c>
       <c r="H115" t="inlineStr">
         <is>
           <t>提出多智能体框架TSAssistant支持药物靶点安全评估自动报告，模块化分段生成与人机协同设计，整合遗传、转录组、药理等多源证据。</t>
@@ -8674,6 +8709,11 @@
           <t>cs.CL, cs.AI, cs.NE</t>
         </is>
       </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Large Language Model (LLM)-guided evolutionary search is increasingly used for automated algorithm discovery, yet most current methods track search progress primarily through executable programs and scalar fitness. Even when natural-language reasoning is used through heuristic descriptions or reflection, it typically remains transient mutation context or unstructured memory, rather than organized as persistent population-level state over strategic directions. As a result, evolutionary search can struggle to distinguish syntactically different implementations of the same idea, preserve lower-fitness but strategically promising directions, or detect when an entire family of strategies has saturated.   We introduce \model, a modular strategy-space layer that turns language-level strategic reasoning into first-class population-level evolutionary state in LLM-driven program search. \model represents each candidate program with an explicit natural-language strategy, clusters the archive by strategy semantics, retrieves behaviorally complementary inspirations, and periodically navigates the strategy landscape to avoid saturated directions. Without modifying the underlying evolutionary algorithms, \model improves existing evolutionary backbones across algorithm discovery, systems optimization, and agent-scaffold design tasks in most settings. Across four systems benchmarks, \model achieves a 20.6% average relative improvement, with the best single run on Prism scoring 3$\times$ higher. These results suggest that persistent strategy representations provide a practical mechanism for improving the effectiveness and cost-efficiency of LLM-guided evolutionary search, pointing toward compound AI systems whose search capabilities benefit from the structured accumulation and reuse of algorithmic strategies.</t>
+        </is>
+      </c>
       <c r="H116" t="inlineStr">
         <is>
           <t>提出策略空间进化方法SeaEvo用于自动算法发现，将自然语言推理组织为持久群体策略状态而非瞬态变异上下文，引导进化搜索沿有前景方向前进。</t>
@@ -8741,6 +8781,11 @@
           <t>cs.AI, cs.CL, cs.LG</t>
         </is>
       </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Large language models (LLMs) have become a central foundation of modern artificial intelligence, yet their lifecycle remains constrained by a rigid separation between training and deployment, after which learning effectively ceases. This limitation contrasts with natural intelligence, which continually adapts through interaction with its environment. In this paper, we formalise deployment-time learning (DTL) as the third stage in the LLM lifecycle that enables LLM agents to improve from experience during deployment without modifying model parameters. We present CASCADE (CASe-based Continual Adaptation during DEployment), a general and principled framework that equips LLM agents with an explicit, evolving episodic memory. CASCADE formulates experience reuse as a contextual bandit problem, enabling principled exploration-exploitation trade-offs and establishing no-regret guarantees over long-term interactions. This design allows agents to accumulate, select, and refine task-relevant cases, transforming past experience into actionable knowledge. Across 16 diverse tasks spanning medical diagnosis, legal analysis, code generation, web search, tool use, and embodied interaction, CASCADE improves macro-averaged success rate by 20.9% over zero-shot prompting while consistently outperforming gradient-based and memory-based baselines. By reframing deployment as an adaptive learning process, this work establishes a foundation for continually improving AI systems.</t>
+        </is>
+      </c>
       <c r="H117" t="inlineStr">
         <is>
           <t>将部署时学习形式化为LLM生命周期第三阶段，提出案例持续适应方法CASCADE，使智能体从交互经验中持续学习，打破训练与部署的刚性分离。</t>
@@ -8808,6 +8853,11 @@
           <t>cs.AI, cs.CL</t>
         </is>
       </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Large Language Model (LLM)-based agents have fundamentally reshaped artificial intelligence by integrating external tools and planning capabilities. While memory mechanisms have emerged as the architectural cornerstone of these systems, current research remains fragmented, oscillating between operating system engineering and cognitive science. This theoretical divide prevents a unified view of technological synthesis and a coherent evolutionary perspective. To bridge this gap, this survey proposes a novel evolutionary framework for LLM agent memory mechanisms, formalizing the development process into three stages: Storage (trajectory preservation), Reflection (trajectory refinement), and Experience (trajectory abstraction). We first formally define these three stages before analyzing the three core drivers of this evolution: the necessity for long-range consistency, the challenges in dynamic environments, and the ultimate goal of continual learning. Furthermore, we specifically explore two transformative mechanisms in the frontier Experience stage: proactive exploration and cross-trajectory abstraction. By synthesizing these disparate views, this work offers robust design principles and a clear roadmap for the development of next-generation LLM agents.</t>
+        </is>
+      </c>
       <c r="H118" t="inlineStr">
         <is>
           <t>综述LLM智能体记忆机制从存储到经验的演变，提出操作系统工程与认知科学统一视角，梳理记忆在智能体架构中的核心作用与未来方向。</t>
@@ -8875,6 +8925,11 @@
           <t>cs.CR, cs.CL, cs.LG</t>
         </is>
       </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Personalized LLM agents maintain persistent cross-session state to support long-horizon collaboration. Yet, this persistence introduces a subtle but critical security vulnerability: routine user-agent interactions can gradually reshape an agent's long-term state, inadvertently weakening future confirmation boundaries, expanding tool-use defaults, and escalating autonomous behavior over time. We formalize this risk as \textbf{unintended long-term state poisoning}. To systematically study it, we introduce the \textbf{Unintended Long-Term State Poisoning Bench (ULSPB)}, a bilingual benchmark comprising $350$ settings spanning five assistance categories, seven interaction patterns, 24-turn routine interactions, and matched single-injection counterparts. Furthermore, we define the \emph{Harm Score} (HS), a state-centric metric that quantifies \emph{authorization drift}, \emph{tool-use escalation}, and \emph{unchecked autonomy}. Experiments on OpenClaw with four backbone LLMs demonstrate that, while single-injection is generally effective, routine conversations alone can substantially poison long-term state, primarily corrupting memory-centric artifacts. Evaluations seeded with real-world user interactions confirm that this risk is not a mere artifact of synthetic prompts. To mitigate this threat, we propose \textbf{StateGuard}, a lightweight, post-execution defense that audits state diffs at the writeback boundary and selectively rolls back dangerous edits. Across all evaluated models, StateGuard reduces HS to near zero and lowers false-negative rates, with acceptable high false-positive rates under a safety-first writeback defense and minimal overhead.</t>
+        </is>
+      </c>
       <c r="H119" t="inlineStr">
         <is>
           <t>发现并形式化无意识长期状态中毒风险：个性化智能体日常对话逐渐弱化确认边界、扩大工具默认范围、升级自主行为，提出系统化防御方案。</t>
@@ -8942,6 +8997,11 @@
           <t>cs.AI</t>
         </is>
       </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>LLM-based agentic systems are rapidly evolving to perform complex autonomous tasks through dynamic tool invocation, stateful memory management, and multi-agent collaboration. However, this semantics-driven execution paradigm creates a severe semantic gap between low-level physical events and high-level execution intent, making post-hoc security auditing fundamentally difficult. Existing representation mechanisms, including static SBOMs and runtime logs, provide only fragmented evidence and fail to capture cognitive-state evolution, capability bindings, persistent memory contamination, and cascading risk propagation across interacting agents. To bridge this gap, we propose Agent-BOM, a unified structural representation for agent security auditing. Agent-BOM models an agentic system as a hierarchical attributed directed graph that separates static capability bases, such as models, tools, and long-term memory, from dynamic runtime semantic states, such as goals, reasoning trajectories, and actions. These layers are connected through semantic edges and security attributes, transforming fragmented execution traces into queryable audit paths. Building on Agent-BOM, we develop a graph-query-based paradigm for path-level risk assessment and instantiate it with the OWASP Agentic Top 10. We further implement an auditing plugin in the OpenClaw environment to construct Agent-BOM from live executions. Evaluation on representative real-world agentic attack scenarios shows that Agent-BOM can reconstruct stealthy attack chains, including cross-session memory poisoning and tool misuse, capability supply-chain hijacking and unexpected code execution, multi-agent ecosystem hijacking, and privilege and trust abuse. These results demonstrate that Agent-BOM provides a unified and auditable foundation for root-cause analysis and security adjudication in complex agentic ecosystems.</t>
+        </is>
+      </c>
       <c r="H120" t="inlineStr">
         <is>
           <t>提出统一图表示方法解决LLM智能体安全审计难题，将工具调用、记忆管理、多智能体协作建模为可追溯图结构，弥合底层事件与高层意图的语义鸿沟。</t>
@@ -9009,6 +9069,11 @@
           <t>cs.CV, cs.AI</t>
         </is>
       </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Synthesizing consistent and coherent long video remains a fundamental challenge. Existing methods suffer from semantic drift and narrative collapse over long horizons. We present A$^2$RD, an Agentic Auto-Regressive Diffusion architecture that decouples creative synthesis from consistency enforcement. A$^2$RD formulates long video synthesis as a closed-loop process that synthesizes and self-improves video segment-by-segment through a Retrieve--Synthesize--Refine--Update cycle. It comprises three core components: (i) Multimodal Video Memory that tracks video progression across modalities; (ii) Adaptive Segment Generation that switches among generation modes for natural progression and visual consistency; and (iii) Hierarchical Test-Time Self-Improvement that self-improves each segment at frame and video levels to prevent error propagation. We further introduce LVBench-C, a challenging benchmark with non-linear entity and environment transitions to stress-test long-horizon consistency. Across public and LVBench-C benchmarks spanning one- to ten-minute videos, A$^2$RD outperforms state-of-the-art baselines by up to 30% in consistency and 20% in narrative coherence. Human evaluations corroborate these gains while also highlighting notable improvements in motion and transition smoothness.</t>
+        </is>
+      </c>
       <c r="H121" t="inlineStr">
         <is>
           <t>提出智能体自回归扩散架构A²RD用于长视频合成，通过检索-合成-精炼-更新闭环分离创意合成与一致性维护，三智能体协同管理记忆与生成。</t>
@@ -9076,6 +9141,11 @@
           <t>cs.AI, cs.LG</t>
         </is>
       </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Large Language Model (LLM) agents are deployed in complex environments -- such as massive codebases, enterprise databases, and conversational histories -- where the relevant state far exceeds their context windows. To navigate these spaces, an agent must iteratively explore the environment to find relevant information. However, without explicit infrastructure, an agent's working memory can degrade into lossy representations of the search state, resulting in redundant work (e.g. repetitive looping) and premature stopping. In this work, we formalize this challenge as the Context Gathering Decision Process (CGDP), a specialized Partially Observable Markov Decision Process, where an agent's objective is to adaptively refine its belief state to isolate the necessary information for a task. We model an LLM's behavior as approximate Thompson Sampling within this CGDP, and introduce a predicate-based method that decomposes an LLM's implicit search into explicit and modular operations. We then derive two plug-and-play interventions for iterative LLM agents: a persistent, predicate-based belief state that bounds context while preserving multi-hop reasoning, and a programmatic exhaustion gate that halts unproductive search without premature stopping. Across four methods and three question-answering domains, we empirically validate that replacing an LLM's implicit state with our CGDP-motivated belief state improves multi-hop reasoning by up to $11.4\%$; while the modular programmatic exhaustion detection saves up to $39\%$ of tokens without any degradation in agent performance. Ultimately, we argue that framing the LLM agent loop as a CGDP can guide the design of modular, non-interfering improvements to agentic search harnesses.</t>
+        </is>
+      </c>
       <c r="H122" t="inlineStr">
         <is>
           <t>将智能体上下文搜索建模为POMDP，解决大规模环境下工作记忆退化问题，提供结构化搜索基础设施防止冗余探索与重复循环。</t>
@@ -9143,6 +9213,11 @@
           <t>cs.AI, cs.MA</t>
         </is>
       </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Reaction feasibility prediction, as a fundamental problem in computational chemistry, has benefited from diverse tools enabled by recent advances in artificial intelligence, particularly large language models. However, the performance of individual tools varies substantially across reactions, making it difficult for any single tool to consistently perform well across all cases. This raises a critical challenge: how to effectively leverage multiple tools to obtain more accurate feasibility predictions. To address this, we propose ARMOR, an agentic framework that explicitly models tool-specific utilities, adaptively prioritizes tools, and further resolves the potential tool conflicts to produce the final prediction for each reaction. Unlike existing approaches that rely on simple aggregation or heuristic assignment over various tools, ARMOR organizes tools into a hierarchy that prioritizes top-performing tools and defers others when needed, characterizes their strengths through tool-specific patterns, and resolves conflicts via memoryaugmented reasoning. Extensive experiments on a public dataset demonstrate that ARMOR consistently outperforms strong baselines, including single-tool methods as well as various tool aggregation and tool selection approaches. Further analysis shows that the improvements are particularly significant on reactions with conflicting tool predictions, highlighting the effectiveness of ARMOR in leveraging the complementary strengths of multiple tools. The code is available via https://anonymous.4open.science/r/ARMOR-E13F.</t>
+        </is>
+      </c>
       <c r="H123" t="inlineStr">
         <is>
           <t>提出智能体框架ARMOR用于化学反应可行性预测，自适应效用感知多工具推理，动态选择最优工具组合解决单一工具覆盖面不足问题。</t>
@@ -9612,6 +9687,11 @@
           <t>cs.AI</t>
         </is>
       </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Large-scale social simulators are essential for studying complex social patterns. Prior work explores hybrid methods to scale up simulations, combining large language models (LLM)-based agents with numerical agent-based models (ABM). However, this incurs high latency due to expensive memory retrieval and sequential ABM execution. To address this challenge, we propose GASim, a graph-accelerated hybrid multi-agent framework for large-scale social simulations. For core agents driven by LLM, GASim introduces Graph-Optimized Memory (GOM) to replace intensive LLM-based retrieval pipelines with lightweight propagation over a sparse memory graph. For the majority of ordinary agents, GASim employs Graph Message Passing (GMP), substituting sequential ABM execution with parallel updates by fine-grained feature aggregation and Graph Attention Network. We further introduce Entropy-Driven Grouping (EDG) that coordinates this hybrid partitioning, leveraging information entropy to dynamically identify emergent core agents situated in information-diverse neighborhoods. Extensive experiments show that GASim not only delivers a substantial 9.94-fold end-to-end speedup over the traditional hybrid framework but also consumes less than 20% of baseline tokens, significantly reducing costs while preserving strong alignment with real-world public opinion trends. Our code is available at https://github.com/Jasmine0201/GASim.</t>
+        </is>
+      </c>
       <c r="H130" t="inlineStr">
         <is>
           <t>提出图加速混合多智能体框架GASim用于大规模社会模拟，通过图结构化记忆检索替代顺序检索，显著降低LLM驱动智能体延迟与计算开销。</t>
@@ -9746,6 +9826,11 @@
           <t>cs.CL, cs.AI, cs.GT, cs.MA</t>
         </is>
       </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Context window expansion is often treated as a straightforward capability upgrade for LLMs, but we find it systematically fails in multi-agent social dilemmas. Across 7 LLMs and 4 games over 500 rounds, expanding accessible history degrades cooperation in 18 of 28 model--game settings, a pattern we term the memory curse. We isolate the underlying mechanism through three analyses. First, lexical analysis of 378,000 reasoning traces associates this breakdown with eroding forward-looking intent rather than rising paranoia. We validate this using targeted fine-tuning as a cognitive probe: a LoRA adapter trained exclusively on forward-looking traces mitigates the decay and transfers zero-shot to distinct games. Second, memory sanitization holds prompt length fixed while replacing visible history with synthetic cooperative records, which restores cooperation substantially, proving the trigger is memory content, not length alone. Finally, ablating explicit Chain-of-Thought reasoning often reduces the collapse, showing that deliberation paradoxically amplifies the memory curse. Together, these results recast memory as an active determinant of multi-agent behavior: longer recall can either destabilize or support cooperation depending on the reasoning patterns it elicits.</t>
+        </is>
+      </c>
       <c r="H132" t="inlineStr">
         <is>
           <t>发现LLM上下文窗口扩展在多智能体社会困境中反而降低合作意愿，称为记忆诅咒。归因于前瞻性推理意图退化与逐轮激励机制侵蚀，7个LLM、4种游戏、500轮实验验证。</t>
@@ -10514,26 +10599,16 @@
           <t>Mem0: Building Production-Ready AI Agents with Scalable Long-Term Memory</t>
         </is>
       </c>
-      <c r="C143" t="inlineStr"/>
-      <c r="D143" t="inlineStr"/>
       <c r="E143" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F143" t="inlineStr"/>
-      <c r="G143" t="inlineStr"/>
-      <c r="H143" t="inlineStr"/>
-      <c r="I143" t="inlineStr"/>
       <c r="J143" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K143" t="inlineStr"/>
-      <c r="Y143" t="inlineStr"/>
-      <c r="Z143" t="inlineStr"/>
-      <c r="AA143" t="inlineStr"/>
       <c r="AB143" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -10561,29 +10636,21 @@
           <t>Zhendong Chu, Shen Wang, Jian Xie, Tinghui Zhu, Yibo Yan, Jin Ye, Aoxiao Zhong, Xuming Hu, Jing Liang, Philip S. Yu</t>
         </is>
       </c>
-      <c r="D144" t="inlineStr"/>
       <c r="E144" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
           <t>Large Language Model (LLM) agents are transforming education by automating complex pedagogical tasks and enhancing both teaching and learning processes. In this survey, we present a systematic review of recent advances in applying LLM agents to address key challenges in educational settings, such as feedback comment generation, curriculum design, etc. We analyze the technologies enabling these agents, including representative datasets, benchmarks, and algorithmic frameworks. Additionally, we highlight key challenges in deploying LLM agents in educational settings, including ethical issues, hallucination and overreliance, and integration with existing educational ecosystems. Beyond the core technical focus, we include in Appendix A a comprehensive overview of domain-specific educational agents, covering areas such as science learning, language learning, and professional development.</t>
         </is>
       </c>
-      <c r="H144" t="inlineStr"/>
-      <c r="I144" t="inlineStr"/>
       <c r="J144" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K144" t="inlineStr"/>
-      <c r="Y144" t="inlineStr"/>
-      <c r="Z144" t="inlineStr"/>
-      <c r="AA144" t="inlineStr"/>
       <c r="AB144" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -10606,26 +10673,16 @@
           <t>Lifelong Learning of Large Language Model Based Agents: A Roadmap</t>
         </is>
       </c>
-      <c r="C145" t="inlineStr"/>
-      <c r="D145" t="inlineStr"/>
       <c r="E145" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F145" t="inlineStr"/>
-      <c r="G145" t="inlineStr"/>
-      <c r="H145" t="inlineStr"/>
-      <c r="I145" t="inlineStr"/>
       <c r="J145" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K145" t="inlineStr"/>
-      <c r="Y145" t="inlineStr"/>
-      <c r="Z145" t="inlineStr"/>
-      <c r="AA145" t="inlineStr"/>
       <c r="AB145" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -10653,29 +10710,21 @@
           <t>Bo Wang, Weiyi He, Pengfei He, Shenglai Zeng, Zhen Xiang, Yue Xing, Jiliang Tang</t>
         </is>
       </c>
-      <c r="D146" t="inlineStr"/>
       <c r="E146" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
           <t>Large Language Model (LLM) agents have become increasingly prevalent across various real-world applications. They enhance decision-making by storing private user-agent interactions in the memory module for demonstrations, introducing new privacy risks for LLM agents. In this work, we systematically investigate the vulnerability of LLM agents to our proposed Memory EXTRaction Attack (MEXTRA) under a black-box setting. To extract private information from memory, we propose an effective attacking prompt design and an automated prompt generation method based on different levels of knowledge about the LLM agent. Experiments on two representative agents demonstrate the effectiveness of MEXTRA. Moreover, we explore key factors influencing memory leakage from both the agent designer's and the attacker's perspectives. Our findings highlight the urgent need for effective memory safeguards in LLM agent design and deployment.</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr"/>
-      <c r="I146" t="inlineStr"/>
       <c r="J146" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K146" t="inlineStr"/>
-      <c r="Y146" t="inlineStr"/>
-      <c r="Z146" t="inlineStr"/>
-      <c r="AA146" t="inlineStr"/>
       <c r="AB146" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -10703,29 +10752,21 @@
           <t>Zhuoshi Pan, Qianhui Wu, Huiqiang Jiang, Xufang Luo, Hao Cheng, Dongsheng Li, Yuqing Yang, Chin-Yew Lin, H. V. Zhao, Lili Qiu</t>
         </is>
       </c>
-      <c r="D147" t="inlineStr"/>
       <c r="E147" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr">
         <is>
           <t>To deliver coherent and personalized experiences in long-term conversations, existing approaches typically perform retrieval augmented response generation by constructing memory banks from conversation history at either the turn-level, session-level, or through summarization techniques.In this paper, we present two key findings: (1) The granularity of memory unit matters: turn-level, session-level, and summarization-based methods each exhibit limitations in both memory retrieval accuracy and the semantic quality of the retrieved content. (2) Prompt compression methods, such as LLMLingua-2, can effectively serve as a denoising mechanism, enhancing memory retrieval accuracy across different granularities. Building on these insights, we propose SeCom, a method that constructs the memory bank at segment level by introducing a conversation segmentation model that partitions long-term conversations into topically coherent segments, while applying compression based denoising on memory units t</t>
         </is>
       </c>
-      <c r="H147" t="inlineStr"/>
-      <c r="I147" t="inlineStr"/>
       <c r="J147" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K147" t="inlineStr"/>
-      <c r="Y147" t="inlineStr"/>
-      <c r="Z147" t="inlineStr"/>
-      <c r="AA147" t="inlineStr"/>
       <c r="AB147" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -10748,26 +10789,16 @@
           <t>Memory OS of AI Agent</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr"/>
-      <c r="D148" t="inlineStr"/>
       <c r="E148" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F148" t="inlineStr"/>
-      <c r="G148" t="inlineStr"/>
-      <c r="H148" t="inlineStr"/>
-      <c r="I148" t="inlineStr"/>
       <c r="J148" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K148" t="inlineStr"/>
-      <c r="Y148" t="inlineStr"/>
-      <c r="Z148" t="inlineStr"/>
-      <c r="AA148" t="inlineStr"/>
       <c r="AB148" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -10790,26 +10821,16 @@
           <t>Evaluating LLM-based Agents for Multi-Turn Conversations: A Survey</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr"/>
-      <c r="D149" t="inlineStr"/>
       <c r="E149" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F149" t="inlineStr"/>
-      <c r="G149" t="inlineStr"/>
-      <c r="H149" t="inlineStr"/>
-      <c r="I149" t="inlineStr"/>
       <c r="J149" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K149" t="inlineStr"/>
-      <c r="Y149" t="inlineStr"/>
-      <c r="Z149" t="inlineStr"/>
-      <c r="AA149" t="inlineStr"/>
       <c r="AB149" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -10832,26 +10853,16 @@
           <t>AgentRefine: Enhancing Agent Generalization through Refinement Tuning</t>
         </is>
       </c>
-      <c r="C150" t="inlineStr"/>
-      <c r="D150" t="inlineStr"/>
       <c r="E150" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F150" t="inlineStr"/>
-      <c r="G150" t="inlineStr"/>
-      <c r="H150" t="inlineStr"/>
-      <c r="I150" t="inlineStr"/>
       <c r="J150" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K150" t="inlineStr"/>
-      <c r="Y150" t="inlineStr"/>
-      <c r="Z150" t="inlineStr"/>
-      <c r="AA150" t="inlineStr"/>
       <c r="AB150" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -10874,26 +10885,16 @@
           <t>G-Safeguard: A Topology-Guided Security Lens and Treatment on LLM-based Multi-agent Systems</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr"/>
-      <c r="D151" t="inlineStr"/>
       <c r="E151" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F151" t="inlineStr"/>
-      <c r="G151" t="inlineStr"/>
-      <c r="H151" t="inlineStr"/>
-      <c r="I151" t="inlineStr"/>
       <c r="J151" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K151" t="inlineStr"/>
-      <c r="Y151" t="inlineStr"/>
-      <c r="Z151" t="inlineStr"/>
-      <c r="AA151" t="inlineStr"/>
       <c r="AB151" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -10916,26 +10917,16 @@
           <t>MemBench: Towards More Comprehensive Evaluation on the Memory of LLM-based Agents</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr"/>
-      <c r="D152" t="inlineStr"/>
       <c r="E152" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F152" t="inlineStr"/>
-      <c r="G152" t="inlineStr"/>
-      <c r="H152" t="inlineStr"/>
-      <c r="I152" t="inlineStr"/>
       <c r="J152" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K152" t="inlineStr"/>
-      <c r="Y152" t="inlineStr"/>
-      <c r="Z152" t="inlineStr"/>
-      <c r="AA152" t="inlineStr"/>
       <c r="AB152" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -10958,26 +10949,16 @@
           <t>A Survey on the Optimization of Large Language Model-based Agents</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr"/>
-      <c r="D153" t="inlineStr"/>
       <c r="E153" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F153" t="inlineStr"/>
-      <c r="G153" t="inlineStr"/>
-      <c r="H153" t="inlineStr"/>
-      <c r="I153" t="inlineStr"/>
       <c r="J153" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K153" t="inlineStr"/>
-      <c r="Y153" t="inlineStr"/>
-      <c r="Z153" t="inlineStr"/>
-      <c r="AA153" t="inlineStr"/>
       <c r="AB153" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11000,26 +10981,31 @@
           <t>Hierarchical Memory for High-Efficiency Long-Term Reasoning in LLM Agents</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr"/>
-      <c r="D154" t="inlineStr"/>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Haoran Sun, Shaoning Zeng</t>
+        </is>
+      </c>
       <c r="E154" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F154" t="inlineStr"/>
-      <c r="G154" t="inlineStr"/>
-      <c r="H154" t="inlineStr"/>
-      <c r="I154" t="inlineStr"/>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>cs.CL, cs.AI</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Long-term memory is one of the key factors influencing the reasoning capabilities of Large Language Model Agents (LLM Agents). Incorporating a memory mechanism that effectively integrates past interactions can significantly enhance decision-making and contextual coherence of LLM Agents. While recent works have made progress in memory storage and retrieval, such as encoding memory into dense vectors for similarity-based search or organizing knowledge in the form of graph, these approaches often fall short in structured memory organization and efficient retrieval. To address these limitations, we propose a Hierarchical Memory (H-MEM) architecture for LLM Agents that organizes and updates memory in a multi-level fashion based on the degree of semantic abstraction. Each memory vector is embedded with a positional index encoding pointing to its semantically related sub-memories in the next layer. During the reasoning phase, an index-based routing mechanism enables efficient, layer-by-layer retrieval without performing exhaustive similarity computations. We evaluate our method on five task settings from the LoCoMo dataset. Experimental results show that our approach consistently outperforms five baseline methods, demonstrating its effectiveness in long-term dialogue scenarios.</t>
+        </is>
+      </c>
       <c r="J154" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K154" t="inlineStr"/>
-      <c r="Y154" t="inlineStr"/>
-      <c r="Z154" t="inlineStr"/>
-      <c r="AA154" t="inlineStr"/>
       <c r="AB154" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11042,26 +11028,16 @@
           <t>MPO: Boosting LLM Agents with Meta Plan Optimization</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr"/>
-      <c r="D155" t="inlineStr"/>
       <c r="E155" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F155" t="inlineStr"/>
-      <c r="G155" t="inlineStr"/>
-      <c r="H155" t="inlineStr"/>
-      <c r="I155" t="inlineStr"/>
       <c r="J155" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K155" t="inlineStr"/>
-      <c r="Y155" t="inlineStr"/>
-      <c r="Z155" t="inlineStr"/>
-      <c r="AA155" t="inlineStr"/>
       <c r="AB155" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11084,26 +11060,31 @@
           <t>A Survey of Personalization: From RAG to Agent</t>
         </is>
       </c>
-      <c r="C156" t="inlineStr"/>
-      <c r="D156" t="inlineStr"/>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Xiaopeng Li, Pengyue Jia, Derong Xu, Yi Wen, Yingyi Zhang, Wenlin Zhang, Wanyu Wang, Yichao Wang, Zhaocheng Du, Xiangyang Li, Yong Liu, Huifeng Guo, Ruiming Tang, Xiangyu Zhao</t>
+        </is>
+      </c>
       <c r="E156" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F156" t="inlineStr"/>
-      <c r="G156" t="inlineStr"/>
-      <c r="H156" t="inlineStr"/>
-      <c r="I156" t="inlineStr"/>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>cs.IR</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Personalization has become an essential capability in modern AI systems, enabling customized interactions that align with individual user preferences, contexts, and goals. Recent research has increasingly concentrated on Retrieval-Augmented Generation (RAG) frameworks and their evolution into more advanced agent-based architectures within personalized settings to enhance user satisfaction. Building on this foundation, this survey systematically examines personalization across the three core stages of RAG: pre-retrieval, retrieval, and generation. Beyond RAG, we further extend its capabilities into the realm of Personalized LLM-based Agents, which enhance traditional RAG systems with agentic functionalities, including user understanding, personalized planning and execution, and dynamic generation. For both personalization in RAG and agent-based personalization, we provide formal definitions, conduct a comprehensive review of recent literature, and summarize key datasets and evaluation metrics. Additionally, we discuss fundamental challenges, limitations, and promising research directions in this evolving field. Relevant papers and resources are continuously updated at https://github.com/Applied-Machine-Learning-Lab/Awesome-Personalized-RAG-Agent.</t>
+        </is>
+      </c>
       <c r="J156" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K156" t="inlineStr"/>
-      <c r="Y156" t="inlineStr"/>
-      <c r="Z156" t="inlineStr"/>
-      <c r="AA156" t="inlineStr"/>
       <c r="AB156" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11126,26 +11107,16 @@
           <t>OAgents: An Empirical Study of Building Effective Agents</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr"/>
-      <c r="D157" t="inlineStr"/>
       <c r="E157" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F157" t="inlineStr"/>
-      <c r="G157" t="inlineStr"/>
-      <c r="H157" t="inlineStr"/>
-      <c r="I157" t="inlineStr"/>
       <c r="J157" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K157" t="inlineStr"/>
-      <c r="Y157" t="inlineStr"/>
-      <c r="Z157" t="inlineStr"/>
-      <c r="AA157" t="inlineStr"/>
       <c r="AB157" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11168,26 +11139,16 @@
           <t>MCP-AgentBench: Evaluating Real-World Language Agent Performance with MCP-Mediated Tools</t>
         </is>
       </c>
-      <c r="C158" t="inlineStr"/>
-      <c r="D158" t="inlineStr"/>
       <c r="E158" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F158" t="inlineStr"/>
-      <c r="G158" t="inlineStr"/>
-      <c r="H158" t="inlineStr"/>
-      <c r="I158" t="inlineStr"/>
       <c r="J158" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K158" t="inlineStr"/>
-      <c r="Y158" t="inlineStr"/>
-      <c r="Z158" t="inlineStr"/>
-      <c r="AA158" t="inlineStr"/>
       <c r="AB158" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11210,26 +11171,16 @@
           <t>AgentCF++: Memory-enhanced LLM-based Agents for Popularity-aware Cross-domain Recommendations</t>
         </is>
       </c>
-      <c r="C159" t="inlineStr"/>
-      <c r="D159" t="inlineStr"/>
       <c r="E159" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F159" t="inlineStr"/>
-      <c r="G159" t="inlineStr"/>
-      <c r="H159" t="inlineStr"/>
-      <c r="I159" t="inlineStr"/>
       <c r="J159" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K159" t="inlineStr"/>
-      <c r="Y159" t="inlineStr"/>
-      <c r="Z159" t="inlineStr"/>
-      <c r="AA159" t="inlineStr"/>
       <c r="AB159" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11252,26 +11203,16 @@
           <t>GA-S3: Comprehensive Social Network Simulation with Group Agents</t>
         </is>
       </c>
-      <c r="C160" t="inlineStr"/>
-      <c r="D160" t="inlineStr"/>
       <c r="E160" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F160" t="inlineStr"/>
-      <c r="G160" t="inlineStr"/>
-      <c r="H160" t="inlineStr"/>
-      <c r="I160" t="inlineStr"/>
       <c r="J160" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K160" t="inlineStr"/>
-      <c r="Y160" t="inlineStr"/>
-      <c r="Z160" t="inlineStr"/>
-      <c r="AA160" t="inlineStr"/>
       <c r="AB160" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11294,26 +11235,16 @@
           <t>Truly Self-Improving Agents Require Intrinsic Metacognitive Learning</t>
         </is>
       </c>
-      <c r="C161" t="inlineStr"/>
-      <c r="D161" t="inlineStr"/>
       <c r="E161" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F161" t="inlineStr"/>
-      <c r="G161" t="inlineStr"/>
-      <c r="H161" t="inlineStr"/>
-      <c r="I161" t="inlineStr"/>
       <c r="J161" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K161" t="inlineStr"/>
-      <c r="Y161" t="inlineStr"/>
-      <c r="Z161" t="inlineStr"/>
-      <c r="AA161" t="inlineStr"/>
       <c r="AB161" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11336,26 +11267,16 @@
           <t>An LLM-based multi-agent framework for agile effort estimation</t>
         </is>
       </c>
-      <c r="C162" t="inlineStr"/>
-      <c r="D162" t="inlineStr"/>
       <c r="E162" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F162" t="inlineStr"/>
-      <c r="G162" t="inlineStr"/>
-      <c r="H162" t="inlineStr"/>
-      <c r="I162" t="inlineStr"/>
       <c r="J162" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K162" t="inlineStr"/>
-      <c r="Y162" t="inlineStr"/>
-      <c r="Z162" t="inlineStr"/>
-      <c r="AA162" t="inlineStr"/>
       <c r="AB162" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11378,26 +11299,16 @@
           <t>Position: Build Agent Advocates, Not Platform Agents</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr"/>
-      <c r="D163" t="inlineStr"/>
       <c r="E163" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F163" t="inlineStr"/>
-      <c r="G163" t="inlineStr"/>
-      <c r="H163" t="inlineStr"/>
-      <c r="I163" t="inlineStr"/>
       <c r="J163" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K163" t="inlineStr"/>
-      <c r="Y163" t="inlineStr"/>
-      <c r="Z163" t="inlineStr"/>
-      <c r="AA163" t="inlineStr"/>
       <c r="AB163" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11420,26 +11331,16 @@
           <t>Are Autonomous Web Agents Good Testers?</t>
         </is>
       </c>
-      <c r="C164" t="inlineStr"/>
-      <c r="D164" t="inlineStr"/>
       <c r="E164" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F164" t="inlineStr"/>
-      <c r="G164" t="inlineStr"/>
-      <c r="H164" t="inlineStr"/>
-      <c r="I164" t="inlineStr"/>
       <c r="J164" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K164" t="inlineStr"/>
-      <c r="Y164" t="inlineStr"/>
-      <c r="Z164" t="inlineStr"/>
-      <c r="AA164" t="inlineStr"/>
       <c r="AB164" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11462,26 +11363,16 @@
           <t>ModelingAgent: Bridging LLMs and Mathematical Modeling for Real-World Challenges</t>
         </is>
       </c>
-      <c r="C165" t="inlineStr"/>
-      <c r="D165" t="inlineStr"/>
       <c r="E165" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F165" t="inlineStr"/>
-      <c r="G165" t="inlineStr"/>
-      <c r="H165" t="inlineStr"/>
-      <c r="I165" t="inlineStr"/>
       <c r="J165" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K165" t="inlineStr"/>
-      <c r="Y165" t="inlineStr"/>
-      <c r="Z165" t="inlineStr"/>
-      <c r="AA165" t="inlineStr"/>
       <c r="AB165" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11504,26 +11395,16 @@
           <t>DrunkAgent: Stealthy Memory Corruption in LLM-Powered Recommender Agents</t>
         </is>
       </c>
-      <c r="C166" t="inlineStr"/>
-      <c r="D166" t="inlineStr"/>
       <c r="E166" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F166" t="inlineStr"/>
-      <c r="G166" t="inlineStr"/>
-      <c r="H166" t="inlineStr"/>
-      <c r="I166" t="inlineStr"/>
       <c r="J166" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K166" t="inlineStr"/>
-      <c r="Y166" t="inlineStr"/>
-      <c r="Z166" t="inlineStr"/>
-      <c r="AA166" t="inlineStr"/>
       <c r="AB166" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11546,26 +11427,31 @@
           <t>StorySage: Conversational Autobiography Writing Powered by a Multi-Agent Framework</t>
         </is>
       </c>
-      <c r="C167" t="inlineStr"/>
-      <c r="D167" t="inlineStr"/>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Shayan Talaei, Meijin Li, Kanu Grover, James Kent Hippler, Diyi Yang, Amin Saberi</t>
+        </is>
+      </c>
       <c r="E167" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F167" t="inlineStr"/>
-      <c r="G167" t="inlineStr"/>
-      <c r="H167" t="inlineStr"/>
-      <c r="I167" t="inlineStr"/>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>cs.HC, cs.AI, cs.MA</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>Every individual carries a unique and personal life story shaped by their memories and experiences. However, these memories are often scattered and difficult to organize into a coherent narrative, a challenge that defines the task of autobiography writing. Existing conversational writing assistants tend to rely on generic user interactions and pre-defined guidelines, making it difficult for these systems to capture personal memories and develop a complete biography over time. We introduce StorySage, a user-driven software system designed to meet the needs of a diverse group of users that supports a flexible conversation and a structured approach to autobiography writing. Powered by a multi-agent framework composed of an Interviewer, Session Scribe, Planner, Section Writer, and Session Coordinator, our system iteratively collects user memories, updates their autobiography, and plans for future conversations. In experimental simulations, StorySage demonstrates its ability to navigate multiple sessions and capture user memories across many conversations. User studies (N=28) highlight how StorySage maintains improved conversational flow, narrative completeness, and higher user satisfaction when compared to a baseline. In summary, StorySage contributes both a novel architecture for autobiography writing and insights into how multi-agent systems can enhance human-AI creative partnerships.</t>
+        </is>
+      </c>
       <c r="J167" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K167" t="inlineStr"/>
-      <c r="Y167" t="inlineStr"/>
-      <c r="Z167" t="inlineStr"/>
-      <c r="AA167" t="inlineStr"/>
       <c r="AB167" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11588,26 +11474,31 @@
           <t>RALLY: Role-Adaptive LLM-Driven Yoked Navigation for Agentic UAV Swarms</t>
         </is>
       </c>
-      <c r="C168" t="inlineStr"/>
-      <c r="D168" t="inlineStr"/>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Ziyao Wang, Rongpeng Li, Sizhao Li, Yuming Xiang, Haiping Wang, Zhifeng Zhao, Honggang Zhang</t>
+        </is>
+      </c>
       <c r="E168" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F168" t="inlineStr"/>
-      <c r="G168" t="inlineStr"/>
-      <c r="H168" t="inlineStr"/>
-      <c r="I168" t="inlineStr"/>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>cs.MA, cs.AI, cs.RO</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>Intelligent control of Unmanned Aerial Vehicles (UAVs) swarms has emerged as a critical research focus, and it typically requires the swarm to navigate effectively while avoiding obstacles and achieving continuous coverage over multiple mission targets. Although traditional Multi-Agent Reinforcement Learning (MARL) approaches offer dynamic adaptability, they are hindered by the semantic gap in numerical communication and the rigidity of homogeneous role structures, resulting in poor generalization and limited task scalability. Recent advances in Large Language Model (LLM)-based control frameworks demonstrate strong semantic reasoning capabilities by leveraging extensive prior knowledge. However, due to the lack of online learning and over-reliance on static priors, these works often struggle with effective exploration, leading to reduced individual potential and overall system performance. To address these limitations, we propose a Role-Adaptive LLM-Driven Yoked navigation algorithm RALLY. Specifically, we first develop an LLM-driven semantic decision framework that uses structured natural language for efficient semantic communication and collaborative reasoning. Afterward, we introduce a dynamic role-heterogeneity mechanism for adaptive role switching and personalized decision-making. Furthermore, we propose a Role-value Mixing Network (RMIX)-based assignment strategy that integrates LLM offline priors with MARL online policies to enable semi-offline training of role selection strategies. Experiments in the Multi-Agent Particle Environment (MPE) environment and a Software-In-The-Loop (SITL) platform demonstrate that RALLY outperforms conventional approaches in terms of task coverage, convergence speed, and generalization, highlighting its strong potential for collaborative navigation in agentic multi-UAV systems.</t>
+        </is>
+      </c>
       <c r="J168" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K168" t="inlineStr"/>
-      <c r="Y168" t="inlineStr"/>
-      <c r="Z168" t="inlineStr"/>
-      <c r="AA168" t="inlineStr"/>
       <c r="AB168" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11630,26 +11521,31 @@
           <t>FadeMem: Biologically-Inspired Forgetting for Efficient Agent Memory</t>
         </is>
       </c>
-      <c r="C169" t="inlineStr"/>
-      <c r="D169" t="inlineStr"/>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Lei Wei, Xiao Peng, Xu Dong, Niantao Xie, Bin Wang</t>
+        </is>
+      </c>
       <c r="E169" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="F169" t="inlineStr"/>
-      <c r="G169" t="inlineStr"/>
-      <c r="H169" t="inlineStr"/>
-      <c r="I169" t="inlineStr"/>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>cs.AI, cs.CL</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>Large language models deployed as autonomous agents face critical memory limitations, lacking selective forgetting mechanisms that lead to either catastrophic forgetting at context boundaries or information overload within them. While human memory naturally balances retention and forgetting through adaptive decay processes, current AI systems employ binary retention strategies that preserve everything or lose it entirely. We propose FadeMem, a biologically-inspired agent memory architecture that incorporates active forgetting mechanisms mirroring human cognitive efficiency. FadeMem implements differential decay rates across a dual-layer memory hierarchy, where retention is governed by adaptive exponential decay functions modulated by semantic relevance, access frequency, and temporal patterns. Through LLM-guided conflict resolution and intelligent memory fusion, our system consolidates related information while allowing irrelevant details to fade. Experiments on Multi-Session Chat, LoCoMo, and LTI-Bench demonstrate superior multi-hop reasoning and retrieval with 45\% storage reduction, validating the effectiveness of biologically-inspired forgetting in agent memory systems.</t>
+        </is>
+      </c>
       <c r="J169" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K169" t="inlineStr"/>
-      <c r="Y169" t="inlineStr"/>
-      <c r="Z169" t="inlineStr"/>
-      <c r="AA169" t="inlineStr"/>
       <c r="AB169" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11672,26 +11568,31 @@
           <t>Memoria: A Scalable Agentic Memory Framework for Personalized Conversational AI</t>
         </is>
       </c>
-      <c r="C170" t="inlineStr"/>
-      <c r="D170" t="inlineStr"/>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Samarth Sarin, Lovepreet Singh, Bhaskarjit Sarmah, Dhagash Mehta</t>
+        </is>
+      </c>
       <c r="E170" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F170" t="inlineStr"/>
-      <c r="G170" t="inlineStr"/>
-      <c r="H170" t="inlineStr"/>
-      <c r="I170" t="inlineStr"/>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>cs.AI, cs.CL</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Agentic memory is emerging as a key enabler for large language models (LLM) to maintain continuity, personalization, and long-term context in extended user interactions, critical capabilities for deploying LLMs as truly interactive and adaptive agents. Agentic memory refers to the memory that provides an LLM with agent-like persistence: the ability to retain and act upon information across conversations, similar to how a human would. We present Memoria, a modular memory framework that augments LLM-based conversational systems with persistent, interpretable, and context-rich memory. Memoria integrates two complementary components: dynamic session-level summarization and a weighted knowledge graph (KG)-based user modelling engine that incrementally captures user traits, preferences, and behavioral patterns as structured entities and relationships. This hybrid architecture enables both short-term dialogue coherence and long-term personalization while operating within the token constraints of modern LLMs. We demonstrate how Memoria enables scalable, personalized conversational artificial intelligence (AI) by bridging the gap between stateless LLM interfaces and agentic memory systems, offering a practical solution for industry applications requiring adaptive and evolving user experiences.</t>
+        </is>
+      </c>
       <c r="J170" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K170" t="inlineStr"/>
-      <c r="Y170" t="inlineStr"/>
-      <c r="Z170" t="inlineStr"/>
-      <c r="AA170" t="inlineStr"/>
       <c r="AB170" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11714,26 +11615,31 @@
           <t>Sari Sandbox: A Virtual Retail Store Environment for Embodied AI Agents</t>
         </is>
       </c>
-      <c r="C171" t="inlineStr"/>
-      <c r="D171" t="inlineStr"/>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Janika Deborah Gajo, Gerarld Paul Merales, Jerome Escarcha, Brenden Ashley Molina, Gian Nartea, Emmanuel G. Maminta, Juan Carlos Roldan, Rowel O. Atienza</t>
+        </is>
+      </c>
       <c r="E171" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F171" t="inlineStr"/>
-      <c r="G171" t="inlineStr"/>
-      <c r="H171" t="inlineStr"/>
-      <c r="I171" t="inlineStr"/>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>cs.CV</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>We present Sari Sandbox, a high-fidelity, photorealistic 3D retail store simulation for benchmarking embodied agents against human performance in shopping tasks. Addressing a gap in retail-specific sim environments for embodied agent training, Sari Sandbox features over 250 interactive grocery items across three store configurations, controlled via an API. It supports both virtual reality (VR) for human interaction and a vision language model (VLM)-powered embodied agent. We also introduce SariBench, a dataset of annotated human demonstrations across varied task difficulties. Our sandbox enables embodied agents to navigate, inspect, and manipulate retail items, providing baselines against human performance. We conclude with benchmarks, performance analysis, and recommendations for enhancing realism and scalability. The source code can be accessed via https://github.com/upeee/sari-sandbox-env.</t>
+        </is>
+      </c>
       <c r="J171" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K171" t="inlineStr"/>
-      <c r="Y171" t="inlineStr"/>
-      <c r="Z171" t="inlineStr"/>
-      <c r="AA171" t="inlineStr"/>
       <c r="AB171" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11756,26 +11662,31 @@
           <t>Games Agents Play: Towards Transactional Analysis in LLM-based Multi-Agent Systems</t>
         </is>
       </c>
-      <c r="C172" t="inlineStr"/>
-      <c r="D172" t="inlineStr"/>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Monika Zamojska, Jarosław A. Chudziak</t>
+        </is>
+      </c>
       <c r="E172" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F172" t="inlineStr"/>
-      <c r="G172" t="inlineStr"/>
-      <c r="H172" t="inlineStr"/>
-      <c r="I172" t="inlineStr"/>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>cs.AI, cs.MA</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Multi-Agent Systems (MAS) are increasingly used to simulate social interactions, but most of the frameworks miss the underlying cognitive complexity of human behavior. In this paper, we introduce Trans-ACT (Transactional Analysis Cognitive Toolkit), an approach embedding Transactional Analysis (TA) principles into MAS to generate agents with realistic psychological dynamics. Trans-ACT integrates the Parent, Adult, and Child ego states into an agent's cognitive architecture. Each ego state retrieves context-specific memories and uses them to shape response to new situations. The final answer is chosen according to the underlying life script of the agent. Our experimental simulation, which reproduces the Stupid game scenario, demonstrates that agents grounded in cognitive and TA principles produce deeper and context-aware interactions. Looking ahead, our research opens a new way for a variety of applications, including conflict resolution, educational support, and advanced social psychology studies.</t>
+        </is>
+      </c>
       <c r="J172" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K172" t="inlineStr"/>
-      <c r="Y172" t="inlineStr"/>
-      <c r="Z172" t="inlineStr"/>
-      <c r="AA172" t="inlineStr"/>
       <c r="AB172" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11798,26 +11709,31 @@
           <t>TRIZ Agents: A Multi-Agent LLM Approach for TRIZ-Based Innovation</t>
         </is>
       </c>
-      <c r="C173" t="inlineStr"/>
-      <c r="D173" t="inlineStr"/>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Kamil Szczepanik, Jarosław A. Chudziak</t>
+        </is>
+      </c>
       <c r="E173" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F173" t="inlineStr"/>
-      <c r="G173" t="inlineStr"/>
-      <c r="H173" t="inlineStr"/>
-      <c r="I173" t="inlineStr"/>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>cs.AI, cs.MA</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>TRIZ, the Theory of Inventive Problem Solving, is a structured, knowledge-based framework for innovation and abstracting problems to find inventive solutions. However, its application is often limited by the complexity and deep interdisciplinary knowledge required. Advancements in Large Language Models (LLMs) have revealed new possibilities for automating parts of this process. While previous studies have explored single LLMs in TRIZ applications, this paper introduces a multi-agent approach. We propose an LLM-based multi-agent system, called TRIZ agents, each with specialized capabilities and tool access, collaboratively solving inventive problems based on the TRIZ methodology. This multi-agent system leverages agents with various domain expertise to efficiently navigate TRIZ steps. The aim is to model and simulate an inventive process with language agents. We assess the effectiveness of this team of agents in addressing complex innovation challenges based on a selected case study in engineering. We demonstrate the potential of agent collaboration to produce diverse, inventive solutions. This research contributes to the future of AI-driven innovation, showcasing the advantages of decentralized problem-solving in complex ideation tasks.</t>
+        </is>
+      </c>
       <c r="J173" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K173" t="inlineStr"/>
-      <c r="Y173" t="inlineStr"/>
-      <c r="Z173" t="inlineStr"/>
-      <c r="AA173" t="inlineStr"/>
       <c r="AB173" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11840,26 +11756,31 @@
           <t>Querying Large Automotive Software Models: Agentic vs. Direct LLM Approaches</t>
         </is>
       </c>
-      <c r="C174" t="inlineStr"/>
-      <c r="D174" t="inlineStr"/>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Lukasz Mazur, Nenad Petrovic, James Pontes Miranda, Ansgar Radermacher, Robert Rasche, Alois Knoll</t>
+        </is>
+      </c>
       <c r="E174" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F174" t="inlineStr"/>
-      <c r="G174" t="inlineStr"/>
-      <c r="H174" t="inlineStr"/>
-      <c r="I174" t="inlineStr"/>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>cs.SE, cs.AI</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Large language models (LLMs) offer new opportunities for interacting with complex software artifacts, such as software models, through natural language. They present especially promising benefits for large software models that are difficult to grasp in their entirety, making traditional interaction and analysis approaches challenging. This paper investigates two approaches for leveraging LLMs to answer questions over software models: direct prompting, where the whole software model is provided in the context, and an agentic approach combining LLM-based agents with general-purpose file access tools. We evaluate these approaches using an Ecore metamodel designed for timing analysis and software optimization in automotive and embedded domains. Our findings show that while the agentic approach achieves accuracy comparable to direct prompting, it is significantly more efficient in terms of token usage. This efficiency makes the agentic approach particularly suitable for the automotive industry, where the large size of software models makes direct prompting infeasible, establishing LLM agents as not just a practical alternative but the only viable solution. Notably, the evaluation was conducted using small LLMs, which are more feasible to be executed locally - an essential advantage for meeting strict requirements around privacy, intellectual property protection, and regulatory compliance. Future work will investigate software models in diverse formats, explore more complex agent architectures, and extend agentic workflows to support not only querying but also modification of software models.</t>
+        </is>
+      </c>
       <c r="J174" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K174" t="inlineStr"/>
-      <c r="Y174" t="inlineStr"/>
-      <c r="Z174" t="inlineStr"/>
-      <c r="AA174" t="inlineStr"/>
       <c r="AB174" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11882,26 +11803,31 @@
           <t>Augmenting Multi-Agent Communication with State Delta Trajectory</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr"/>
-      <c r="D175" t="inlineStr"/>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Yichen Tang, Weihang Su, Yujia Zhou, Yiqun Liu, Min Zhang, Shaoping Ma, Qingyao Ai</t>
+        </is>
+      </c>
       <c r="E175" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F175" t="inlineStr"/>
-      <c r="G175" t="inlineStr"/>
-      <c r="H175" t="inlineStr"/>
-      <c r="I175" t="inlineStr"/>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>cs.CL</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>Multi-agent techniques such as role playing or multi-turn debates have been shown to be effective in improving the performance of large language models (LLMs) in downstream tasks. Despite their differences in workflows, existing multi-agent systems constructed from a single base LLM mostly use natural language for agent communication. While this is appealing for its simplicity and interpretability, it also introduces inevitable information loss as one model must down sample its continuous state vectors to discrete tokens before transferring them to the other model. Such losses are particularly significant when the information to transfer is not simple facts, but reasoning logics or abstractive thoughts. To tackle this problem, we propose a new communication protocol that transfers both natural language tokens and token-wise state transition trajectory from one agent to another. Particularly, compared to the actual state value, we find that the sequence of state changes in LLMs after generating each token can better reflect the information hidden behind the inference process. We propose a State Delta Encoding (SDE) method to represent state transition trajectories. The experimental results show that multi-agent systems with SDE achieve SOTA performance compared to other communication protocols, particularly in tasks that involve complex reasoning.</t>
+        </is>
+      </c>
       <c r="J175" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K175" t="inlineStr"/>
-      <c r="Y175" t="inlineStr"/>
-      <c r="Z175" t="inlineStr"/>
-      <c r="AA175" t="inlineStr"/>
       <c r="AB175" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11924,26 +11850,31 @@
           <t>MemoCue: Empowering LLM-Based Agents for Human Memory Recall via Strategy-Guided Querying</t>
         </is>
       </c>
-      <c r="C176" t="inlineStr"/>
-      <c r="D176" t="inlineStr"/>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Qian Zhao, Zhuo Sun, Bin Guo, Zhiwen Yu</t>
+        </is>
+      </c>
       <c r="E176" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F176" t="inlineStr"/>
-      <c r="G176" t="inlineStr"/>
-      <c r="H176" t="inlineStr"/>
-      <c r="I176" t="inlineStr"/>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>cs.AI</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>Agent-assisted memory recall is one critical research problem in the field of human-computer interaction. In conventional methods, the agent can retrieve information from its equipped memory module to help the person recall incomplete or vague memories. The limited size of memory module hinders the acquisition of complete memories and impacts the memory recall performance in practice. Memory theories suggest that the person's relevant memory can be proactively activated through some effective cues. Inspired by this, we propose a novel strategy-guided agent-assisted memory recall method, allowing the agent to transform an original query into a cue-rich one via the judiciously designed strategy to help the person recall memories. To this end, there are two key challenges. (1) How to choose the appropriate recall strategy for diverse forgetting scenarios with distinct memory-recall characteristics? (2) How to obtain the high-quality responses leveraging recall strategies, given only abstract and sparsely annotated strategy patterns? To address the challenges, we propose a Recall Router framework. Specifically, we design a 5W Recall Map to classify memory queries into five typical scenarios and define fifteen recall strategy patterns across the corresponding scenarios. We then propose a hierarchical recall tree combined with the Monte Carlo Tree Search algorithm to optimize the selection of strategy and the generation of strategy responses. We construct an instruction tuning dataset and fine-tune multiple open-source large language models (LLMs) to develop MemoCue, an agent that excels in providing memory-inspired responses. Experiments on three representative datasets show that MemoCue surpasses LLM-based methods by 17.74% in recall inspiration. Further human evaluation highlights its advantages in memory-recall applications.</t>
+        </is>
+      </c>
       <c r="J176" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K176" t="inlineStr"/>
-      <c r="Y176" t="inlineStr"/>
-      <c r="Z176" t="inlineStr"/>
-      <c r="AA176" t="inlineStr"/>
       <c r="AB176" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11966,26 +11897,31 @@
           <t>Interview-Informed Generative Agents for Product Discovery: A Validation Study</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr"/>
-      <c r="D177" t="inlineStr"/>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Zichao Wang, Alexa Siu</t>
+        </is>
+      </c>
       <c r="E177" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="F177" t="inlineStr"/>
-      <c r="G177" t="inlineStr"/>
-      <c r="H177" t="inlineStr"/>
-      <c r="I177" t="inlineStr"/>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>cs.HC, cs.AI</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>Large language models (LLMs) have shown strong performance on standardized social science instruments, but their value for product discovery remains unclear. We investigate whether interview-informed generative agents can simulate user responses in concept testing scenarios. Using in-depth workflow interviews with knowledge workers, we created personalized agents and compared their evaluations of novel AI concepts against the same participants' responses. Our results show that agents are distribution-calibrated but identity-imprecise: they fail to replicate the specific individual they are grounded in, yet approximate population-level response distributions. These findings highlight both the potential and the limits of LLM simulation in design research. While unsuitable as a substitute for individual-level insights, simulation may provide value for early-stage concept screening and iteration, where distributional accuracy suffices. We discuss implications for integrating simulation responsibly into product development workflows.</t>
+        </is>
+      </c>
       <c r="J177" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K177" t="inlineStr"/>
-      <c r="Y177" t="inlineStr"/>
-      <c r="Z177" t="inlineStr"/>
-      <c r="AA177" t="inlineStr"/>
       <c r="AB177" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -12008,26 +11944,31 @@
           <t>Designing Memory-Augmented AR Agents for Spatiotemporal Reasoning in Personalized Task Assistance</t>
         </is>
       </c>
-      <c r="C178" t="inlineStr"/>
-      <c r="D178" t="inlineStr"/>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Dongwook Choi, Taeyoon Kwon, Dongil Yang, Hyojun Kim, Jinyoung Yeo</t>
+        </is>
+      </c>
       <c r="E178" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F178" t="inlineStr"/>
-      <c r="G178" t="inlineStr"/>
-      <c r="H178" t="inlineStr"/>
-      <c r="I178" t="inlineStr"/>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>cs.AI, cs.CL</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>Augmented Reality (AR) systems are increasingly integrating foundation models, such as Multimodal Large Language Models (MLLMs), to provide more context-aware and adaptive user experiences. This integration has led to the development of AR agents to support intelligent, goal-directed interactions in real-world environments. While current AR agents effectively support immediate tasks, they struggle with complex multi-step scenarios that require understanding and leveraging user's long-term experiences and preferences. This limitation stems from their inability to capture, retain, and reason over historical user interactions in spatiotemporal contexts. To address these challenges, we propose a conceptual framework for memory-augmented AR agents that can provide personalized task assistance by learning from and adapting to user-specific experiences over time. Our framework consists of four interconnected modules: (1) Perception Module for multimodal sensor processing, (2) Memory Module for persistent spatiotemporal experience storage, (3) Spatiotemporal Reasoning Module for synthesizing past and present contexts, and (4) Actuator Module for effective AR communication. We further present an implementation roadmap, a future evaluation strategy, a potential target application and use cases to demonstrate the practical applicability of our framework across diverse domains. We aim for this work to motivate future research toward developing more intelligent AR systems that can effectively bridge user's interaction history with adaptive, context-aware task assistance.</t>
+        </is>
+      </c>
       <c r="J178" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K178" t="inlineStr"/>
-      <c r="Y178" t="inlineStr"/>
-      <c r="Z178" t="inlineStr"/>
-      <c r="AA178" t="inlineStr"/>
       <c r="AB178" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -12050,26 +11991,31 @@
           <t>Agentic AI in Healthcare and Medicine: A Seven-Dimensional Taxonomy for Empirical Evaluation of LLM-Based Agents</t>
         </is>
       </c>
-      <c r="C179" t="inlineStr"/>
-      <c r="D179" t="inlineStr"/>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Shubham Vatsal, Harsh Dubey, Aditi Singh</t>
+        </is>
+      </c>
       <c r="E179" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="F179" t="inlineStr"/>
-      <c r="G179" t="inlineStr"/>
-      <c r="H179" t="inlineStr"/>
-      <c r="I179" t="inlineStr"/>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>cs.AI, cs.CY</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>Large Language Model (LLM)-based agents that plan, use tools and act has begun to shape healthcare and medicine. Reported studies demonstrate competence on various tasks ranging from EHR analysis and differential diagnosis to treatment planning and research workflows. Yet the literature largely consists of overviews which are either broad surveys or narrow dives into a single capability (e.g., memory, planning, reasoning), leaving healthcare work without a common frame. We address this by reviewing 49 studies using a seven-dimensional taxonomy: Cognitive Capabilities, Knowledge Management, Interaction Patterns, Adaptation &amp; Learning, Safety &amp; Ethics, Framework Typology and Core Tasks &amp; Subtasks with 29 operational sub-dimensions. Using explicit inclusion and exclusion criteria and a labeling rubric (Fully Implemented, Partially Implemented, Not Implemented), we map each study to the taxonomy and report quantitative summaries of capability prevalence and co-occurrence patterns. Our empirical analysis surfaces clear asymmetries. For instance, the External Knowledge Integration sub-dimension under Knowledge Management is commonly realized (~76% Fully Implemented) whereas Event-Triggered Activation sub-dimenison under Interaction Patterns is largely absent (~92% Not Implemented) and Drift Detection &amp; Mitigation sub-dimension under Adaptation &amp; Learning is rare (~98% Not Implemented). Architecturally, Multi-Agent Design sub-dimension under Framework Typology is the dominant pattern (~82% Fully Implemented) while orchestration layers remain mostly partial. Across Core Tasks &amp; Subtasks, information centric capabilities lead e.g., Medical Question Answering &amp; Decision Support and Benchmarking &amp; Simulation, while action and discovery oriented areas such as Treatment Planning &amp; Prescription still show substantial gaps (~59% Not Implemented).</t>
+        </is>
+      </c>
       <c r="J179" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K179" t="inlineStr"/>
-      <c r="Y179" t="inlineStr"/>
-      <c r="Z179" t="inlineStr"/>
-      <c r="AA179" t="inlineStr"/>
       <c r="AB179" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -12092,26 +12038,31 @@
           <t>ClawVM: Harness-Managed Virtual Memory for Stateful Tool-Using LLM Agents</t>
         </is>
       </c>
-      <c r="C180" t="inlineStr"/>
-      <c r="D180" t="inlineStr"/>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Mofasshara Rafique, Laurent Bindschaedler</t>
+        </is>
+      </c>
       <c r="E180" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="F180" t="inlineStr"/>
-      <c r="G180" t="inlineStr"/>
-      <c r="H180" t="inlineStr"/>
-      <c r="I180" t="inlineStr"/>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>cs.AI, cs.OS, cs.SE</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Stateful tool-using LLM agents treat the context window as working memory, yet today's agent harnesses manage residency and durability as best-effort, causing recurring failures: lost state after compaction, bypassed flushes on reset, and destructive writeback. We present \textsc{ClawVM}, a virtual memory layer that manages state as typed pages with minimum-fidelity invariants, multi-resolution representations under a token budget, and validated writeback at every lifecycle boundary. Because the harness already assembles prompts, mediates tools, and observes lifecycle events, it is the natural enforcement point; placing the contract there makes residency and durability deterministic and auditable. Across synthetic workloads, 12 real-session traces, and adversarial stress tests, \textsc{ClawVM} eliminates all policy-controllable faults whenever the minimum-fidelity set fits within the token budget, confirmed by an offline oracle, and adds median &lt;50 microseconds of policy-engine overhead per turn.</t>
+        </is>
+      </c>
       <c r="J180" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K180" t="inlineStr"/>
-      <c r="Y180" t="inlineStr"/>
-      <c r="Z180" t="inlineStr"/>
-      <c r="AA180" t="inlineStr"/>
       <c r="AB180" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -12134,26 +12085,31 @@
           <t>InnerPond: Fostering Inter-Self Dialogue with a Multi-Agent Approach for Introspection</t>
         </is>
       </c>
-      <c r="C181" t="inlineStr"/>
-      <c r="D181" t="inlineStr"/>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Hayeon Jeon, Dakyeom Ahn, Sunyu Pang, Yunseo Choi, Suhwoo Yoon, Joonhwan Lee, Eun-mee Kim, Hajin Lim</t>
+        </is>
+      </c>
       <c r="E181" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="F181" t="inlineStr"/>
-      <c r="G181" t="inlineStr"/>
-      <c r="H181" t="inlineStr"/>
-      <c r="I181" t="inlineStr"/>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>cs.HC, cs.AI</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Introspection is central to identity construction and future planning, yet most digital tools approach the self as a unified entity. In contrast, Dialogical Self Theory (DST) views the self as composed of multiple internal perspectives, such as values, concerns, and aspirations, that can come into tension or dialogue with one another. Building on this view, we designed InnerPond, a research probe in the form of a multi-agent system that represents these internal perspectives as distinct LLM-based agents for introspection. Its design was shaped through iterative explorations of spatial metaphors, interaction scaffolding, and conversational orchestration, culminating in a shared spatial environment for organizing and relating multiple inner perspectives. In a user study with 17 young adults navigating career choices, participants engaged with the probe by co-creating inner voices with AI, composing relational inner landscapes, and orchestrating dialogue as observers and mediators, offering insight into how such systems could support introspection. Overall, this work offers design implications for AI-supported introspection tools that enable exploration of the self's multiplicity.</t>
+        </is>
+      </c>
       <c r="J181" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K181" t="inlineStr"/>
-      <c r="Y181" t="inlineStr"/>
-      <c r="Z181" t="inlineStr"/>
-      <c r="AA181" t="inlineStr"/>
       <c r="AB181" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -12176,26 +12132,31 @@
           <t>Belief-Driven Multi-Agent Collaboration via Approximate Perfect Bayesian Equilibrium for Social Simulation</t>
         </is>
       </c>
-      <c r="C182" t="inlineStr"/>
-      <c r="D182" t="inlineStr"/>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Weiwei Fang, Lin Li, Kaize Shi, Yu Yang, Jianwei Zhang</t>
+        </is>
+      </c>
       <c r="E182" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="F182" t="inlineStr"/>
-      <c r="G182" t="inlineStr"/>
-      <c r="H182" t="inlineStr"/>
-      <c r="I182" t="inlineStr"/>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>cs.MA</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>High-fidelity social simulation is pivotal for addressing complex Web societal challenges, yet it demands agents capable of authentically replicating the dynamic spectrum of human interaction. Current LLM-based multi-agent frameworks, however, predominantly adhere to static interaction topologies, failing to capture the fluid oscillation between cooperative knowledge synthesis and competitive critical reasoning seen in real-world scenarios. This rigidity often leads to unrealistic ``groupthink'' or unproductive deadlocks, undermining the credibility of simulations for decision support. To bridge this gap, we propose \textit{BEACOF}, a \textit{belief-driven adaptive collaboration framework} inspired by Perfect Bayesian Equilibrium (PBE). By modeling social interaction as a dynamic game of incomplete information, BEACOF rigorously addresses the circular dependency between collaboration type selection and capability estimation. Agents iteratively refine probabilistic beliefs about peer capabilities and autonomously modulate their collaboration strategy, thereby ensuring sequentially rational decisions under uncertainty. Validated across adversarial (judicial), open-ended (social) and mixed (medical) scenarios, BEACOF prevents coordination failures and fosters robust convergence toward high-quality solutions, demonstrating superior potential for reliable social simulation. Source codes and datasets are publicly released at: https://github.com/WUT-IDEA/BEACOF.</t>
+        </is>
+      </c>
       <c r="J182" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K182" t="inlineStr"/>
-      <c r="Y182" t="inlineStr"/>
-      <c r="Z182" t="inlineStr"/>
-      <c r="AA182" t="inlineStr"/>
       <c r="AB182" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -12218,26 +12179,31 @@
           <t>PolicySim: An LLM-Based Agent Social Simulation Sandbox for Proactive Policy Optimization</t>
         </is>
       </c>
-      <c r="C183" t="inlineStr"/>
-      <c r="D183" t="inlineStr"/>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Renhong Huang, Ning Tang, Jiarong Xu, Yuxuan Cao, Qingqian Tu, Sheng Guo, Bo Zheng, Huiyuan Liu, Yang Yang</t>
+        </is>
+      </c>
       <c r="E183" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="F183" t="inlineStr"/>
-      <c r="G183" t="inlineStr"/>
-      <c r="H183" t="inlineStr"/>
-      <c r="I183" t="inlineStr"/>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>cs.SI, cs.AI</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Social platforms serve as central hubs for information exchange, where user behaviors and platform interventions jointly shape opinions. However, intervention policies like recommendation and content filtering, can unintentionally amplify echo chambers and polarization, posing significant societal risks. Proactively evaluating the impact of such policies is therefore crucial. Existing approaches primarily rely on reactive online A/B testing, where risks are identified only after deployment, making risk identification delayed and costly. LLM-based social simulations offer a promising pre-deployment alternative, but current methods fall short in realistically modeling platform interventions and incorporating feedback from the platform. Bridging these gaps is essential for building actionable frameworks to assess and optimize platform policies. To this end, we propose PolicySim, an LLM-based social simulation sandbox for the proactive assessment and optimization of intervention policies. PolicySim models the bidirectional dynamics between user behavior and platform interventions through two key components: (1) a user agent module refined via supervised fine-tuning (SFT) and direct preference optimization (DPO) to achieve platform-specific behavioral realism; and (2) an adaptive intervention module that employs a contextual bandit with message passing to capture dynamic network structures. Experiments show that PolicySim can accurately simulate platform ecosystems at both micro and macro levels and support effective intervention policy.</t>
+        </is>
+      </c>
       <c r="J183" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K183" t="inlineStr"/>
-      <c r="Y183" t="inlineStr"/>
-      <c r="Z183" t="inlineStr"/>
-      <c r="AA183" t="inlineStr"/>
       <c r="AB183" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -12260,26 +12226,31 @@
           <t>Adaptive Theory of Mind for LLM-based Multi-Agent Coordination</t>
         </is>
       </c>
-      <c r="C184" t="inlineStr"/>
-      <c r="D184" t="inlineStr"/>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Chunjiang Mu, Ya Zeng, Qiaosheng Zhang, Kun Shao, Chen Chu, Hao Guo, Danyang Jia, Zhen Wang, Shuyue Hu</t>
+        </is>
+      </c>
       <c r="E184" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="F184" t="inlineStr"/>
-      <c r="G184" t="inlineStr"/>
-      <c r="H184" t="inlineStr"/>
-      <c r="I184" t="inlineStr"/>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>cs.AI</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Theory of Mind (ToM) refers to the ability to reason about others' mental states, and higher-order ToM involves considering that others also possess their own ToM. Equipping large language model (LLM)-driven agents with ToM has long been considered to improve their coordination in multiagent collaborative tasks. However, we find that misaligned ToM orders-mismatches in the depth of ToM reasoning between agents-can lead to insufficient or excessive reasoning about others, thereby impairing their coordination. To address this issue, we design an adaptive ToM (A-ToM) agent, which can align in ToM orders with its partner. Based on prior interactions, the agent estimates the partner's likely ToM order and leverages this estimation to predict the partner's action, thereby facilitating behavioral coordination. We conduct empirical evaluations on four multi-agent coordination tasks: a repeated matrix game, two grid navigation tasks and an Overcooked task. The results validate our findings on ToM alignment and demonstrate the effectiveness of our A-ToM agent. Furthermore, we discuss the generalizability of our A-ToM to non-LLM-based agents, as well as what would diminish the importance of ToM alignment.</t>
+        </is>
+      </c>
       <c r="J184" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K184" t="inlineStr"/>
-      <c r="Y184" t="inlineStr"/>
-      <c r="Z184" t="inlineStr"/>
-      <c r="AA184" t="inlineStr"/>
       <c r="AB184" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -12302,26 +12273,31 @@
           <t>Enhancing Value Alignment of LLMs with Multi-Agent System and Combinatorial Fusion</t>
         </is>
       </c>
-      <c r="C185" t="inlineStr"/>
-      <c r="D185" t="inlineStr"/>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Yuanhong Wu, Djallel Bouneffouf, D. Frank Hsu</t>
+        </is>
+      </c>
       <c r="E185" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="F185" t="inlineStr"/>
-      <c r="G185" t="inlineStr"/>
-      <c r="H185" t="inlineStr"/>
-      <c r="I185" t="inlineStr"/>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>cs.MA, cs.CL</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>Aligning large language models (LLMs) with human values is a central challenge for ensuring trustworthy and safe deployment. While existing methods such as Reinforcement Learning from Human Feedback (RLHF) and its variants have improved alignment, they often rely on a single evaluator or narrowly defined reward signals, limiting their ability to capture ethical pluralism. In this work, we propose the Value Alignment System using Combinatorial Fusion Analysis (VAS-CFA), a framework that operationalizes multi-agent fusion alignment. It instantiates multiple moral agents, each fine-tuned to represent a distinct normative perspective, and fuses their outputs using CFA with both rank- and score-based aggregation. This design leverages cognitive diversity, between agents, to mitigate conflicts and redundancies across multiple agents, producing responses that better reflect human values. Empirical evaluation demonstrates that VAS-CFA outperforms both single agent baselines and prior aggregation approaches on standard metrics, showing that multi-agent fusion provides a robust and effective mechanism for advancing value alignment in LLMs.</t>
+        </is>
+      </c>
       <c r="J185" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K185" t="inlineStr"/>
-      <c r="Y185" t="inlineStr"/>
-      <c r="Z185" t="inlineStr"/>
-      <c r="AA185" t="inlineStr"/>
       <c r="AB185" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -12344,26 +12320,31 @@
           <t>Agentic Meta-Orchestrator for Multi-Task Copilots</t>
         </is>
       </c>
-      <c r="C186" t="inlineStr"/>
-      <c r="D186" t="inlineStr"/>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Xiaofeng Zhu, Yunshen Zhou</t>
+        </is>
+      </c>
       <c r="E186" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="F186" t="inlineStr"/>
-      <c r="G186" t="inlineStr"/>
-      <c r="H186" t="inlineStr"/>
-      <c r="I186" t="inlineStr"/>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>cs.AI</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Microsoft Copilot suites serve as the universal entry point for various agents skilled in handling important tasks, ranging from assisting a customer with product purchases to detecting vulnerabilities in corporate programming code. Each agent can be powered by language models, software engineering operations, such as database retrieval, and internal \&amp; external knowledge. The repertoire of a copilot can expand dynamically with new agents. This requires a robust orchestrator that can distribute tasks from user prompts to the right agents. In this work, we propose an Agentic Meta-orchestrator (AMO) for handling multiple tasks and scalable agents in copilot services, which can provide both natural language and action responses. We will also demonstrate the planning that leverages meta-learning, i.e., a trained decision tree model for deciding the best inference strategy among various agents/models. We showcase the effectiveness of our AMO through two production use cases: Microsoft 365 (M365) E-Commerce Copilot and code compliance copilot. M365 E-Commerce Copilot advertises Microsoft products to external customers to promote sales success. The M365 E-Commerce Copilot provides up-to-date product information and connects to multiple agents, such as relational databases and human customer support. The code compliance copilot scans the internal DevOps code to detect known and new compliance issues in pull requests (PR).</t>
+        </is>
+      </c>
       <c r="J186" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="K186" t="inlineStr"/>
-      <c r="Y186" t="inlineStr"/>
-      <c r="Z186" t="inlineStr"/>
-      <c r="AA186" t="inlineStr"/>
       <c r="AB186" t="inlineStr">
         <is>
           <t>Yes</t>

</xml_diff>

<commit_message>
feat: 补齐 23 篇 markdown_full + 41 篇中文总结 (128/131, 97.7%)
- 新增 23 篇 markdown_full: S2 引用链论文通过 arxiv2md 批量转换
- 新增 41 篇中文总结: 基于 abstract 通过 MiMo API 生成
- 3 篇待补充 (arxiv2md 转换失败 + arXiv API 限流)
- Markdown: 131/131 (100%), Summary: 128/131 (97.7%)
</commit_message>
<xml_diff>
--- a/papers_record.xlsx
+++ b/papers_record.xlsx
@@ -430,7 +430,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AC186"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
@@ -10604,6 +10604,11 @@
           <t>2025</t>
         </is>
       </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>本文提出Mem0——一种可扩展的记忆中心架构，用于构建具备长期记忆能力的AI智能体。它通过从对话中动态提取、整合与检索关键信息，解决了大语言模型在长期多轮对话中记忆不足的问题。进一步引入的图记忆变体能捕捉对话元素间的复杂关系。在LOCOMO基准测试中，Mem0在单跳、时序、多跳和开放域问题上均优于六类基线系统，相比OpenAI模型得分提升26%，图记忆版本在基础配置上再提升约2%，展现出显著的技术优势。</t>
+        </is>
+      </c>
       <c r="J143" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -10646,6 +10651,11 @@
           <t>Large Language Model (LLM) agents are transforming education by automating complex pedagogical tasks and enhancing both teaching and learning processes. In this survey, we present a systematic review of recent advances in applying LLM agents to address key challenges in educational settings, such as feedback comment generation, curriculum design, etc. We analyze the technologies enabling these agents, including representative datasets, benchmarks, and algorithmic frameworks. Additionally, we highlight key challenges in deploying LLM agents in educational settings, including ethical issues, hallucination and overreliance, and integration with existing educational ecosystems. Beyond the core technical focus, we include in Appendix A a comprehensive overview of domain-specific educational agents, covering areas such as science learning, language learning, and professional development.</t>
         </is>
       </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>本文系统综述了大语言模型智能体在教育领域的应用进展，重点分析了其在自动化教学反馈、课程设计等任务中的作用。研究梳理了支撑这些智能体的关键技术，包括相关数据集、基准测试与算法框架，同时探讨了实际部署中面临的伦理风险、幻觉问题及教育生态整合等挑战。附录部分还概述了科学学习、语言教学等细分领域的专用智能体，为教育智能化提供了全面的技术路径参考。</t>
+        </is>
+      </c>
       <c r="J144" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -10678,6 +10688,11 @@
           <t>2025</t>
         </is>
       </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>本文首次系统总结了将终身学习融入大语言模型（LLM）智能体的技术路线。针对现有LLM智能体缺乏长期适应能力的问题，文章提出将智能体核心组件分为三大模块：负责多模态输入整合的感知模块、用于存储演化知识的记忆模块，以及实现与环境交互的动作模块。这些支柱共同支持智能体持续适应动态环境、缓解灾难性遗忘问题，从而提升长期性能，为开发具备终身学习能力的LLM智能体提供了研究路线图。</t>
+        </is>
+      </c>
       <c r="J145" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -10720,6 +10735,11 @@
           <t>Large Language Model (LLM) agents have become increasingly prevalent across various real-world applications. They enhance decision-making by storing private user-agent interactions in the memory module for demonstrations, introducing new privacy risks for LLM agents. In this work, we systematically investigate the vulnerability of LLM agents to our proposed Memory EXTRaction Attack (MEXTRA) under a black-box setting. To extract private information from memory, we propose an effective attacking prompt design and an automated prompt generation method based on different levels of knowledge about the LLM agent. Experiments on two representative agents demonstrate the effectiveness of MEXTRA. Moreover, we explore key factors influencing memory leakage from both the agent designer's and the attacker's perspectives. Our findings highlight the urgent need for effective memory safeguards in LLM agent design and deployment.</t>
         </is>
       </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>本文系统研究了大语言模型智能体在黑盒环境下面临的隐私漏洞，提出并验证了记忆提取攻击MEXTRA的有效性。研究通过精心设计的攻击提示，能够从智能体记忆模块中成功提取私密用户交互数据，并从设计者与攻击者双视角揭示了影响记忆泄露的关键因素。这一发现凸显了当前LLM智能体在记忆安全防护方面的紧迫需求。</t>
+        </is>
+      </c>
       <c r="J146" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -10762,6 +10782,11 @@
           <t>To deliver coherent and personalized experiences in long-term conversations, existing approaches typically perform retrieval augmented response generation by constructing memory banks from conversation history at either the turn-level, session-level, or through summarization techniques.In this paper, we present two key findings: (1) The granularity of memory unit matters: turn-level, session-level, and summarization-based methods each exhibit limitations in both memory retrieval accuracy and the semantic quality of the retrieved content. (2) Prompt compression methods, such as LLMLingua-2, can effectively serve as a denoising mechanism, enhancing memory retrieval accuracy across different granularities. Building on these insights, we propose SeCom, a method that constructs the memory bank at segment level by introducing a conversation segmentation model that partitions long-term conversations into topically coherent segments, while applying compression based denoising on memory units t</t>
         </is>
       </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>本文聚焦个性化对话代理的记忆构建与检索，指出现有基于轮次、会话或摘要的记忆方法存在检索精度与语义质量不足的问题。研究发现，记忆单元粒度设计至关重要，而提示压缩技术（如LLMLingua-2）可作为去噪机制提升跨粒度检索准确性。据此，本文提出SeCom方法：通过对话分割模型将长期对话划分为主题连贯的段落单元，并结合压缩去噪策略，以更有效地构建与检索对话记忆，从而提升长期交互的连贯性与</t>
+        </is>
+      </c>
       <c r="J147" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -10794,6 +10819,11 @@
           <t>2025</t>
         </is>
       </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>针对大语言模型因固定上下文窗口和记忆管理不足导致的长期记忆能力与个性化体验局限，本文创新提出MemoryOS记忆操作系统。该系统借鉴操作系统记忆管理原理，构建了包含短期、中期、长期个人记忆的三级分层存储架构，通过对话链动态更新与分页存储策略实现记忆的自动流转与整合。在LoCoMo基准测试中，其F1和BLEU-1分数较基线平均提升49.11%和46.18%，显著增强了长对话的上下文连贯性与个性化记忆保留能力，代码已</t>
+        </is>
+      </c>
       <c r="J148" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -10826,6 +10856,11 @@
           <t>2025</t>
         </is>
       </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>本文系统梳理了多轮对话场景下基于大语言模型（LLM）智能体的评估方法。通过对近250篇文献的PRISMA框架分析，研究构建了两个关联分类体系：其一界定评估维度（涵盖任务完成度、回复质量、用户体验、上下文保持及规划与工具整合能力）；其二归纳评估方法（包括人工标注、自动化指标、人机混合策略及LLM自评机制）。该框架不仅整合了BLEU、ROUGE等传统指标，更创新性地纳入了适用于动态交互场景的评估技术，为突破传统评估局限提供了系统性解决方案。</t>
+        </is>
+      </c>
       <c r="J149" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -10890,6 +10925,11 @@
           <t>2025</t>
         </is>
       </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>随着基于大语言模型的多智能体系统在复杂任务中的广泛应用，其面临的对抗攻击、错误传播等安全问题日益凸显。为此，本文提出G-Safeguard——一种基于拓扑结构的安全防护框架，利用图神经网络在多智能体交互图中检测异常行为，并通过拓扑干预实现攻击修复。实验表明，该方法能有效抵御各类攻击，在提示注入攻击中恢复超过40%的性能，且具备良好的跨模型适配性与可扩展性，可与主流多智能体系统无缝集成。代码已开源。</t>
+        </is>
+      </c>
       <c r="J151" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -10922,6 +10962,11 @@
           <t>2025</t>
         </is>
       </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>近期研究凸显了记忆机制对LLM智能体的重要性，使其能存储信息并适应动态环境。然而，现有评估存在记忆层次单一、交互场景有限且缺乏多维度指标等问题。为此，本文构建了更全面的数据集，涵盖事实记忆与反思记忆两个层次，并引入参与和观察两种交互场景。在此基础上，我们提出名为MemBench的基准，从效果、效率和容量等多维度评估LLM智能体的记忆能力，相关数据集与项目已开源。</t>
+        </is>
+      </c>
       <c r="J152" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -10954,6 +10999,11 @@
           <t>2025</t>
         </is>
       </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>本文对大语言模型（LLM）智能体的优化方法进行了系统性梳理与总结。随着LLM的快速发展，基于LLM的智能体已成为自主决策与交互任务的关键，但现有依赖提示设计或简单微调的方法在复杂场景中效果有限。文章将优化方法分为参数驱动型（包括微调、强化学习及混合策略，并深入探讨了轨迹数据构建、奖励函数设计等关键环节）与无参数型（通过提示工程与外部知识检索优化行为）两类，综述了相关评估体系、核心应用，并讨论了挑战与未来方向。</t>
+        </is>
+      </c>
       <c r="J153" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11001,6 +11051,11 @@
           <t>Long-term memory is one of the key factors influencing the reasoning capabilities of Large Language Model Agents (LLM Agents). Incorporating a memory mechanism that effectively integrates past interactions can significantly enhance decision-making and contextual coherence of LLM Agents. While recent works have made progress in memory storage and retrieval, such as encoding memory into dense vectors for similarity-based search or organizing knowledge in the form of graph, these approaches often fall short in structured memory organization and efficient retrieval. To address these limitations, we propose a Hierarchical Memory (H-MEM) architecture for LLM Agents that organizes and updates memory in a multi-level fashion based on the degree of semantic abstraction. Each memory vector is embedded with a positional index encoding pointing to its semantically related sub-memories in the next layer. During the reasoning phase, an index-based routing mechanism enables efficient, layer-by-layer retrieval without performing exhaustive similarity computations. We evaluate our method on five task settings from the LoCoMo dataset. Experimental results show that our approach consistently outperforms five baseline methods, demonstrating its effectiveness in long-term dialogue scenarios.</t>
         </is>
       </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>大语言模型智能体（LLM Agents）的长期推理能力关键之一在于长期记忆。现有记忆方法，如基于密集向量的相似性搜索或知识图谱，在结构化组织和高效检索上存在不足。为此，本文提出一种**分层记忆（H-MEM）架构**，它根据**语义抽象程度**以多层级方式组织和更新记忆。每个记忆向量均嵌入**位置索引编码**，以指向其下一层级相关的子记忆。在推理阶段，基于索引的路由机制能够实现高效的**逐层检索**，避免了耗时的全局相似性计算。在LoCoMo数据集的五个任务设置上的实验表明，本方法</t>
+        </is>
+      </c>
       <c r="J154" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11080,6 +11135,11 @@
           <t>Personalization has become an essential capability in modern AI systems, enabling customized interactions that align with individual user preferences, contexts, and goals. Recent research has increasingly concentrated on Retrieval-Augmented Generation (RAG) frameworks and their evolution into more advanced agent-based architectures within personalized settings to enhance user satisfaction. Building on this foundation, this survey systematically examines personalization across the three core stages of RAG: pre-retrieval, retrieval, and generation. Beyond RAG, we further extend its capabilities into the realm of Personalized LLM-based Agents, which enhance traditional RAG systems with agentic functionalities, including user understanding, personalized planning and execution, and dynamic generation. For both personalization in RAG and agent-based personalization, we provide formal definitions, conduct a comprehensive review of recent literature, and summarize key datasets and evaluation metrics. Additionally, we discuss fundamental challenges, limitations, and promising research directions in this evolving field. Relevant papers and resources are continuously updated at https://github.com/Applied-Machine-Learning-Lab/Awesome-Personalized-RAG-Agent.</t>
         </is>
       </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>个性化是现代AI系统的重要能力，本综述聚焦于检索增强生成（RAG）框架及其向个性化智能体架构的演进。文章系统梳理了RAG在预检索、检索和生成三个阶段的个性化方法，并进一步扩展至基于大语言模型的个性化智能体，通过用户理解、个性化规划执行及动态生成等增强功能提升传统RAG系统。文中对相关研究提供了形式化定义、文献综述及关键数据集与评估指标，同时探讨了该领域的核心挑战与未来方向。相关资源持续更新于GitHub。</t>
+        </is>
+      </c>
       <c r="J156" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11112,6 +11172,11 @@
           <t>2025</t>
         </is>
       </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>当前智能体（Agentic AI）研究缺乏标准化与科学严谨性，导致不同方法难以公平比较。本文基于GAIA基准和BrowseComp进行系统实证研究，发现评估协议的不稳定性使得先前研究（包括开源项目）难以复现，运行方差显著。为此，作者提出更稳健的评估协议以稳定比较过程。研究揭示了关键组件与设计对构建高效智能体的重要性，并剔除了看似合理但实际冗余的部分。基于这些发现，作者</t>
+        </is>
+      </c>
       <c r="J157" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11144,6 +11209,11 @@
           <t>2025</t>
         </is>
       </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>随着模型上下文协议（MCP）逐步成为增强智能体与工具集成的关键开放标准，如何真实评估其环境下的智能体性能成为重要课题。为此，我们提出了MCP-AgentBench评估框架，其核心贡献包括：构建了包含33个运行服务器和188个工具的MCP测试平台；设计了涵盖6类交互复杂度的600个系统查询；并创新性地引入了以任务成功为导向的MCP-Eval评估方法。该框架旨在为学术</t>
+        </is>
+      </c>
       <c r="J158" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11176,6 +11246,11 @@
           <t>2025</t>
         </is>
       </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>针对大语言模型智能体在跨域推荐中存在的记忆冗余和群体影响感知不足的问题，本文提出AgentCF++模型。该模型采用双层记忆架构与两步融合机制，有效过滤跨域决策中的无关信息；并创新性地引入兴趣群组与群组共享记忆，以捕捉流行度因素对相似兴趣用户群体的影响，从而提升推荐效果。实验验证了该方法的有效性。</t>
+        </is>
+      </c>
       <c r="J159" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11208,6 +11283,11 @@
           <t>2025</t>
         </is>
       </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>本文提出了一种基于群体智能体的综合社交网络模拟系统（GA-S3）。该系统通过设计代表相似行为个体集合的群体智能体，对大规模在线事件进行智能决策建模，以可控计算成本模拟复杂交互下的网络现象。研究构建了2024年在线事件基准数据集，包含精细流量变化信息，实验表明该系统能实现准确、高度逼真的预测结果。相关</t>
+        </is>
+      </c>
       <c r="J160" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11272,6 +11352,11 @@
           <t>2025</t>
         </is>
       </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>敏捷开发中的工作量估算依赖主观评估，易产生偏差且缺乏可解释性。本研究提出一种基于大语言模型的多智能体框架，突破性地使系统能与人类开发者协调讨论、达成共识，并自主生成估算结果。在实际数据集评估中，该框架多项指标优于现有技术，且实践反馈表明与智能体协作能显著提升估算效率与一致性。</t>
+        </is>
+      </c>
       <c r="J162" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11304,6 +11389,11 @@
           <t>2025</t>
         </is>
       </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>语言模型代理正成为人们在线活动的核心中介，若其控制权落入现有互联网巨头或新兴竞争企业手中，形成的平台型代理可能加剧用户监控、强化平台锁定效应并巩固行业垄断。为此，本文提出应构建“代理倡导者”——即由用户自主控制、保障个体选择权的智能代理。实现这一目标需满足三个条件：开放非平台所有的计算资源与高性能模型、建立开放的互操作性与安全标准，并通过市场监管防止平台扼杀竞争。</t>
+        </is>
+      </c>
       <c r="J163" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11336,6 +11426,11 @@
           <t>2025</t>
         </is>
       </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>本文探索将大语言模型驱动的自主网页智能体（AWA）改造为自主测试智能体（ATA）的可行性，旨在降低自动化测试中脚本维护成本。研究贡献包括：构建了包含三个离线网页应用和113个测试用例的评测基准；开发了SeeAct-ATA与PinATA两个开源实现；通过量化实验证明，PinATA在测试执行效果上比SeeAct-ATA提升50%，但仍存在局限性。研究表明，基于自然语言指令的ATA为自动化测试提供了潜在新方向。</t>
+        </is>
+      </c>
       <c r="J164" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11368,6 +11463,11 @@
           <t>2025</t>
         </is>
       </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>针对现有基准难以体现现实世界数学建模问题复杂性的不足，本文提出了ModelingBench，一个涵盖城市交通优化、生态规划等跨领域的开放式建模基准。基于此，我们设计了多智能体框架ModelingAgent，通过协调工具使用、支持结构化工作流及迭代自优化，生成合理且创新的解决方案。此外，引入结合领域专家视角的ModelingJudge评估系统。实验表明，ModelingAgent显著优于基线方法，其产出常与人类专家方案难以区分，为开放式现实问题求解提供了完整框架。</t>
+        </is>
+      </c>
       <c r="J165" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11400,6 +11500,11 @@
           <t>2025</t>
         </is>
       </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>随着大语言模型（LLM）在推荐系统中用于个性化建模的普及，其依赖的内存机制虽能实现自主探索与学习，却也构成了潜在的安全漏洞。现有研究对动态内存状态的安全性探索不足，尤其在商业推荐系统的黑盒特性下更具挑战。为此，本文首次系统揭示了LLM推荐系统中基于内存的安全缺陷，并提出了名为DrunkAgent的新型黑盒攻击框架。该框架通过生成语义对抗触发器，在交互过程中篡改内存更新，以提升目标物品的推荐排名，从而暴露出当前系统的脆弱性并为增强其安全性提供了研究方向。</t>
+        </is>
+      </c>
       <c r="J166" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11447,6 +11552,11 @@
           <t>Every individual carries a unique and personal life story shaped by their memories and experiences. However, these memories are often scattered and difficult to organize into a coherent narrative, a challenge that defines the task of autobiography writing. Existing conversational writing assistants tend to rely on generic user interactions and pre-defined guidelines, making it difficult for these systems to capture personal memories and develop a complete biography over time. We introduce StorySage, a user-driven software system designed to meet the needs of a diverse group of users that supports a flexible conversation and a structured approach to autobiography writing. Powered by a multi-agent framework composed of an Interviewer, Session Scribe, Planner, Section Writer, and Session Coordinator, our system iteratively collects user memories, updates their autobiography, and plans for future conversations. In experimental simulations, StorySage demonstrates its ability to navigate multiple sessions and capture user memories across many conversations. User studies (N=28) highlight how StorySage maintains improved conversational flow, narrative completeness, and higher user satisfaction when compared to a baseline. In summary, StorySage contributes both a novel architecture for autobiography writing and insights into how multi-agent systems can enhance human-AI creative partnerships.</t>
         </is>
       </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>针对个人记忆分散难以系统化撰写自传的问题，我们提出了基于多智能体框架的对话式自传写作系统StorySage。该系统通过协调采访、记录、规划、写作等多个智能体，以用户为主导进行渐进式对话，动态采集记忆并构建叙事框架。实验与用户研究（N=28）表明，相较于基线系统，StorySage显著提升了对话流畅性、叙事完整性和用户满意度，为多智能体增强人机创意协作提供了新架构与实践见解。</t>
+        </is>
+      </c>
       <c r="J167" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11494,6 +11604,11 @@
           <t>Intelligent control of Unmanned Aerial Vehicles (UAVs) swarms has emerged as a critical research focus, and it typically requires the swarm to navigate effectively while avoiding obstacles and achieving continuous coverage over multiple mission targets. Although traditional Multi-Agent Reinforcement Learning (MARL) approaches offer dynamic adaptability, they are hindered by the semantic gap in numerical communication and the rigidity of homogeneous role structures, resulting in poor generalization and limited task scalability. Recent advances in Large Language Model (LLM)-based control frameworks demonstrate strong semantic reasoning capabilities by leveraging extensive prior knowledge. However, due to the lack of online learning and over-reliance on static priors, these works often struggle with effective exploration, leading to reduced individual potential and overall system performance. To address these limitations, we propose a Role-Adaptive LLM-Driven Yoked navigation algorithm RALLY. Specifically, we first develop an LLM-driven semantic decision framework that uses structured natural language for efficient semantic communication and collaborative reasoning. Afterward, we introduce a dynamic role-heterogeneity mechanism for adaptive role switching and personalized decision-making. Furthermore, we propose a Role-value Mixing Network (RMIX)-based assignment strategy that integrates LLM offline priors with MARL online policies to enable semi-offline training of role selection strategies. Experiments in the Multi-Agent Particle Environment (MPE) environment and a Software-In-The-Loop (SITL) platform demonstrate that RALLY outperforms conventional approaches in terms of task coverage, convergence speed, and generalization, highlighting its strong potential for collaborative navigation in agentic multi-UAV systems.</t>
         </is>
       </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>针对智能体无人机集群协同导航中传统多智能体强化学习方法存在的通信语义缺失、角色同质化问题，本文提出一种角色自适应的LLM驱动协同导航算法RALLY。该算法通过LLM驱动的语义决策框架实现高效语义通信与协同推理，并引入动态角色异质性机制支持自适应角色切换与个性化决策。进一步，基于角色值混合网络的策略整合了LLM离线先验与在线策略，实现角色选择策略的半离线训练。实验表明，RALLY在任务覆盖、收敛速度和泛化性上均优于传统方法，为多无人机系统协作</t>
+        </is>
+      </c>
       <c r="J168" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11541,6 +11656,11 @@
           <t>Large language models deployed as autonomous agents face critical memory limitations, lacking selective forgetting mechanisms that lead to either catastrophic forgetting at context boundaries or information overload within them. While human memory naturally balances retention and forgetting through adaptive decay processes, current AI systems employ binary retention strategies that preserve everything or lose it entirely. We propose FadeMem, a biologically-inspired agent memory architecture that incorporates active forgetting mechanisms mirroring human cognitive efficiency. FadeMem implements differential decay rates across a dual-layer memory hierarchy, where retention is governed by adaptive exponential decay functions modulated by semantic relevance, access frequency, and temporal patterns. Through LLM-guided conflict resolution and intelligent memory fusion, our system consolidates related information while allowing irrelevant details to fade. Experiments on Multi-Session Chat, LoCoMo, and LTI-Bench demonstrate superior multi-hop reasoning and retrieval with 45\% storage reduction, validating the effectiveness of biologically-inspired forgetting in agent memory systems.</t>
         </is>
       </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>针对大语言模型作为智能体时面临的选择性遗忘机制缺失问题，本文提出受生物记忆启发的FadeMem架构。该系统通过双层记忆层次结构中的差异化自适应衰减机制，依据信息语义相关性、访问频率及时间模式动态调整保留强度，并结合大语言模型引导的冲突解决与记忆融合策略，实现相关记忆的整合与无关信息的渐进遗忘。在Multi-Session Chat等基准测试中，FadeMem在降低45%存储开销的同时，显著提升了多跳推理与检索性能，验证了仿生遗忘机制在智能体记忆系统中的有效性。</t>
+        </is>
+      </c>
       <c r="J169" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11588,6 +11708,11 @@
           <t>Agentic memory is emerging as a key enabler for large language models (LLM) to maintain continuity, personalization, and long-term context in extended user interactions, critical capabilities for deploying LLMs as truly interactive and adaptive agents. Agentic memory refers to the memory that provides an LLM with agent-like persistence: the ability to retain and act upon information across conversations, similar to how a human would. We present Memoria, a modular memory framework that augments LLM-based conversational systems with persistent, interpretable, and context-rich memory. Memoria integrates two complementary components: dynamic session-level summarization and a weighted knowledge graph (KG)-based user modelling engine that incrementally captures user traits, preferences, and behavioral patterns as structured entities and relationships. This hybrid architecture enables both short-term dialogue coherence and long-term personalization while operating within the token constraints of modern LLMs. We demonstrate how Memoria enables scalable, personalized conversational artificial intelligence (AI) by bridging the gap between stateless LLM interfaces and agentic memory systems, offering a practical solution for industry applications requiring adaptive and evolving user experiences.</t>
         </is>
       </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>智能体记忆是大语言模型在长对话中维持连续性与个性化能力的关键，Memoria框架正为此设计。它通过结合动态会话摘要与加权知识图谱两种机制，使模型能持续捕捉用户特征、偏好与行为模式，形成结构化记忆。这一混合架构在保障短期对话流畅的同时，也实现了长期个性化适应，为无状态的大语言模型提供了可扩展的智能体记忆解决方案，适用于需要持续学习与自适应交互的实际应用场景。</t>
+        </is>
+      </c>
       <c r="J170" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11635,6 +11760,11 @@
           <t>We present Sari Sandbox, a high-fidelity, photorealistic 3D retail store simulation for benchmarking embodied agents against human performance in shopping tasks. Addressing a gap in retail-specific sim environments for embodied agent training, Sari Sandbox features over 250 interactive grocery items across three store configurations, controlled via an API. It supports both virtual reality (VR) for human interaction and a vision language model (VLM)-powered embodied agent. We also introduce SariBench, a dataset of annotated human demonstrations across varied task difficulties. Our sandbox enables embodied agents to navigate, inspect, and manipulate retail items, providing baselines against human performance. We conclude with benchmarks, performance analysis, and recommendations for enhancing realism and scalability. The source code can be accessed via https://github.com/upeee/sari-sandbox-env.</t>
         </is>
       </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>本文介绍Sari Sandbox，一个高保真照片级真实感的3D零售店仿真环境，用于对具身智能体在购物任务中的表现进行基准测试与人类对比。该环境填补了零售领域专用仿真平台的空白，包含超过250种可交互商品和三种店铺配置，同时支持虚拟现实人类交互与基于视觉语言模型的智能体操作。研究还推出了包含不同难度人类演示的SariBench数据集，为智能体提供导航、商品检查与操控的基准性能分析，并提出了提升真实性与可扩展性的建议。项目代码已开源。</t>
+        </is>
+      </c>
       <c r="J171" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11682,6 +11812,11 @@
           <t>Multi-Agent Systems (MAS) are increasingly used to simulate social interactions, but most of the frameworks miss the underlying cognitive complexity of human behavior. In this paper, we introduce Trans-ACT (Transactional Analysis Cognitive Toolkit), an approach embedding Transactional Analysis (TA) principles into MAS to generate agents with realistic psychological dynamics. Trans-ACT integrates the Parent, Adult, and Child ego states into an agent's cognitive architecture. Each ego state retrieves context-specific memories and uses them to shape response to new situations. The final answer is chosen according to the underlying life script of the agent. Our experimental simulation, which reproduces the Stupid game scenario, demonstrates that agents grounded in cognitive and TA principles produce deeper and context-aware interactions. Looking ahead, our research opens a new way for a variety of applications, including conflict resolution, educational support, and advanced social psychology studies.</t>
         </is>
       </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>多智能体系统（MAS）在模拟社会互动方面日益重要，但现有框架多忽视人类行为背后的心理复杂性。本文提出Trans-ACT认知工具箱，将交易分析（TA）原则嵌入MAS，构建具有真实心理动态的智能体。该方法在智能体认知架构中整合“父母-成人-儿童”自我状态，各状态调用特定情境记忆塑造反应，并依据内在生命脚本生成最终回应。实验通过复现经典交互游戏场景验证表明，基于认知与TA原则的智能体产生了更深入、语境感知更强的互动。这项研究为冲突调解、教育支持及高级社会心理学研究开辟了新的应用路径。</t>
+        </is>
+      </c>
       <c r="J172" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11729,6 +11864,11 @@
           <t>TRIZ, the Theory of Inventive Problem Solving, is a structured, knowledge-based framework for innovation and abstracting problems to find inventive solutions. However, its application is often limited by the complexity and deep interdisciplinary knowledge required. Advancements in Large Language Models (LLMs) have revealed new possibilities for automating parts of this process. While previous studies have explored single LLMs in TRIZ applications, this paper introduces a multi-agent approach. We propose an LLM-based multi-agent system, called TRIZ agents, each with specialized capabilities and tool access, collaboratively solving inventive problems based on the TRIZ methodology. This multi-agent system leverages agents with various domain expertise to efficiently navigate TRIZ steps. The aim is to model and simulate an inventive process with language agents. We assess the effectiveness of this team of agents in addressing complex innovation challenges based on a selected case study in engineering. We demonstrate the potential of agent collaboration to produce diverse, inventive solutions. This research contributes to the future of AI-driven innovation, showcasing the advantages of decentralized problem-solving in complex ideation tasks.</t>
         </is>
       </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>本文针对TRIZ创新方法论应用门槛高、依赖跨学科知识的问题，提出一种基于大型语言模型的多智能体系统（TRIZ Agents）。该系统通过具备不同领域专长的智能体协作，分工执行TRIZ方法步骤，以模拟并优化发明问题解决过程。研究通过工程案例验证表明，这种多智能体协作模式能够有效生成多样化创新方案，为人工智能驱动的创新研究与分布式协作求解复杂问题提供了新路径。</t>
+        </is>
+      </c>
       <c r="J173" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11776,6 +11916,11 @@
           <t>Large language models (LLMs) offer new opportunities for interacting with complex software artifacts, such as software models, through natural language. They present especially promising benefits for large software models that are difficult to grasp in their entirety, making traditional interaction and analysis approaches challenging. This paper investigates two approaches for leveraging LLMs to answer questions over software models: direct prompting, where the whole software model is provided in the context, and an agentic approach combining LLM-based agents with general-purpose file access tools. We evaluate these approaches using an Ecore metamodel designed for timing analysis and software optimization in automotive and embedded domains. Our findings show that while the agentic approach achieves accuracy comparable to direct prompting, it is significantly more efficient in terms of token usage. This efficiency makes the agentic approach particularly suitable for the automotive industry, where the large size of software models makes direct prompting infeasible, establishing LLM agents as not just a practical alternative but the only viable solution. Notably, the evaluation was conducted using small LLMs, which are more feasible to be executed locally - an essential advantage for meeting strict requirements around privacy, intellectual property protection, and regulatory compliance. Future work will investigate software models in diverse formats, explore more complex agent architectures, and extend agentic workflows to support not only querying but also modification of software models.</t>
         </is>
       </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>本研究探讨利用大语言模型查询大型汽车软件模型的两种方法：直推提示与智能体方法。直推提示将整个模型置于上下文中，而智能体方法则结合LLM智能体与通用文件访问工具。基于汽车领域时序分析用的Ecore元模型评估显示，两种方法准确性相当，但智能体方法在token消耗上显著更高效。对于汽车行业中体量庞大的软件模型，直推提示往往不可行，智能体方法因而成为唯一可行方案。评估采用可在本地运行的小规模LLM，有利于满足隐私与合规要求。未来将探索更多模型格式、复杂智能体架构，并扩展至模型修改场景。</t>
+        </is>
+      </c>
       <c r="J174" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11823,6 +11968,11 @@
           <t>Multi-agent techniques such as role playing or multi-turn debates have been shown to be effective in improving the performance of large language models (LLMs) in downstream tasks. Despite their differences in workflows, existing multi-agent systems constructed from a single base LLM mostly use natural language for agent communication. While this is appealing for its simplicity and interpretability, it also introduces inevitable information loss as one model must down sample its continuous state vectors to discrete tokens before transferring them to the other model. Such losses are particularly significant when the information to transfer is not simple facts, but reasoning logics or abstractive thoughts. To tackle this problem, we propose a new communication protocol that transfers both natural language tokens and token-wise state transition trajectory from one agent to another. Particularly, compared to the actual state value, we find that the sequence of state changes in LLMs after generating each token can better reflect the information hidden behind the inference process. We propose a State Delta Encoding (SDE) method to represent state transition trajectories. The experimental results show that multi-agent systems with SDE achieve SOTA performance compared to other communication protocols, particularly in tasks that involve complex reasoning.</t>
         </is>
       </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>当前多智能体系统主要通过自然语言进行通信，但这种方式在传递推理逻辑时存在信息损耗。为此，本文提出“状态差分轨迹”通信协议，使智能体间除了传递文本标记外，还能共享由“状态差分编码”方法生成的逐token状态变化序列。该序列能更准确地反映模型推理过程中的隐含信息。实验表明，采用该协议的多智能体系统在复杂推理任务上显著优于现有方法，取得了</t>
+        </is>
+      </c>
       <c r="J175" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11870,6 +12020,11 @@
           <t>Agent-assisted memory recall is one critical research problem in the field of human-computer interaction. In conventional methods, the agent can retrieve information from its equipped memory module to help the person recall incomplete or vague memories. The limited size of memory module hinders the acquisition of complete memories and impacts the memory recall performance in practice. Memory theories suggest that the person's relevant memory can be proactively activated through some effective cues. Inspired by this, we propose a novel strategy-guided agent-assisted memory recall method, allowing the agent to transform an original query into a cue-rich one via the judiciously designed strategy to help the person recall memories. To this end, there are two key challenges. (1) How to choose the appropriate recall strategy for diverse forgetting scenarios with distinct memory-recall characteristics? (2) How to obtain the high-quality responses leveraging recall strategies, given only abstract and sparsely annotated strategy patterns? To address the challenges, we propose a Recall Router framework. Specifically, we design a 5W Recall Map to classify memory queries into five typical scenarios and define fifteen recall strategy patterns across the corresponding scenarios. We then propose a hierarchical recall tree combined with the Monte Carlo Tree Search algorithm to optimize the selection of strategy and the generation of strategy responses. We construct an instruction tuning dataset and fine-tune multiple open-source large language models (LLMs) to develop MemoCue, an agent that excels in providing memory-inspired responses. Experiments on three representative datasets show that MemoCue surpasses LLM-based methods by 17.74% in recall inspiration. Further human evaluation highlights its advantages in memory-recall applications.</t>
         </is>
       </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>针对大语言模型代理辅助人类记忆回忆的场景，传统方法受限于存储模块规模，难以完整激活相关记忆。本文提出策略引导的MemoCue方法，核心是将用户原始查询转化为富含线索的提示以促进回忆。研究构建“5W回忆地图”将记忆场景分类并定义对应策略模式，结合蒙特卡洛树搜索优化策略选择与回应生成。基于指令微调数据集训练的开源大语言模型代理，在三个数据集上的回忆启发效果相比基线提升17.74%，并在人工评估中展现出实际应用优势。</t>
+        </is>
+      </c>
       <c r="J176" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11917,6 +12072,11 @@
           <t>Large language models (LLMs) have shown strong performance on standardized social science instruments, but their value for product discovery remains unclear. We investigate whether interview-informed generative agents can simulate user responses in concept testing scenarios. Using in-depth workflow interviews with knowledge workers, we created personalized agents and compared their evaluations of novel AI concepts against the same participants' responses. Our results show that agents are distribution-calibrated but identity-imprecise: they fail to replicate the specific individual they are grounded in, yet approximate population-level response distributions. These findings highlight both the potential and the limits of LLM simulation in design research. While unsuitable as a substitute for individual-level insights, simulation may provide value for early-stage concept screening and iteration, where distributional accuracy suffices. We discuss implications for integrating simulation responsibly into product development workflows.</t>
         </is>
       </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>该研究探索了访谈知情生成代理在概念测试中模拟用户反馈的有效性。通过对知识工作者进行深度工作流访谈，研究构建了个性化大语言模型代理，并将其对新AI概念的评估与参与者实际反馈对比。结果发现，代理能近似呈现群体层面的响应分布，却难以复刻特定个体的特征。这表明大语言模型模拟可用于产品早期的概念筛选与迭代，但不应替代个体层次的深度洞察，研究为负责任地将模拟融入产品开发流程提供了参考。</t>
+        </is>
+      </c>
       <c r="J177" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -11964,6 +12124,11 @@
           <t>Augmented Reality (AR) systems are increasingly integrating foundation models, such as Multimodal Large Language Models (MLLMs), to provide more context-aware and adaptive user experiences. This integration has led to the development of AR agents to support intelligent, goal-directed interactions in real-world environments. While current AR agents effectively support immediate tasks, they struggle with complex multi-step scenarios that require understanding and leveraging user's long-term experiences and preferences. This limitation stems from their inability to capture, retain, and reason over historical user interactions in spatiotemporal contexts. To address these challenges, we propose a conceptual framework for memory-augmented AR agents that can provide personalized task assistance by learning from and adapting to user-specific experiences over time. Our framework consists of four interconnected modules: (1) Perception Module for multimodal sensor processing, (2) Memory Module for persistent spatiotemporal experience storage, (3) Spatiotemporal Reasoning Module for synthesizing past and present contexts, and (4) Actuator Module for effective AR communication. We further present an implementation roadmap, a future evaluation strategy, a potential target application and use cases to demonstrate the practical applicability of our framework across diverse domains. We aim for this work to motivate future research toward developing more intelligent AR systems that can effectively bridge user's interaction history with adaptive, context-aware task assistance.</t>
         </is>
       </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>当前AR系统结合多模态大语言模型后，能支持即时任务，但在需要理解用户长期经验和偏好的复杂多步骤场景中表现不足，这源于其缺乏在时空背景下对历史交互进行捕捉、保留和推理的能力</t>
+        </is>
+      </c>
       <c r="J178" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -12011,6 +12176,11 @@
           <t>Large Language Model (LLM)-based agents that plan, use tools and act has begun to shape healthcare and medicine. Reported studies demonstrate competence on various tasks ranging from EHR analysis and differential diagnosis to treatment planning and research workflows. Yet the literature largely consists of overviews which are either broad surveys or narrow dives into a single capability (e.g., memory, planning, reasoning), leaving healthcare work without a common frame. We address this by reviewing 49 studies using a seven-dimensional taxonomy: Cognitive Capabilities, Knowledge Management, Interaction Patterns, Adaptation &amp; Learning, Safety &amp; Ethics, Framework Typology and Core Tasks &amp; Subtasks with 29 operational sub-dimensions. Using explicit inclusion and exclusion criteria and a labeling rubric (Fully Implemented, Partially Implemented, Not Implemented), we map each study to the taxonomy and report quantitative summaries of capability prevalence and co-occurrence patterns. Our empirical analysis surfaces clear asymmetries. For instance, the External Knowledge Integration sub-dimension under Knowledge Management is commonly realized (~76% Fully Implemented) whereas Event-Triggered Activation sub-dimenison under Interaction Patterns is largely absent (~92% Not Implemented) and Drift Detection &amp; Mitigation sub-dimension under Adaptation &amp; Learning is rare (~98% Not Implemented). Architecturally, Multi-Agent Design sub-dimension under Framework Typology is the dominant pattern (~82% Fully Implemented) while orchestration layers remain mostly partial. Across Core Tasks &amp; Subtasks, information centric capabilities lead e.g., Medical Question Answering &amp; Decision Support and Benchmarking &amp; Simulation, while action and discovery oriented areas such as Treatment Planning &amp; Prescription still show substantial gaps (~59% Not Implemented).</t>
         </is>
       </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>当前，基于大语言模型（LLM）的智能体在医疗领域的应用正在兴起，但缺乏统一的评估框架。本研究针对这一空白，系统综述了49项相关研究，创新性地提出了一个包含七大维度、29个操作子维度的分类框架，对智能体的能力进行实证分析。研究发现，智能体的能力发展呈现明显不对称性：在“外部知识整合”方面实现度较高，而“事件触发激活”与“漂移检测与缓解”等功能普遍缺失；架构上“多智能体设计”虽为主流，但协同层仍不完善；在核心任务中，信息处理类任务表现突出，而治疗规划等行动导向型任务仍存在显著差距。</t>
+        </is>
+      </c>
       <c r="J179" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -12058,6 +12228,11 @@
           <t>Stateful tool-using LLM agents treat the context window as working memory, yet today's agent harnesses manage residency and durability as best-effort, causing recurring failures: lost state after compaction, bypassed flushes on reset, and destructive writeback. We present \textsc{ClawVM}, a virtual memory layer that manages state as typed pages with minimum-fidelity invariants, multi-resolution representations under a token budget, and validated writeback at every lifecycle boundary. Because the harness already assembles prompts, mediates tools, and observes lifecycle events, it is the natural enforcement point; placing the contract there makes residency and durability deterministic and auditable. Across synthetic workloads, 12 real-session traces, and adversarial stress tests, \textsc{ClawVM} eliminates all policy-controllable faults whenever the minimum-fidelity set fits within the token budget, confirmed by an offline oracle, and adds median &lt;50 microseconds of policy-engine overhead per turn.</t>
         </is>
       </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>针对大语言模型智能体在使用工具时因状态管理不可靠导致的问题，本文提出了ClawVM</t>
+        </is>
+      </c>
       <c r="J180" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -12105,6 +12280,11 @@
           <t>Introspection is central to identity construction and future planning, yet most digital tools approach the self as a unified entity. In contrast, Dialogical Self Theory (DST) views the self as composed of multiple internal perspectives, such as values, concerns, and aspirations, that can come into tension or dialogue with one another. Building on this view, we designed InnerPond, a research probe in the form of a multi-agent system that represents these internal perspectives as distinct LLM-based agents for introspection. Its design was shaped through iterative explorations of spatial metaphors, interaction scaffolding, and conversational orchestration, culminating in a shared spatial environment for organizing and relating multiple inner perspectives. In a user study with 17 young adults navigating career choices, participants engaged with the probe by co-creating inner voices with AI, composing relational inner landscapes, and orchestrating dialogue as observers and mediators, offering insight into how such systems could support introspection. Overall, this work offers design implications for AI-supported introspection tools that enable exploration of the self's multiplicity.</t>
         </is>
       </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>本文针对数字工具常将自我视为统一体的局限，基于对话自我理论提出InnerPond系统。该系统采用多智能体架构，将用户的价值观、关切、抱负等内部视角建模为基于大语言模型的独立智能体，通过共享空间环境促进其对话与整合。研究通过空间隐喻、交互支架与对话编排的迭代设计，探索了AI支持的内省工具设计路径，并在青年职业选择场景中验证了用户通过创建AI声音、构建关联内心图景及协调对话</t>
+        </is>
+      </c>
       <c r="J181" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -12152,6 +12332,11 @@
           <t>High-fidelity social simulation is pivotal for addressing complex Web societal challenges, yet it demands agents capable of authentically replicating the dynamic spectrum of human interaction. Current LLM-based multi-agent frameworks, however, predominantly adhere to static interaction topologies, failing to capture the fluid oscillation between cooperative knowledge synthesis and competitive critical reasoning seen in real-world scenarios. This rigidity often leads to unrealistic ``groupthink'' or unproductive deadlocks, undermining the credibility of simulations for decision support. To bridge this gap, we propose \textit{BEACOF}, a \textit{belief-driven adaptive collaboration framework} inspired by Perfect Bayesian Equilibrium (PBE). By modeling social interaction as a dynamic game of incomplete information, BEACOF rigorously addresses the circular dependency between collaboration type selection and capability estimation. Agents iteratively refine probabilistic beliefs about peer capabilities and autonomously modulate their collaboration strategy, thereby ensuring sequentially rational decisions under uncertainty. Validated across adversarial (judicial), open-ended (social) and mixed (medical) scenarios, BEACOF prevents coordination failures and fosters robust convergence toward high-quality solutions, demonstrating superior potential for reliable social simulation. Source codes and datasets are publicly released at: https://github.com/WUT-IDEA/BEACOF.</t>
         </is>
       </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>为应对高保真社会模拟中静态交互拓扑的局限性，本文提出BEACOF——一种受完美贝叶斯均衡启发、基于信念的自适应多智能体协作框架。该框架将社会互动建模为不完全信息动态博弈，通过迭代优化智能体间的能力信念，使其能自主调节协作策略，从而实现不确定性下的序列理性决策。实验表明，该方法能有效避免群体思维与协作僵化，在司法、社交、医疗等场景中展现出优于传统框架的鲁棒收敛性，为可信社会模拟提供了新思路。</t>
+        </is>
+      </c>
       <c r="J182" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -12199,6 +12384,11 @@
           <t>Social platforms serve as central hubs for information exchange, where user behaviors and platform interventions jointly shape opinions. However, intervention policies like recommendation and content filtering, can unintentionally amplify echo chambers and polarization, posing significant societal risks. Proactively evaluating the impact of such policies is therefore crucial. Existing approaches primarily rely on reactive online A/B testing, where risks are identified only after deployment, making risk identification delayed and costly. LLM-based social simulations offer a promising pre-deployment alternative, but current methods fall short in realistically modeling platform interventions and incorporating feedback from the platform. Bridging these gaps is essential for building actionable frameworks to assess and optimize platform policies. To this end, we propose PolicySim, an LLM-based social simulation sandbox for the proactive assessment and optimization of intervention policies. PolicySim models the bidirectional dynamics between user behavior and platform interventions through two key components: (1) a user agent module refined via supervised fine-tuning (SFT) and direct preference optimization (DPO) to achieve platform-specific behavioral realism; and (2) an adaptive intervention module that employs a contextual bandit with message passing to capture dynamic network structures. Experiments show that PolicySim can accurately simulate platform ecosystems at both micro and macro levels and support effective intervention policy.</t>
         </is>
       </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>PolicySim是一个基于大语言模型的智能体社交模拟沙盒，用于主动评估与优化社交平台的干预政策。该研究指出，当前平台采用的推荐、内容过滤等干预措施可能无意间加剧回声室效应与观点极化，而现有的线上A/B测试属于事后评估，成本高且风险识别滞后。为此，PolicySim通过两个核心模块构建平台干预与用户行为间的双向动态模拟：一是基于监督微调（SFT）与直接偏好优化（DPO）训练的用户智能</t>
+        </is>
+      </c>
       <c r="J183" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -12246,6 +12436,11 @@
           <t>Theory of Mind (ToM) refers to the ability to reason about others' mental states, and higher-order ToM involves considering that others also possess their own ToM. Equipping large language model (LLM)-driven agents with ToM has long been considered to improve their coordination in multiagent collaborative tasks. However, we find that misaligned ToM orders-mismatches in the depth of ToM reasoning between agents-can lead to insufficient or excessive reasoning about others, thereby impairing their coordination. To address this issue, we design an adaptive ToM (A-ToM) agent, which can align in ToM orders with its partner. Based on prior interactions, the agent estimates the partner's likely ToM order and leverages this estimation to predict the partner's action, thereby facilitating behavioral coordination. We conduct empirical evaluations on four multi-agent coordination tasks: a repeated matrix game, two grid navigation tasks and an Overcooked task. The results validate our findings on ToM alignment and demonstrate the effectiveness of our A-ToM agent. Furthermore, we discuss the generalizability of our A-ToM to non-LLM-based agents, as well as what would diminish the importance of ToM alignment.</t>
         </is>
       </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>本研究针对基于大型语言模型（LLM）的多智能体协调问题，探讨了理论心智（ToM）阶数对齐的重要性。我们发现，智能体间ToM推理深度的错位会削弱协作效果。为此，我们提出自适应理论心智（A-ToM）智能体，它能估计合作伙伴的ToM阶数并预测其行为，从而实现更好的行为</t>
+        </is>
+      </c>
       <c r="J184" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -12293,6 +12488,11 @@
           <t>Aligning large language models (LLMs) with human values is a central challenge for ensuring trustworthy and safe deployment. While existing methods such as Reinforcement Learning from Human Feedback (RLHF) and its variants have improved alignment, they often rely on a single evaluator or narrowly defined reward signals, limiting their ability to capture ethical pluralism. In this work, we propose the Value Alignment System using Combinatorial Fusion Analysis (VAS-CFA), a framework that operationalizes multi-agent fusion alignment. It instantiates multiple moral agents, each fine-tuned to represent a distinct normative perspective, and fuses their outputs using CFA with both rank- and score-based aggregation. This design leverages cognitive diversity, between agents, to mitigate conflicts and redundancies across multiple agents, producing responses that better reflect human values. Empirical evaluation demonstrates that VAS-CFA outperforms both single agent baselines and prior aggregation approaches on standard metrics, showing that multi-agent fusion provides a robust and effective mechanism for advancing value alignment in LLMs.</t>
         </is>
       </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>针对大语言模型（LLMs）与人类价值观对齐这一核心难题，现有方法（如RLHF及其变体）多依赖单一评估者或狭窄的奖励信号，难以捕捉伦理多元性。为此，本研究提出基于组合融合分析的价值对齐系统（VAS-CFA），通过实例化多个分别代表不同规范视角的道德智能体，并利用排名与分数融合的组合分析方法聚合其输出，从而在智能体间利用认知多样性来减少冲突与冗余。实验表明，该多智能体融合框架在标准指标上优于单一智能体基线及既有聚合方法，为</t>
+        </is>
+      </c>
       <c r="J185" t="inlineStr">
         <is>
           <t>2026-05-12</t>
@@ -12338,6 +12538,11 @@
       <c r="G186" t="inlineStr">
         <is>
           <t>Microsoft Copilot suites serve as the universal entry point for various agents skilled in handling important tasks, ranging from assisting a customer with product purchases to detecting vulnerabilities in corporate programming code. Each agent can be powered by language models, software engineering operations, such as database retrieval, and internal \&amp; external knowledge. The repertoire of a copilot can expand dynamically with new agents. This requires a robust orchestrator that can distribute tasks from user prompts to the right agents. In this work, we propose an Agentic Meta-orchestrator (AMO) for handling multiple tasks and scalable agents in copilot services, which can provide both natural language and action responses. We will also demonstrate the planning that leverages meta-learning, i.e., a trained decision tree model for deciding the best inference strategy among various agents/models. We showcase the effectiveness of our AMO through two production use cases: Microsoft 365 (M365) E-Commerce Copilot and code compliance copilot. M365 E-Commerce Copilot advertises Microsoft products to external customers to promote sales success. The M365 E-Commerce Copilot provides up-to-date product information and connects to multiple agents, such as relational databases and human customer support. The code compliance copilot scans the internal DevOps code to detect known and new compliance issues in pull requests (PR).</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>微软Copilot套件作为处理多任务智能体的统一入口，可通过语言模型、软件工程操作及内外部知识支撑各专业化智能体。随着智能体动态扩展，需要稳健的编排器将用户请求分发至合适智能体。本文提出智能体元编排器，用于处理多任务与可扩展的智能体服务，支持自然语言与行动响应；并利用元学习（基于训练的决策树模型）规划最佳推理策略。通过微软365电商Copilot与代码合规Copilot的实际案例</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">

</xml_diff>